<commit_message>
refactor(assets): readable logo file names in assets/img/logos/
Renames the 101 portfolio logos from hashes to company slugs
(e.g. pismo.png), updates the spreadsheet and every reference in
index.html, and removes 34 unreferenced images. Also publishes the
new sites for Movile, Ascenty, Neurogram and Revert.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romerorodrigues/Documents/GitHub/romerorodrigues.com/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{875EF6B2-5558-9C4E-A0FB-F9904F573B4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{477B47F4-D569-DA4D-8D07-6FE87C7A1B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -393,7 +393,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="376">
   <si>
     <t>Prioridade</t>
   </si>
@@ -485,7 +485,7 @@
     <t>https://www.buscape.com.br</t>
   </si>
   <si>
-    <t>6425515db5.png</t>
+    <t>buscape.png</t>
   </si>
   <si>
     <t>Pismo</t>
@@ -500,7 +500,7 @@
     <t>https://www.pismo.io/</t>
   </si>
   <si>
-    <t>7b32850226.png</t>
+    <t>pismo.png</t>
   </si>
   <si>
     <t>Wayfair</t>
@@ -512,7 +512,7 @@
     <t>https://www.wayfair.com</t>
   </si>
   <si>
-    <t>7006159f38.png</t>
+    <t>wayfair.png</t>
   </si>
   <si>
     <t>Wellhub</t>
@@ -521,7 +521,7 @@
     <t>https://wellhub.com/pt-br/</t>
   </si>
   <si>
-    <t>713b217bd1.png</t>
+    <t>wellhub.png</t>
   </si>
   <si>
     <t>Olist</t>
@@ -533,7 +533,7 @@
     <t>https://olist.com</t>
   </si>
   <si>
-    <t>05513689a9.png</t>
+    <t>olist.png</t>
   </si>
   <si>
     <t>Hotmart</t>
@@ -542,7 +542,7 @@
     <t>https://hotmart.com/en</t>
   </si>
   <si>
-    <t>0091b93521.png</t>
+    <t>hotmart.png</t>
   </si>
   <si>
     <t>VTEX</t>
@@ -551,7 +551,7 @@
     <t>https://www.vtex.com/en-us</t>
   </si>
   <si>
-    <t>963036fff1.png</t>
+    <t>vtex.png</t>
   </si>
   <si>
     <t>Rappi</t>
@@ -560,13 +560,13 @@
     <t>https://www.rappi.com.br</t>
   </si>
   <si>
-    <t>996b11623c.png</t>
+    <t>rappi.png</t>
   </si>
   <si>
     <t>Ascenty</t>
   </si>
   <si>
-    <t>f0e2b4b7e5.png</t>
+    <t>ascenty.png</t>
   </si>
   <si>
     <t>TOTVS</t>
@@ -578,7 +578,7 @@
     <t>https://www.totvs.com</t>
   </si>
   <si>
-    <t>67d3e7019f.png</t>
+    <t>totvs.png</t>
   </si>
   <si>
     <t>NeoGrid</t>
@@ -587,7 +587,7 @@
     <t>https://neogrid.com</t>
   </si>
   <si>
-    <t>d24a5faea5.png</t>
+    <t>neogrid.png</t>
   </si>
   <si>
     <t>Endeavor Brasil</t>
@@ -596,7 +596,7 @@
     <t>https://brasil.endeavor.org/</t>
   </si>
   <si>
-    <t>b3001c0150.png</t>
+    <t>endeavor-brasil.png</t>
   </si>
   <si>
     <t>Movile</t>
@@ -605,10 +605,10 @@
     <t>Movile · iFood</t>
   </si>
   <si>
-    <t>63f15d3a90.png</t>
-  </si>
-  <si>
-    <t>526f10b82c.png</t>
+    <t>movile.png</t>
+  </si>
+  <si>
+    <t>ifood.png</t>
   </si>
   <si>
     <t>Movile; iFood</t>
@@ -620,7 +620,7 @@
     <t>https://avenia.io</t>
   </si>
   <si>
-    <t>593662bf50.png</t>
+    <t>avenia.png</t>
   </si>
   <si>
     <t>Hero Seguros</t>
@@ -629,13 +629,13 @@
     <t>https://heroseguros.com.br/</t>
   </si>
   <si>
-    <t>1abdf56dac.png</t>
+    <t>hero-seguros.png</t>
   </si>
   <si>
     <t>Revert</t>
   </si>
   <si>
-    <t>20049a1c94.png</t>
+    <t>revert.png</t>
   </si>
   <si>
     <t>Alia.do</t>
@@ -644,7 +644,7 @@
     <t>https://alia.do</t>
   </si>
   <si>
-    <t>b6f4b92125.png</t>
+    <t>alia-do.png</t>
   </si>
   <si>
     <t>Celero</t>
@@ -653,7 +653,7 @@
     <t>https://celero.com.br</t>
   </si>
   <si>
-    <t>1eeb112b43.png</t>
+    <t>celero.png</t>
   </si>
   <si>
     <t>Doc9</t>
@@ -662,7 +662,7 @@
     <t>https://doc9.com.br/</t>
   </si>
   <si>
-    <t>97f1418353.png</t>
+    <t>doc9.png</t>
   </si>
   <si>
     <t>Jumpad</t>
@@ -671,7 +671,7 @@
     <t>https://jumpad.ai/</t>
   </si>
   <si>
-    <t>3fe9022228.png</t>
+    <t>jumpad.png</t>
   </si>
   <si>
     <t>Mercado de Recebíveis</t>
@@ -680,13 +680,13 @@
     <t>https://mercadoderecebiveis.com.br/</t>
   </si>
   <si>
-    <t>0d095c967b.png</t>
+    <t>mercado-de-recebiveis.png</t>
   </si>
   <si>
     <t>Neurogram</t>
   </si>
   <si>
-    <t>8af8202e5e.png</t>
+    <t>neurogram.png</t>
   </si>
   <si>
     <t>PipeImob</t>
@@ -695,7 +695,7 @@
     <t>https://pipeimob.com.br/</t>
   </si>
   <si>
-    <t>2880f53836.png</t>
+    <t>pipeimob.png</t>
   </si>
   <si>
     <t>Vaas</t>
@@ -704,7 +704,7 @@
     <t>https://vaas.com.br/</t>
   </si>
   <si>
-    <t>4bfe37b1ca.png</t>
+    <t>vaas.png</t>
   </si>
   <si>
     <t>Blips</t>
@@ -713,7 +713,7 @@
     <t>https://www.blips.com.br</t>
   </si>
   <si>
-    <t>16b675b3ab.png</t>
+    <t>blips.png</t>
   </si>
   <si>
     <t>Horuss</t>
@@ -722,7 +722,7 @@
     <t>https://www.horuss.ai/</t>
   </si>
   <si>
-    <t>9f1c1b0735.png</t>
+    <t>horuss.png</t>
   </si>
   <si>
     <t>Turn2C</t>
@@ -731,13 +731,13 @@
     <t>https://turn2c.com</t>
   </si>
   <si>
-    <t>adde0bf608.png</t>
+    <t>turn2c.png</t>
   </si>
   <si>
     <t>Cycles</t>
   </si>
   <si>
-    <t>aabc314b38.png</t>
+    <t>cycles.png</t>
   </si>
   <si>
     <t>Delfos</t>
@@ -746,7 +746,7 @@
     <t>https://www.delfos.energy/</t>
   </si>
   <si>
-    <t>b88afc0b6a.png</t>
+    <t>delfos.png</t>
   </si>
   <si>
     <t>Fiibo</t>
@@ -755,13 +755,13 @@
     <t>https://fiibo.com.br</t>
   </si>
   <si>
-    <t>7c2b6844ee.png</t>
+    <t>fiibo.png</t>
   </si>
   <si>
     <t>Fin-X</t>
   </si>
   <si>
-    <t>54076a9f5d.png</t>
+    <t>fin-x.png</t>
   </si>
   <si>
     <t>Hubii</t>
@@ -770,7 +770,7 @@
     <t>https://hubii.com.br/</t>
   </si>
   <si>
-    <t>544cfee6b8.png</t>
+    <t>hubii.png</t>
   </si>
   <si>
     <t>Mission Brasil</t>
@@ -779,7 +779,7 @@
     <t>https://missionbrasil.com.br/</t>
   </si>
   <si>
-    <t>6890f6ec1b.png</t>
+    <t>mission-brasil.png</t>
   </si>
   <si>
     <t>Trinus</t>
@@ -788,19 +788,19 @@
     <t>https://trinus.co</t>
   </si>
   <si>
-    <t>2f0f5faa11.png</t>
+    <t>trinus.png</t>
   </si>
   <si>
     <t>Upik</t>
   </si>
   <si>
-    <t>4718288ba8.png</t>
+    <t>upik.png</t>
   </si>
   <si>
     <t>Smart Break</t>
   </si>
   <si>
-    <t>2d210083e8.png</t>
+    <t>smart-break.png</t>
   </si>
   <si>
     <t>XP Inc.</t>
@@ -809,7 +809,7 @@
     <t>Sócio e executivo</t>
   </si>
   <si>
-    <t>ada4f0bb15.png</t>
+    <t>xp-inc.png</t>
   </si>
   <si>
     <t>CondoConta</t>
@@ -818,7 +818,7 @@
     <t>https://condoconta.com.br</t>
   </si>
   <si>
-    <t>3e6bed0147.png</t>
+    <t>condoconta.png</t>
   </si>
   <si>
     <t>Headline Brasil</t>
@@ -830,7 +830,7 @@
     <t>https://headline.com</t>
   </si>
   <si>
-    <t>18cb582104.png</t>
+    <t>headline-brasil.png</t>
   </si>
   <si>
     <t>Kzas</t>
@@ -839,7 +839,7 @@
     <t>Saída</t>
   </si>
   <si>
-    <t>4d10fac6e0.png</t>
+    <t>kzas.png</t>
   </si>
   <si>
     <t>Tembici</t>
@@ -848,7 +848,7 @@
     <t>https://www.tembici.com.br/pt/</t>
   </si>
   <si>
-    <t>2b7618efb4.png</t>
+    <t>tembici.png</t>
   </si>
   <si>
     <t>eureciclo</t>
@@ -857,7 +857,7 @@
     <t>https://eureciclo.com.br/</t>
   </si>
   <si>
-    <t>9d2bf2cbac.png</t>
+    <t>eureciclo.png</t>
   </si>
   <si>
     <t>ABC da Construção</t>
@@ -866,7 +866,7 @@
     <t>https://www.abcdaconstrucao.com.br/</t>
   </si>
   <si>
-    <t>348ad66045.png</t>
+    <t>abc-da-construcao.png</t>
   </si>
   <si>
     <t>Antecipa</t>
@@ -875,7 +875,7 @@
     <t>https://antecipa.com/</t>
   </si>
   <si>
-    <t>5563fbb64d.png</t>
+    <t>antecipa.png</t>
   </si>
   <si>
     <t>Housi</t>
@@ -884,7 +884,7 @@
     <t>https://housi.com</t>
   </si>
   <si>
-    <t>9136f294e9.png</t>
+    <t>housi.png</t>
   </si>
   <si>
     <t>GigU</t>
@@ -893,7 +893,7 @@
     <t>https://site.stopclub.com.br/</t>
   </si>
   <si>
-    <t>ac0ff90114.png</t>
+    <t>gigu.png</t>
   </si>
   <si>
     <t>Vittude</t>
@@ -902,7 +902,7 @@
     <t>https://vittude.com/</t>
   </si>
   <si>
-    <t>48dc284e66.png</t>
+    <t>vittude.png</t>
   </si>
   <si>
     <t>Repassa</t>
@@ -914,7 +914,7 @@
     <t>https://www.repassa.com.br</t>
   </si>
   <si>
-    <t>fdaf35ff75.png</t>
+    <t>repassa.png</t>
   </si>
   <si>
     <t>https://braziljournal.com/renner-compra-repassa-e-entra-no-mercado-de-usados/</t>
@@ -932,7 +932,7 @@
     <t>https://www.abfintechs.com.br/</t>
   </si>
   <si>
-    <t>3bd9b9bc6d.png</t>
+    <t>abfintechs.png</t>
   </si>
   <si>
     <t>Consulta do Bem</t>
@@ -941,7 +941,7 @@
     <t>Encerrada</t>
   </si>
   <si>
-    <t>096f0873fe.png</t>
+    <t>consulta-do-bem.png</t>
   </si>
   <si>
     <t>Curupira</t>
@@ -953,13 +953,13 @@
     <t>https://www.ceneo.pl/</t>
   </si>
   <si>
-    <t>b5e21647e8.png</t>
+    <t>ceneo.png</t>
   </si>
   <si>
     <t>Compari</t>
   </si>
   <si>
-    <t>dd8c455ccc.png</t>
+    <t>compari.png</t>
   </si>
   <si>
     <t>Drezzi</t>
@@ -968,7 +968,7 @@
     <t>Heureka</t>
   </si>
   <si>
-    <t>9bbdd734d2.png</t>
+    <t>heureka.png</t>
   </si>
   <si>
     <t>In Loco</t>
@@ -977,7 +977,7 @@
     <t>https://www.incognia.com/</t>
   </si>
   <si>
-    <t>9de7f1d8c8.png</t>
+    <t>in-loco.png</t>
   </si>
   <si>
     <t>Misshobby</t>
@@ -986,7 +986,7 @@
     <t>https://www.misshobby.com/it</t>
   </si>
   <si>
-    <t>f1157cd8d3.png</t>
+    <t>misshobby.png</t>
   </si>
   <si>
     <t>Naspers / Prosus</t>
@@ -995,7 +995,7 @@
     <t>https://www.prosus.com</t>
   </si>
   <si>
-    <t>530b76dd78.png</t>
+    <t>naspers-prosus.png</t>
   </si>
   <si>
     <t>PayU</t>
@@ -1004,13 +1004,13 @@
     <t>https://corporate.payu.com</t>
   </si>
   <si>
-    <t>a21633992e.png</t>
+    <t>payu.png</t>
   </si>
   <si>
     <t>Pazaruvaj</t>
   </si>
   <si>
-    <t>118369684d.png</t>
+    <t>pazaruvaj.png</t>
   </si>
   <si>
     <t>PriceCheck</t>
@@ -1022,13 +1022,13 @@
     <t>https://www.shoppydoo.it/</t>
   </si>
   <si>
-    <t>2ef87b6724.png</t>
+    <t>shoppydoo.png</t>
   </si>
   <si>
     <t>Trovaprezzi</t>
   </si>
   <si>
-    <t>05ba33d3e6.png</t>
+    <t>trovaprezzi.png</t>
   </si>
   <si>
     <t>Ucuzu</t>
@@ -1040,7 +1040,7 @@
     <t>Árukereső</t>
   </si>
   <si>
-    <t>0dfa51baf7.png</t>
+    <t>arukereso.png</t>
   </si>
   <si>
     <t>Btarget</t>
@@ -1052,7 +1052,7 @@
     <t>https://www.cuponeria.com.br</t>
   </si>
   <si>
-    <t>320e04926e.png</t>
+    <t>cuponeria.png</t>
   </si>
   <si>
     <t>Redpoint e.ventures</t>
@@ -1061,25 +1061,25 @@
     <t>https://rpev.com.br/</t>
   </si>
   <si>
-    <t>da50e23068.png</t>
+    <t>redpoint-e-ventures.png</t>
   </si>
   <si>
     <t>Shopcliq</t>
   </si>
   <si>
-    <t>1c8bca54ba.png</t>
+    <t>shopcliq.png</t>
   </si>
   <si>
     <t>Brandsclub</t>
   </si>
   <si>
-    <t>12c335338a.png</t>
+    <t>brandsclub.png</t>
   </si>
   <si>
     <t>DineroMail</t>
   </si>
   <si>
-    <t>7651fc3af4.png</t>
+    <t>dineromail.png</t>
   </si>
   <si>
     <t>MeuCarrinho</t>
@@ -1091,7 +1091,7 @@
     <t>https://modait.com.br/</t>
   </si>
   <si>
-    <t>385240fa1b.png</t>
+    <t>moda-it.png</t>
   </si>
   <si>
     <t>Navegg</t>
@@ -1100,7 +1100,7 @@
     <t>https://www.navegg.com/br</t>
   </si>
   <si>
-    <t>8f73ae2a32.png</t>
+    <t>navegg.png</t>
   </si>
   <si>
     <t>Recomind.net</t>
@@ -1115,31 +1115,31 @@
     <t>https://jivemaua.com.br:443/</t>
   </si>
   <si>
-    <t>f49b6eee17.png</t>
+    <t>jive.png</t>
   </si>
   <si>
     <t>PagosOnline</t>
   </si>
   <si>
-    <t>0fea4ac44e.png</t>
+    <t>pagosonline.png</t>
   </si>
   <si>
     <t>SaveMe</t>
   </si>
   <si>
-    <t>d6454f271a.png</t>
+    <t>saveme.png</t>
   </si>
   <si>
     <t>eBehavior</t>
   </si>
   <si>
-    <t>1e927e8b4c.png</t>
+    <t>ebehavior.png</t>
   </si>
   <si>
     <t>Lomadee</t>
   </si>
   <si>
-    <t>15e4202322.png</t>
+    <t>lomadee.png</t>
   </si>
   <si>
     <t>Bcash / Pagamento Digital</t>
@@ -1148,7 +1148,7 @@
     <t>Bcash</t>
   </si>
   <si>
-    <t>f489bd4096.png</t>
+    <t>pagamento-digital.png</t>
   </si>
   <si>
     <t>Pagamento Digital</t>
@@ -1157,13 +1157,13 @@
     <t>FControl</t>
   </si>
   <si>
-    <t>7d7def01a3.png</t>
+    <t>fcontrol.png</t>
   </si>
   <si>
     <t>E-bit</t>
   </si>
   <si>
-    <t>3a3bf47353.png</t>
+    <t>e-bit.png</t>
   </si>
   <si>
     <t>Bondfaro</t>
@@ -1172,13 +1172,13 @@
     <t>https://www.bondfaro.com.br/</t>
   </si>
   <si>
-    <t>02c33a4b5c.png</t>
+    <t>bondfaro.png</t>
   </si>
   <si>
     <t>CortaContas</t>
   </si>
   <si>
-    <t>10dad44d65.png</t>
+    <t>cortacontas.png</t>
   </si>
   <si>
     <t>QueBarato!</t>
@@ -1187,7 +1187,7 @@
     <t>https://www.quebarato.com.br/</t>
   </si>
   <si>
-    <t>530a049ea4.png</t>
+    <t>quebarato.png</t>
   </si>
   <si>
     <t>All in</t>
@@ -1223,7 +1223,7 @@
     <t>https://bovplatform.com/about</t>
   </si>
   <si>
-    <t>a1dc086833.png</t>
+    <t>bovcontrol.png</t>
   </si>
   <si>
     <t>Canal da Peça</t>
@@ -1232,7 +1232,7 @@
     <t>https://www.canaldapeca.com.br/</t>
   </si>
   <si>
-    <t>6b67c13db1.png</t>
+    <t>canal-da-peca.png</t>
   </si>
   <si>
     <t>Clicksign</t>
@@ -1241,7 +1241,7 @@
     <t>https://www.clicksign.com</t>
   </si>
   <si>
-    <t>aa020bf137.png</t>
+    <t>clicksign.png</t>
   </si>
   <si>
     <t>ContaPaga</t>
@@ -1250,7 +1250,7 @@
     <t>DirectTalk</t>
   </si>
   <si>
-    <t>6022056f1e.png</t>
+    <t>directtalk.png</t>
   </si>
   <si>
     <t>Galena</t>
@@ -1259,7 +1259,7 @@
     <t>https://www.galena.com</t>
   </si>
   <si>
-    <t>da9240af2a.png</t>
+    <t>galena.png</t>
   </si>
   <si>
     <t>Grubster / ChefsClub</t>
@@ -1271,7 +1271,7 @@
     <t>Humortadela</t>
   </si>
   <si>
-    <t>0cf980daec.png</t>
+    <t>humortadela.png</t>
   </si>
   <si>
     <t>Ingresse</t>
@@ -1280,7 +1280,7 @@
     <t>https://ingresse.com/</t>
   </si>
   <si>
-    <t>7d65ca6dde.png</t>
+    <t>ingresse.png</t>
   </si>
   <si>
     <t>Jet8</t>
@@ -1289,7 +1289,7 @@
     <t>https://jet8.io/</t>
   </si>
   <si>
-    <t>f6a286ee47.png</t>
+    <t>jet8.png</t>
   </si>
   <si>
     <t>LOFTY / ROOMORAMA</t>
@@ -1316,7 +1316,7 @@
     <t>https://marketup.com</t>
   </si>
   <si>
-    <t>4047ffd9a4.png</t>
+    <t>marketup.png</t>
   </si>
   <si>
     <t>Moneto</t>
@@ -1325,7 +1325,7 @@
     <t>OrderIn</t>
   </si>
   <si>
-    <t>62f4f9938d.png</t>
+    <t>orderin.png</t>
   </si>
   <si>
     <t>Prontmed</t>
@@ -1334,7 +1334,7 @@
     <t>https://www.prontmed.com</t>
   </si>
   <si>
-    <t>b4494154ca.png</t>
+    <t>prontmed.png</t>
   </si>
   <si>
     <t>Qipu / MEI Grátis</t>
@@ -1343,13 +1343,13 @@
     <t>https://qipu.com.br/</t>
   </si>
   <si>
-    <t>289192bf69.png</t>
+    <t>qipu-mei-gratis.png</t>
   </si>
   <si>
     <t>Quero Educação</t>
   </si>
   <si>
-    <t>d491f7a1ff.png</t>
+    <t>quero-educacao.png</t>
   </si>
   <si>
     <t>RecargaPay</t>
@@ -1358,7 +1358,7 @@
     <t>https://recargapay.com.br</t>
   </si>
   <si>
-    <t>c262835caf.png</t>
+    <t>recargapay.png</t>
   </si>
   <si>
     <t>SP Ventures</t>
@@ -1367,13 +1367,13 @@
     <t>https://spventures.com.br/</t>
   </si>
   <si>
-    <t>d15738202b.png</t>
+    <t>sp-ventures.png</t>
   </si>
   <si>
     <t>Scup</t>
   </si>
   <si>
-    <t>b4b241d87d.png</t>
+    <t>scup.png</t>
   </si>
   <si>
     <t>SetYou</t>
@@ -1382,7 +1382,7 @@
     <t>https://setyou.com.br/</t>
   </si>
   <si>
-    <t>80498a675b.png</t>
+    <t>setyou.png</t>
   </si>
   <si>
     <t>Shoes4you</t>
@@ -1391,7 +1391,7 @@
     <t>https://shoes4you.com.br/</t>
   </si>
   <si>
-    <t>164d131ac4.png</t>
+    <t>shoes4you.png</t>
   </si>
   <si>
     <t>Siga Seu Time</t>
@@ -1403,13 +1403,13 @@
     <t>https://www.viagogo.com/</t>
   </si>
   <si>
-    <t>b14d2ee246.png</t>
+    <t>viagogo.png</t>
   </si>
   <si>
     <t>ViajaNet</t>
   </si>
   <si>
-    <t>d98ba85a96.png</t>
+    <t>viajanet.png</t>
   </si>
   <si>
     <t>Zup</t>
@@ -1418,7 +1418,7 @@
     <t>https://zup.com.br/</t>
   </si>
   <si>
-    <t>477f11fab3.png</t>
+    <t>zup.png</t>
   </si>
   <si>
     <t>youHotel</t>
@@ -1509,6 +1509,18 @@
   </si>
   <si>
     <t>Sócio de Gestora</t>
+  </si>
+  <si>
+    <t>https://ascenty.com/</t>
+  </si>
+  <si>
+    <t>https://www.ifood.com.br/</t>
+  </si>
+  <si>
+    <t>https://neurogram.com/</t>
+  </si>
+  <si>
+    <t>https://revertai.com.br/</t>
   </si>
 </sst>
 </file>
@@ -1591,7 +1603,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1608,6 +1620,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2515,6 +2528,9 @@
       <c r="O12" s="5">
         <v>2010</v>
       </c>
+      <c r="Q12" s="8" t="s">
+        <v>373</v>
+      </c>
       <c r="R12" t="s">
         <v>70</v>
       </c>
@@ -2659,6 +2675,9 @@
       <c r="P16" t="s">
         <v>44</v>
       </c>
+      <c r="Q16" s="8" t="s">
+        <v>372</v>
+      </c>
       <c r="R16" t="s">
         <v>57</v>
       </c>
@@ -3047,6 +3066,9 @@
       <c r="P27" t="s">
         <v>44</v>
       </c>
+      <c r="Q27" s="8" t="s">
+        <v>374</v>
+      </c>
       <c r="R27" t="s">
         <v>97</v>
       </c>
@@ -3292,6 +3314,9 @@
       </c>
       <c r="O34" s="5">
         <v>2026</v>
+      </c>
+      <c r="Q34" s="8" t="s">
+        <v>375</v>
       </c>
       <c r="R34" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
feat(portfolio): 18 logos novos ou trocados
Novos: AWL Leads, Curupira, CyberCook, Lema21, Loteria Brasil, Mirum,
PriceCheck, youHotel, Lulu, MeuCarrinho, Urbanizo e ChefsClub/Grubster.
Trocados (nome de arquivo novo, por causa do cache de uma semana):
Buscapé, Bondfaro, Redpoint eventures, SaveMe, Scup e SP Ventures, que
mostravam imagem errada ou só o símbolo.

Fundo transparente a partir das bordas (o branco de dentro do logo fica),
recortados no conteúdo, com o WebP gerado pelo imagens.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -971,7 +971,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>buscape.png</t>
+          <t>buscape-2026.png</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>redpoint-e-ventures.png</t>
+          <t>redpoint-eventures.png</t>
         </is>
       </c>
       <c r="T62" t="inlineStr"/>
@@ -5217,7 +5217,11 @@
           <t>https://www.crunchbase.com/organization/meucarrinho</t>
         </is>
       </c>
-      <c r="S66" t="inlineStr"/>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>meucarrinho.png</t>
+        </is>
+      </c>
       <c r="T66" t="inlineStr"/>
       <c r="U66" t="inlineStr"/>
       <c r="V66" t="inlineStr"/>
@@ -5453,7 +5457,11 @@
           <t>https://www.crunchbase.com/organization/urbanizo</t>
         </is>
       </c>
-      <c r="S70" t="inlineStr"/>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>urbanizo.png</t>
+        </is>
+      </c>
       <c r="T70" t="inlineStr"/>
       <c r="U70" t="inlineStr"/>
       <c r="V70" t="inlineStr"/>
@@ -5569,7 +5577,7 @@
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>saveme.png</t>
+          <t>saveme-2026.png</t>
         </is>
       </c>
       <c r="T72" t="inlineStr"/>
@@ -5939,7 +5947,7 @@
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>bondfaro.png</t>
+          <t>bondfaro-2026.png</t>
         </is>
       </c>
       <c r="T78" t="inlineStr"/>
@@ -6169,7 +6177,11 @@
           <t>https://www.crunchbase.com/organization/mirum-agency; https://www.crunchbase.com/organization/m%C3%ADdia-digital</t>
         </is>
       </c>
-      <c r="S82" t="inlineStr"/>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>mirum.png</t>
+        </is>
+      </c>
       <c r="T82" t="inlineStr"/>
       <c r="U82" t="inlineStr"/>
       <c r="V82" t="inlineStr"/>
@@ -6275,7 +6287,11 @@
           <t>https://www.crunchbase.com/organization/awl-fee7</t>
         </is>
       </c>
-      <c r="S84" t="inlineStr"/>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>awl-leads.png</t>
+        </is>
+      </c>
       <c r="T84" t="inlineStr"/>
       <c r="U84" t="inlineStr"/>
       <c r="V84" t="inlineStr"/>
@@ -6625,7 +6641,11 @@
           <t>https://www.crunchbase.com/organization/grubster</t>
         </is>
       </c>
-      <c r="S90" t="inlineStr"/>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>chefsclub-grubster.png</t>
+        </is>
+      </c>
       <c r="T90" t="inlineStr"/>
       <c r="U90" t="inlineStr"/>
       <c r="V90" t="inlineStr"/>
@@ -6794,7 +6814,11 @@
           <t>https://www.crunchbase.com/organization/lema21</t>
         </is>
       </c>
-      <c r="S93" t="inlineStr"/>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>lema21.png</t>
+        </is>
+      </c>
       <c r="T93" t="inlineStr"/>
       <c r="U93" t="inlineStr"/>
       <c r="V93" t="inlineStr"/>
@@ -7032,7 +7056,7 @@
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>sp-ventures.png</t>
+          <t>sp-ventures-2026.png</t>
         </is>
       </c>
       <c r="T97" t="inlineStr"/>
@@ -7549,7 +7573,11 @@
           <t>https://www.crunchbase.com/organization/pricecheck</t>
         </is>
       </c>
-      <c r="S106" t="inlineStr"/>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>pricecheck.png</t>
+        </is>
+      </c>
       <c r="T106" t="inlineStr"/>
       <c r="U106" t="inlineStr"/>
       <c r="V106" t="inlineStr"/>
@@ -7942,7 +7970,11 @@
           <t>https://www.crunchbase.com/organization/curupira</t>
         </is>
       </c>
-      <c r="S113" t="inlineStr"/>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>curupira.png</t>
+        </is>
+      </c>
       <c r="T113" t="inlineStr"/>
       <c r="U113" t="inlineStr"/>
       <c r="V113" t="inlineStr"/>
@@ -7997,7 +8029,11 @@
       </c>
       <c r="Q114" t="inlineStr"/>
       <c r="R114" t="inlineStr"/>
-      <c r="S114" t="inlineStr"/>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>cybercook.png</t>
+        </is>
+      </c>
       <c r="T114" t="inlineStr"/>
       <c r="U114" t="inlineStr"/>
       <c r="V114" t="inlineStr"/>
@@ -8048,7 +8084,11 @@
       <c r="P115" t="inlineStr"/>
       <c r="Q115" t="inlineStr"/>
       <c r="R115" t="inlineStr"/>
-      <c r="S115" t="inlineStr"/>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>loteria-brasil.png</t>
+        </is>
+      </c>
       <c r="T115" t="inlineStr"/>
       <c r="U115" t="inlineStr"/>
       <c r="V115" t="inlineStr"/>
@@ -8370,7 +8410,11 @@
           <t>https://www.crunchbase.com/organization/lulu-2</t>
         </is>
       </c>
-      <c r="S121" t="inlineStr"/>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>lulu-app.png</t>
+        </is>
+      </c>
       <c r="T121" t="inlineStr"/>
       <c r="U121" t="inlineStr"/>
       <c r="V121" t="inlineStr"/>
@@ -8533,7 +8577,7 @@
       </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t>scup.png</t>
+          <t>scup-2026.png</t>
         </is>
       </c>
       <c r="T124" t="inlineStr"/>
@@ -8696,7 +8740,11 @@
           <t>https://www.crunchbase.com/organization/youhotel</t>
         </is>
       </c>
-      <c r="S127" t="inlineStr"/>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>youhotel.png</t>
+        </is>
+      </c>
       <c r="T127" t="inlineStr"/>
       <c r="U127" t="inlineStr"/>
       <c r="V127" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(logos): Great Hill na Trajetória; Jet8, Moneto e OrderIn no portfólio
- Great Hill Partners no marco de 2005 (Série B do Buscapé).
- Jet8 e OrderIn trocados (nome de arquivo novo, por causa do cache);
  os antigos saem do repositório.
- Moneto ganha logo.
- OrderIn vinha em branco sobre fundo escuro: fundo virou transparência
  (o degradê do ícone também) e o texto ficou escuro, para o card claro.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -8298,7 +8298,7 @@
       <c r="R119" t="inlineStr"/>
       <c r="S119" t="inlineStr">
         <is>
-          <t>jet8.png</t>
+          <t>jet8-2026.png</t>
         </is>
       </c>
       <c r="T119" t="inlineStr"/>
@@ -8465,7 +8465,11 @@
           <t>https://www.crunchbase.com/organization/contapaga</t>
         </is>
       </c>
-      <c r="S122" t="inlineStr"/>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>moneto.png</t>
+        </is>
+      </c>
       <c r="T122" t="inlineStr"/>
       <c r="U122" t="inlineStr"/>
       <c r="V122" t="inlineStr"/>
@@ -8522,7 +8526,7 @@
       </c>
       <c r="S123" t="inlineStr">
         <is>
-          <t>orderin.png</t>
+          <t>orderin-2026.png</t>
         </is>
       </c>
       <c r="T123" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(portfolio): Biosphera (B&Partners), investimento anjo
Card com logo, status Ativa e perfil no Crunchbase (b-partners-6cab).
Sem site por enquanto: bpartners.com.br está fora do ar e biosphera.io é
domínio estacionado. Portfólio passa a 125 empresas (124 na versão EN).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Empresas'!$A$1:$Z$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Empresas'!$A$1:$Z$128</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -736,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z127"/>
+  <dimension ref="A1:Z128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6303,7 +6303,7 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>1010</t>
+          <t>1005</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -6314,7 +6314,7 @@
       <c r="C85" s="5" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
-          <t>BovControl</t>
+          <t>Biosphera (B&amp;Partners)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -6335,20 +6335,20 @@
       </c>
       <c r="N85" t="inlineStr"/>
       <c r="O85" s="5" t="inlineStr"/>
-      <c r="P85" t="inlineStr"/>
-      <c r="Q85" t="inlineStr">
-        <is>
-          <t>https://bovplatform.com/about</t>
-        </is>
-      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr"/>
       <c r="R85" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/bovcontrol</t>
+          <t>https://www.crunchbase.com/organization/b-partners-6cab</t>
         </is>
       </c>
       <c r="S85" t="inlineStr">
         <is>
-          <t>bovcontrol.png</t>
+          <t>biosphera.png</t>
         </is>
       </c>
       <c r="T85" t="inlineStr"/>
@@ -6357,12 +6357,16 @@
       <c r="W85" t="inlineStr"/>
       <c r="X85" t="inlineStr"/>
       <c r="Y85" t="inlineStr"/>
-      <c r="Z85" t="inlineStr"/>
+      <c r="Z85" t="inlineStr">
+        <is>
+          <t>Anjo. Site: bpartners.com.br fora do ar em 28/09/2026; biosphera.io é domínio estacionado.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>1020</t>
+          <t>1010</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
@@ -6373,7 +6377,7 @@
       <c r="C86" s="5" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Canal da Peça</t>
+          <t>BovControl</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -6397,17 +6401,17 @@
       <c r="P86" t="inlineStr"/>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>https://www.canaldapeca.com.br/</t>
+          <t>https://bovplatform.com/about</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/canal-da-pe%C3%A7a</t>
+          <t>https://www.crunchbase.com/organization/bovcontrol</t>
         </is>
       </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t>canal-da-peca.png</t>
+          <t>bovcontrol.png</t>
         </is>
       </c>
       <c r="T86" t="inlineStr"/>
@@ -6421,7 +6425,7 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>1030</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -6432,7 +6436,7 @@
       <c r="C87" s="5" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Clicksign</t>
+          <t>Canal da Peça</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -6453,24 +6457,20 @@
       </c>
       <c r="N87" t="inlineStr"/>
       <c r="O87" s="5" t="inlineStr"/>
-      <c r="P87" t="inlineStr">
-        <is>
-          <t>Ativa</t>
-        </is>
-      </c>
+      <c r="P87" t="inlineStr"/>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>https://www.clicksign.com</t>
+          <t>https://www.canaldapeca.com.br/</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/clicksign</t>
+          <t>https://www.crunchbase.com/organization/canal-da-pe%C3%A7a</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>clicksign.png</t>
+          <t>canal-da-peca.png</t>
         </is>
       </c>
       <c r="T87" t="inlineStr"/>
@@ -6484,7 +6484,7 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>1040</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
@@ -6495,7 +6495,7 @@
       <c r="C88" s="5" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
-          <t>DirectTalk</t>
+          <t>Clicksign</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -6521,15 +6521,19 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q88" t="inlineStr"/>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>https://www.clicksign.com</t>
+        </is>
+      </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/hi-platform</t>
+          <t>https://www.crunchbase.com/organization/clicksign</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>directtalk.png</t>
+          <t>clicksign.png</t>
         </is>
       </c>
       <c r="T88" t="inlineStr"/>
@@ -6543,7 +6547,7 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>1050</t>
+          <t>1040</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -6554,7 +6558,7 @@
       <c r="C89" s="5" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Galena</t>
+          <t>DirectTalk</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -6575,20 +6579,20 @@
       </c>
       <c r="N89" t="inlineStr"/>
       <c r="O89" s="5" t="inlineStr"/>
-      <c r="P89" t="inlineStr"/>
-      <c r="Q89" t="inlineStr">
-        <is>
-          <t>https://www.galena.com</t>
-        </is>
-      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr"/>
       <c r="R89" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/galena-c08c</t>
+          <t>https://www.crunchbase.com/organization/hi-platform</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>galena.png</t>
+          <t>directtalk.png</t>
         </is>
       </c>
       <c r="T89" t="inlineStr"/>
@@ -6602,7 +6606,7 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>1060</t>
+          <t>1050</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
@@ -6613,7 +6617,7 @@
       <c r="C90" s="5" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Grubster / ChefsClub</t>
+          <t>Galena</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -6635,15 +6639,19 @@
       <c r="N90" t="inlineStr"/>
       <c r="O90" s="5" t="inlineStr"/>
       <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="inlineStr"/>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>https://www.galena.com</t>
+        </is>
+      </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/grubster</t>
+          <t>https://www.crunchbase.com/organization/galena-c08c</t>
         </is>
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>chefsclub-grubster.png</t>
+          <t>galena.png</t>
         </is>
       </c>
       <c r="T90" t="inlineStr"/>
@@ -6657,7 +6665,7 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>1070</t>
+          <t>1060</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -6668,7 +6676,7 @@
       <c r="C91" s="5" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Humortadela</t>
+          <t>Grubster / ChefsClub</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -6691,10 +6699,14 @@
       <c r="O91" s="5" t="inlineStr"/>
       <c r="P91" t="inlineStr"/>
       <c r="Q91" t="inlineStr"/>
-      <c r="R91" t="inlineStr"/>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/grubster</t>
+        </is>
+      </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>humortadela.png</t>
+          <t>chefsclub-grubster.png</t>
         </is>
       </c>
       <c r="T91" t="inlineStr"/>
@@ -6708,7 +6720,7 @@
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>1080</t>
+          <t>1070</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
@@ -6719,7 +6731,7 @@
       <c r="C92" s="5" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Ingresse</t>
+          <t>Humortadela</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -6741,19 +6753,11 @@
       <c r="N92" t="inlineStr"/>
       <c r="O92" s="5" t="inlineStr"/>
       <c r="P92" t="inlineStr"/>
-      <c r="Q92" t="inlineStr">
-        <is>
-          <t>https://ingresse.com/</t>
-        </is>
-      </c>
-      <c r="R92" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/ingresse</t>
-        </is>
-      </c>
+      <c r="Q92" t="inlineStr"/>
+      <c r="R92" t="inlineStr"/>
       <c r="S92" t="inlineStr">
         <is>
-          <t>ingresse.png</t>
+          <t>humortadela.png</t>
         </is>
       </c>
       <c r="T92" t="inlineStr"/>
@@ -6767,7 +6771,7 @@
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>1090</t>
+          <t>1080</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -6778,7 +6782,7 @@
       <c r="C93" s="5" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Lema21</t>
+          <t>Ingresse</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -6797,26 +6801,22 @@
         <f>IF(L93&lt;&gt;"",L93,_xlfn.TEXTJOIN(" · ",TRUE,IF(F93&lt;&gt;"","Fundador",""),IF(G93&lt;&gt;"","Anjo",""),IF(H93&lt;&gt;"","VC",""),IF(I93&lt;&gt;"","Gestão",""),IF(J93&lt;&gt;"","Conselho",""),IF(K93&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N93" t="inlineStr">
-        <is>
-          <t>Vendida à Essilor</t>
-        </is>
-      </c>
+      <c r="N93" t="inlineStr"/>
       <c r="O93" s="5" t="inlineStr"/>
-      <c r="P93" t="inlineStr">
-        <is>
-          <t>Adquirida</t>
-        </is>
-      </c>
-      <c r="Q93" t="inlineStr"/>
+      <c r="P93" t="inlineStr"/>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>https://ingresse.com/</t>
+        </is>
+      </c>
       <c r="R93" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/lema21</t>
+          <t>https://www.crunchbase.com/organization/ingresse</t>
         </is>
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>lema21.png</t>
+          <t>ingresse.png</t>
         </is>
       </c>
       <c r="T93" t="inlineStr"/>
@@ -6830,7 +6830,7 @@
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>1090</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
@@ -6841,7 +6841,7 @@
       <c r="C94" s="5" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Prontmed</t>
+          <t>Lema21</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -6860,26 +6860,26 @@
         <f>IF(L94&lt;&gt;"",L94,_xlfn.TEXTJOIN(" · ",TRUE,IF(F94&lt;&gt;"","Fundador",""),IF(G94&lt;&gt;"","Anjo",""),IF(H94&lt;&gt;"","VC",""),IF(I94&lt;&gt;"","Gestão",""),IF(J94&lt;&gt;"","Conselho",""),IF(K94&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N94" t="inlineStr"/>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>Vendida à Essilor</t>
+        </is>
+      </c>
       <c r="O94" s="5" t="inlineStr"/>
       <c r="P94" t="inlineStr">
         <is>
-          <t>Ativa</t>
-        </is>
-      </c>
-      <c r="Q94" t="inlineStr">
-        <is>
-          <t>https://www.prontmed.com</t>
-        </is>
-      </c>
+          <t>Adquirida</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr"/>
       <c r="R94" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/prontmed</t>
+          <t>https://www.crunchbase.com/organization/lema21</t>
         </is>
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>prontmed.png</t>
+          <t>lema21.png</t>
         </is>
       </c>
       <c r="T94" t="inlineStr"/>
@@ -6893,7 +6893,7 @@
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>1110</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -6904,7 +6904,7 @@
       <c r="C95" s="5" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Qipu / MEI Grátis</t>
+          <t>Prontmed</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -6925,20 +6925,24 @@
       </c>
       <c r="N95" t="inlineStr"/>
       <c r="O95" s="5" t="inlineStr"/>
-      <c r="P95" t="inlineStr"/>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>https://qipu.com.br/</t>
+          <t>https://www.prontmed.com</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/qipu</t>
+          <t>https://www.crunchbase.com/organization/prontmed</t>
         </is>
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>qipu-mei-gratis.png</t>
+          <t>prontmed.png</t>
         </is>
       </c>
       <c r="T95" t="inlineStr"/>
@@ -6952,7 +6956,7 @@
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>1120</t>
+          <t>1110</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
@@ -6963,7 +6967,7 @@
       <c r="C96" s="5" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Quero Educação</t>
+          <t>Qipu / MEI Grátis</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -6984,20 +6988,20 @@
       </c>
       <c r="N96" t="inlineStr"/>
       <c r="O96" s="5" t="inlineStr"/>
-      <c r="P96" t="inlineStr">
-        <is>
-          <t>Ativa</t>
-        </is>
-      </c>
-      <c r="Q96" t="inlineStr"/>
+      <c r="P96" t="inlineStr"/>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>https://qipu.com.br/</t>
+        </is>
+      </c>
       <c r="R96" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/quero-education</t>
+          <t>https://www.crunchbase.com/organization/qipu</t>
         </is>
       </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t>quero-educacao.png</t>
+          <t>qipu-mei-gratis.png</t>
         </is>
       </c>
       <c r="T96" t="inlineStr"/>
@@ -7011,7 +7015,7 @@
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>1130</t>
+          <t>1120</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -7022,7 +7026,7 @@
       <c r="C97" s="5" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
-          <t>SP Ventures</t>
+          <t>Quero Educação</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -7043,20 +7047,20 @@
       </c>
       <c r="N97" t="inlineStr"/>
       <c r="O97" s="5" t="inlineStr"/>
-      <c r="P97" t="inlineStr"/>
-      <c r="Q97" t="inlineStr">
-        <is>
-          <t>https://spventures.com.br/</t>
-        </is>
-      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr"/>
       <c r="R97" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/sp-ventures</t>
+          <t>https://www.crunchbase.com/organization/quero-education</t>
         </is>
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>sp-ventures-2026.png</t>
+          <t>quero-educacao.png</t>
         </is>
       </c>
       <c r="T97" t="inlineStr"/>
@@ -7070,7 +7074,7 @@
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>1140</t>
+          <t>1130</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
@@ -7081,7 +7085,7 @@
       <c r="C98" s="5" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
-          <t>SetYou</t>
+          <t>SP Ventures</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -7105,17 +7109,17 @@
       <c r="P98" t="inlineStr"/>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>https://setyou.com.br/</t>
+          <t>https://spventures.com.br/</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/set-you</t>
+          <t>https://www.crunchbase.com/organization/sp-ventures</t>
         </is>
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>setyou.png</t>
+          <t>sp-ventures-2026.png</t>
         </is>
       </c>
       <c r="T98" t="inlineStr"/>
@@ -7129,7 +7133,7 @@
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>1150</t>
+          <t>1140</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -7140,17 +7144,17 @@
       <c r="C99" s="5" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
-          <t>ViajaNet</t>
+          <t>SetYou</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" s="5" t="inlineStr"/>
-      <c r="G99" s="5" t="inlineStr"/>
-      <c r="H99" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H99" s="5" t="inlineStr"/>
       <c r="I99" s="5" t="inlineStr"/>
       <c r="J99" s="5" t="inlineStr"/>
       <c r="K99" s="5" t="inlineStr"/>
@@ -7162,15 +7166,19 @@
       <c r="N99" t="inlineStr"/>
       <c r="O99" s="5" t="inlineStr"/>
       <c r="P99" t="inlineStr"/>
-      <c r="Q99" t="inlineStr"/>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>https://setyou.com.br/</t>
+        </is>
+      </c>
       <c r="R99" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/viajanet</t>
+          <t>https://www.crunchbase.com/organization/set-you</t>
         </is>
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t>viajanet.png</t>
+          <t>setyou.png</t>
         </is>
       </c>
       <c r="T99" t="inlineStr"/>
@@ -7184,7 +7192,7 @@
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1150</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
@@ -7195,45 +7203,37 @@
       <c r="C100" s="5" t="inlineStr"/>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Ceneo</t>
+          <t>ViajaNet</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" s="5" t="inlineStr"/>
       <c r="G100" s="5" t="inlineStr"/>
-      <c r="H100" s="5" t="inlineStr"/>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I100" s="5" t="inlineStr"/>
       <c r="J100" s="5" t="inlineStr"/>
-      <c r="K100" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K100" s="5" t="inlineStr"/>
       <c r="L100" t="inlineStr"/>
       <c r="M100" s="6">
         <f>IF(L100&lt;&gt;"",L100,_xlfn.TEXTJOIN(" · ",TRUE,IF(F100&lt;&gt;"","Fundador",""),IF(G100&lt;&gt;"","Anjo",""),IF(H100&lt;&gt;"","VC",""),IF(I100&lt;&gt;"","Gestão",""),IF(J100&lt;&gt;"","Conselho",""),IF(K100&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
       <c r="N100" t="inlineStr"/>
-      <c r="O100" s="5" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
+      <c r="O100" s="5" t="inlineStr"/>
       <c r="P100" t="inlineStr"/>
-      <c r="Q100" t="inlineStr">
-        <is>
-          <t>https://www.ceneo.pl/</t>
-        </is>
-      </c>
+      <c r="Q100" t="inlineStr"/>
       <c r="R100" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/ceneo</t>
+          <t>https://www.crunchbase.com/organization/viajanet</t>
         </is>
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>ceneo.png</t>
+          <t>viajanet.png</t>
         </is>
       </c>
       <c r="T100" t="inlineStr"/>
@@ -7247,7 +7247,7 @@
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -7258,7 +7258,7 @@
       <c r="C101" s="5" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Compari</t>
+          <t>Ceneo</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -7284,11 +7284,19 @@
         </is>
       </c>
       <c r="P101" t="inlineStr"/>
-      <c r="Q101" t="inlineStr"/>
-      <c r="R101" t="inlineStr"/>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>https://www.ceneo.pl/</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/ceneo</t>
+        </is>
+      </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>compari.png</t>
+          <t>ceneo.png</t>
         </is>
       </c>
       <c r="T101" t="inlineStr"/>
@@ -7302,7 +7310,7 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
@@ -7313,7 +7321,7 @@
       <c r="C102" s="5" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Drezzi</t>
+          <t>Compari</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -7340,12 +7348,12 @@
       </c>
       <c r="P102" t="inlineStr"/>
       <c r="Q102" t="inlineStr"/>
-      <c r="R102" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/drezzy</t>
-        </is>
-      </c>
-      <c r="S102" t="inlineStr"/>
+      <c r="R102" t="inlineStr"/>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>compari.png</t>
+        </is>
+      </c>
       <c r="T102" t="inlineStr"/>
       <c r="U102" t="inlineStr"/>
       <c r="V102" t="inlineStr"/>
@@ -7357,7 +7365,7 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
@@ -7368,7 +7376,7 @@
       <c r="C103" s="5" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Heureka</t>
+          <t>Drezzi</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -7397,14 +7405,10 @@
       <c r="Q103" t="inlineStr"/>
       <c r="R103" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/heureka-group</t>
-        </is>
-      </c>
-      <c r="S103" t="inlineStr">
-        <is>
-          <t>heureka.png</t>
-        </is>
-      </c>
+          <t>https://www.crunchbase.com/organization/drezzy</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr"/>
       <c r="T103" t="inlineStr"/>
       <c r="U103" t="inlineStr"/>
       <c r="V103" t="inlineStr"/>
@@ -7416,31 +7420,31 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>1904</t>
-        </is>
-      </c>
-      <c r="B104" s="5" t="inlineStr"/>
+          <t>1903</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="C104" s="5" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Misshobby</t>
+          <t>Heureka</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" s="5" t="inlineStr"/>
       <c r="G104" s="5" t="inlineStr"/>
       <c r="H104" s="5" t="inlineStr"/>
-      <c r="I104" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J104" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K104" s="5" t="inlineStr"/>
+      <c r="I104" s="5" t="inlineStr"/>
+      <c r="J104" s="5" t="inlineStr"/>
+      <c r="K104" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L104" t="inlineStr"/>
       <c r="M104" s="6">
         <f>IF(L104&lt;&gt;"",L104,_xlfn.TEXTJOIN(" · ",TRUE,IF(F104&lt;&gt;"","Fundador",""),IF(G104&lt;&gt;"","Anjo",""),IF(H104&lt;&gt;"","VC",""),IF(I104&lt;&gt;"","Gestão",""),IF(J104&lt;&gt;"","Conselho",""),IF(K104&lt;&gt;"","Buscapé","")))</f>
@@ -7453,15 +7457,15 @@
         </is>
       </c>
       <c r="P104" t="inlineStr"/>
-      <c r="Q104" t="inlineStr">
-        <is>
-          <t>https://www.misshobby.com/it</t>
-        </is>
-      </c>
-      <c r="R104" t="inlineStr"/>
+      <c r="Q104" t="inlineStr"/>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/heureka-group</t>
+        </is>
+      </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>misshobby.png</t>
+          <t>heureka.png</t>
         </is>
       </c>
       <c r="T104" t="inlineStr"/>
@@ -7475,31 +7479,31 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>1905</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1904</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr"/>
       <c r="C105" s="5" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Pazaruvaj</t>
+          <t>Misshobby</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" s="5" t="inlineStr"/>
       <c r="G105" s="5" t="inlineStr"/>
       <c r="H105" s="5" t="inlineStr"/>
-      <c r="I105" s="5" t="inlineStr"/>
-      <c r="J105" s="5" t="inlineStr"/>
-      <c r="K105" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I105" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J105" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K105" s="5" t="inlineStr"/>
       <c r="L105" t="inlineStr"/>
       <c r="M105" s="6">
         <f>IF(L105&lt;&gt;"",L105,_xlfn.TEXTJOIN(" · ",TRUE,IF(F105&lt;&gt;"","Fundador",""),IF(G105&lt;&gt;"","Anjo",""),IF(H105&lt;&gt;"","VC",""),IF(I105&lt;&gt;"","Gestão",""),IF(J105&lt;&gt;"","Conselho",""),IF(K105&lt;&gt;"","Buscapé","")))</f>
@@ -7512,11 +7516,15 @@
         </is>
       </c>
       <c r="P105" t="inlineStr"/>
-      <c r="Q105" t="inlineStr"/>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>https://www.misshobby.com/it</t>
+        </is>
+      </c>
       <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr">
         <is>
-          <t>pazaruvaj.png</t>
+          <t>misshobby.png</t>
         </is>
       </c>
       <c r="T105" t="inlineStr"/>
@@ -7530,7 +7538,7 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1905</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
@@ -7541,7 +7549,7 @@
       <c r="C106" s="5" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
-          <t>PriceCheck</t>
+          <t>Pazaruvaj</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -7568,14 +7576,10 @@
       </c>
       <c r="P106" t="inlineStr"/>
       <c r="Q106" t="inlineStr"/>
-      <c r="R106" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/pricecheck</t>
-        </is>
-      </c>
+      <c r="R106" t="inlineStr"/>
       <c r="S106" t="inlineStr">
         <is>
-          <t>pricecheck.png</t>
+          <t>pazaruvaj.png</t>
         </is>
       </c>
       <c r="T106" t="inlineStr"/>
@@ -7589,7 +7593,7 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
@@ -7600,7 +7604,7 @@
       <c r="C107" s="5" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
-          <t>ShoppyDoo</t>
+          <t>PriceCheck</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -7626,19 +7630,15 @@
         </is>
       </c>
       <c r="P107" t="inlineStr"/>
-      <c r="Q107" t="inlineStr">
-        <is>
-          <t>https://www.shoppydoo.it/</t>
-        </is>
-      </c>
+      <c r="Q107" t="inlineStr"/>
       <c r="R107" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/shoppydoo</t>
+          <t>https://www.crunchbase.com/organization/pricecheck</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>shoppydoo.png</t>
+          <t>pricecheck.png</t>
         </is>
       </c>
       <c r="T107" t="inlineStr"/>
@@ -7652,7 +7652,7 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
@@ -7663,7 +7663,7 @@
       <c r="C108" s="5" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Trovaprezzi</t>
+          <t>ShoppyDoo</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -7689,15 +7689,19 @@
         </is>
       </c>
       <c r="P108" t="inlineStr"/>
-      <c r="Q108" t="inlineStr"/>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>https://www.shoppydoo.it/</t>
+        </is>
+      </c>
       <c r="R108" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/trovaprezzi-it-d087</t>
+          <t>https://www.crunchbase.com/organization/shoppydoo</t>
         </is>
       </c>
       <c r="S108" t="inlineStr">
         <is>
-          <t>trovaprezzi.png</t>
+          <t>shoppydoo.png</t>
         </is>
       </c>
       <c r="T108" t="inlineStr"/>
@@ -7711,7 +7715,7 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
@@ -7722,7 +7726,7 @@
       <c r="C109" s="5" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Ucuzu</t>
+          <t>Trovaprezzi</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -7749,8 +7753,16 @@
       </c>
       <c r="P109" t="inlineStr"/>
       <c r="Q109" t="inlineStr"/>
-      <c r="R109" t="inlineStr"/>
-      <c r="S109" t="inlineStr"/>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/trovaprezzi-it-d087</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>trovaprezzi.png</t>
+        </is>
+      </c>
       <c r="T109" t="inlineStr"/>
       <c r="U109" t="inlineStr"/>
       <c r="V109" t="inlineStr"/>
@@ -7762,7 +7774,7 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
@@ -7773,7 +7785,7 @@
       <c r="C110" s="5" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Vcene</t>
+          <t>Ucuzu</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
@@ -7800,11 +7812,7 @@
       </c>
       <c r="P110" t="inlineStr"/>
       <c r="Q110" t="inlineStr"/>
-      <c r="R110" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/vcene</t>
-        </is>
-      </c>
+      <c r="R110" t="inlineStr"/>
       <c r="S110" t="inlineStr"/>
       <c r="T110" t="inlineStr"/>
       <c r="U110" t="inlineStr"/>
@@ -7817,7 +7825,7 @@
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
@@ -7828,7 +7836,7 @@
       <c r="C111" s="5" t="inlineStr"/>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Árukereső</t>
+          <t>Vcene</t>
         </is>
       </c>
       <c r="E111" t="inlineStr"/>
@@ -7857,14 +7865,10 @@
       <c r="Q111" t="inlineStr"/>
       <c r="R111" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/%C3%A1rukeres%C5%91</t>
-        </is>
-      </c>
-      <c r="S111" t="inlineStr">
-        <is>
-          <t>arukereso.png</t>
-        </is>
-      </c>
+          <t>https://www.crunchbase.com/organization/vcene</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr"/>
       <c r="T111" t="inlineStr"/>
       <c r="U111" t="inlineStr"/>
       <c r="V111" t="inlineStr"/>
@@ -7876,7 +7880,7 @@
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
@@ -7887,20 +7891,20 @@
       <c r="C112" s="5" t="inlineStr"/>
       <c r="D112" t="inlineStr">
         <is>
-          <t>FocoSoft</t>
+          <t>Árukereső</t>
         </is>
       </c>
       <c r="E112" t="inlineStr"/>
-      <c r="F112" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="F112" s="5" t="inlineStr"/>
       <c r="G112" s="5" t="inlineStr"/>
       <c r="H112" s="5" t="inlineStr"/>
       <c r="I112" s="5" t="inlineStr"/>
       <c r="J112" s="5" t="inlineStr"/>
-      <c r="K112" s="5" t="inlineStr"/>
+      <c r="K112" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L112" t="inlineStr"/>
       <c r="M112" s="6">
         <f>IF(L112&lt;&gt;"",L112,_xlfn.TEXTJOIN(" · ",TRUE,IF(F112&lt;&gt;"","Fundador",""),IF(G112&lt;&gt;"","Anjo",""),IF(H112&lt;&gt;"","VC",""),IF(I112&lt;&gt;"","Gestão",""),IF(J112&lt;&gt;"","Conselho",""),IF(K112&lt;&gt;"","Buscapé","")))</f>
@@ -7909,13 +7913,21 @@
       <c r="N112" t="inlineStr"/>
       <c r="O112" s="5" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="P112" t="inlineStr"/>
       <c r="Q112" t="inlineStr"/>
-      <c r="R112" t="inlineStr"/>
-      <c r="S112" t="inlineStr"/>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/%C3%A1rukeres%C5%91</t>
+        </is>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>arukereso.png</t>
+        </is>
+      </c>
       <c r="T112" t="inlineStr"/>
       <c r="U112" t="inlineStr"/>
       <c r="V112" t="inlineStr"/>
@@ -7927,7 +7939,7 @@
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
@@ -7938,16 +7950,16 @@
       <c r="C113" s="5" t="inlineStr"/>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Curupira</t>
+          <t>FocoSoft</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
-      <c r="F113" s="5" t="inlineStr"/>
-      <c r="G113" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr"/>
       <c r="H113" s="5" t="inlineStr"/>
       <c r="I113" s="5" t="inlineStr"/>
       <c r="J113" s="5" t="inlineStr"/>
@@ -7960,21 +7972,13 @@
       <c r="N113" t="inlineStr"/>
       <c r="O113" s="5" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="P113" t="inlineStr"/>
       <c r="Q113" t="inlineStr"/>
-      <c r="R113" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/curupira</t>
-        </is>
-      </c>
-      <c r="S113" t="inlineStr">
-        <is>
-          <t>curupira.png</t>
-        </is>
-      </c>
+      <c r="R113" t="inlineStr"/>
+      <c r="S113" t="inlineStr"/>
       <c r="T113" t="inlineStr"/>
       <c r="U113" t="inlineStr"/>
       <c r="V113" t="inlineStr"/>
@@ -7986,7 +7990,7 @@
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="B114" s="5" t="inlineStr">
@@ -7997,7 +8001,7 @@
       <c r="C114" s="5" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
-          <t>CyberCook / Vila Mulher</t>
+          <t>Curupira</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
@@ -8019,19 +8023,19 @@
       <c r="N114" t="inlineStr"/>
       <c r="O114" s="5" t="inlineStr">
         <is>
-          <t>2004</t>
-        </is>
-      </c>
-      <c r="P114" t="inlineStr">
-        <is>
-          <t>Ativa</t>
-        </is>
-      </c>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr"/>
       <c r="Q114" t="inlineStr"/>
-      <c r="R114" t="inlineStr"/>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/curupira</t>
+        </is>
+      </c>
       <c r="S114" t="inlineStr">
         <is>
-          <t>cybercook.png</t>
+          <t>curupira.png</t>
         </is>
       </c>
       <c r="T114" t="inlineStr"/>
@@ -8045,7 +8049,7 @@
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>2030</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
@@ -8056,7 +8060,7 @@
       <c r="C115" s="5" t="inlineStr"/>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Loteria Brasil</t>
+          <t>CyberCook / Vila Mulher</t>
         </is>
       </c>
       <c r="E115" t="inlineStr"/>
@@ -8081,12 +8085,16 @@
           <t>2004</t>
         </is>
       </c>
-      <c r="P115" t="inlineStr"/>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q115" t="inlineStr"/>
       <c r="R115" t="inlineStr"/>
       <c r="S115" t="inlineStr">
         <is>
-          <t>loteria-brasil.png</t>
+          <t>cybercook.png</t>
         </is>
       </c>
       <c r="T115" t="inlineStr"/>
@@ -8100,7 +8108,7 @@
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>2040</t>
+          <t>2030</t>
         </is>
       </c>
       <c r="B116" s="5" t="inlineStr">
@@ -8111,7 +8119,7 @@
       <c r="C116" s="5" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
-          <t>eHub</t>
+          <t>Loteria Brasil</t>
         </is>
       </c>
       <c r="E116" t="inlineStr"/>
@@ -8138,12 +8146,12 @@
       </c>
       <c r="P116" t="inlineStr"/>
       <c r="Q116" t="inlineStr"/>
-      <c r="R116" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/ehub</t>
-        </is>
-      </c>
-      <c r="S116" t="inlineStr"/>
+      <c r="R116" t="inlineStr"/>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>loteria-brasil.png</t>
+        </is>
+      </c>
       <c r="T116" t="inlineStr"/>
       <c r="U116" t="inlineStr"/>
       <c r="V116" t="inlineStr"/>
@@ -8155,7 +8163,7 @@
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>2040</t>
         </is>
       </c>
       <c r="B117" s="5" t="inlineStr">
@@ -8166,7 +8174,7 @@
       <c r="C117" s="5" t="inlineStr"/>
       <c r="D117" t="inlineStr">
         <is>
-          <t>ContaPaga</t>
+          <t>eHub</t>
         </is>
       </c>
       <c r="E117" t="inlineStr"/>
@@ -8186,16 +8194,16 @@
         <v/>
       </c>
       <c r="N117" t="inlineStr"/>
-      <c r="O117" s="5" t="inlineStr"/>
-      <c r="P117" t="inlineStr">
-        <is>
-          <t>Ativa</t>
-        </is>
-      </c>
+      <c r="O117" s="5" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr"/>
       <c r="Q117" t="inlineStr"/>
       <c r="R117" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/contapaga</t>
+          <t>https://www.crunchbase.com/organization/ehub</t>
         </is>
       </c>
       <c r="S117" t="inlineStr"/>
@@ -8210,7 +8218,7 @@
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>2060</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="B118" s="5" t="inlineStr">
@@ -8221,7 +8229,7 @@
       <c r="C118" s="5" t="inlineStr"/>
       <c r="D118" t="inlineStr">
         <is>
-          <t>HospedeVIP</t>
+          <t>ContaPaga</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -8242,9 +8250,17 @@
       </c>
       <c r="N118" t="inlineStr"/>
       <c r="O118" s="5" t="inlineStr"/>
-      <c r="P118" t="inlineStr"/>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q118" t="inlineStr"/>
-      <c r="R118" t="inlineStr"/>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/contapaga</t>
+        </is>
+      </c>
       <c r="S118" t="inlineStr"/>
       <c r="T118" t="inlineStr"/>
       <c r="U118" t="inlineStr"/>
@@ -8257,7 +8273,7 @@
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>2070</t>
+          <t>2060</t>
         </is>
       </c>
       <c r="B119" s="5" t="inlineStr">
@@ -8268,7 +8284,7 @@
       <c r="C119" s="5" t="inlineStr"/>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Jet8</t>
+          <t>HospedeVIP</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -8290,17 +8306,9 @@
       <c r="N119" t="inlineStr"/>
       <c r="O119" s="5" t="inlineStr"/>
       <c r="P119" t="inlineStr"/>
-      <c r="Q119" t="inlineStr">
-        <is>
-          <t>https://jet8.io/</t>
-        </is>
-      </c>
+      <c r="Q119" t="inlineStr"/>
       <c r="R119" t="inlineStr"/>
-      <c r="S119" t="inlineStr">
-        <is>
-          <t>jet8-2026.png</t>
-        </is>
-      </c>
+      <c r="S119" t="inlineStr"/>
       <c r="T119" t="inlineStr"/>
       <c r="U119" t="inlineStr"/>
       <c r="V119" t="inlineStr"/>
@@ -8312,7 +8320,7 @@
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>2080</t>
+          <t>2070</t>
         </is>
       </c>
       <c r="B120" s="5" t="inlineStr">
@@ -8323,7 +8331,7 @@
       <c r="C120" s="5" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
-          <t>LOFTY / ROOMORAMA</t>
+          <t>Jet8</t>
         </is>
       </c>
       <c r="E120" t="inlineStr"/>
@@ -8347,15 +8355,15 @@
       <c r="P120" t="inlineStr"/>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>https://roomorama.com/</t>
-        </is>
-      </c>
-      <c r="R120" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/roomorama; https://www.crunchbase.com/organization/lofty-ai</t>
-        </is>
-      </c>
-      <c r="S120" t="inlineStr"/>
+          <t>https://jet8.io/</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr"/>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>jet8-2026.png</t>
+        </is>
+      </c>
       <c r="T120" t="inlineStr"/>
       <c r="U120" t="inlineStr"/>
       <c r="V120" t="inlineStr"/>
@@ -8367,7 +8375,7 @@
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>2090</t>
+          <t>2080</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
@@ -8378,7 +8386,7 @@
       <c r="C121" s="5" t="inlineStr"/>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Lulu App</t>
+          <t>LOFTY / ROOMORAMA</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -8399,22 +8407,18 @@
       </c>
       <c r="N121" t="inlineStr"/>
       <c r="O121" s="5" t="inlineStr"/>
-      <c r="P121" t="inlineStr">
-        <is>
-          <t>Adquirida</t>
-        </is>
-      </c>
-      <c r="Q121" t="inlineStr"/>
+      <c r="P121" t="inlineStr"/>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>https://roomorama.com/</t>
+        </is>
+      </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/lulu-2</t>
-        </is>
-      </c>
-      <c r="S121" t="inlineStr">
-        <is>
-          <t>lulu-app.png</t>
-        </is>
-      </c>
+          <t>https://www.crunchbase.com/organization/roomorama; https://www.crunchbase.com/organization/lofty-ai</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr"/>
       <c r="T121" t="inlineStr"/>
       <c r="U121" t="inlineStr"/>
       <c r="V121" t="inlineStr"/>
@@ -8426,7 +8430,7 @@
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>2090</t>
         </is>
       </c>
       <c r="B122" s="5" t="inlineStr">
@@ -8437,7 +8441,7 @@
       <c r="C122" s="5" t="inlineStr"/>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Moneto</t>
+          <t>Lulu App</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -8458,16 +8462,20 @@
       </c>
       <c r="N122" t="inlineStr"/>
       <c r="O122" s="5" t="inlineStr"/>
-      <c r="P122" t="inlineStr"/>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Adquirida</t>
+        </is>
+      </c>
       <c r="Q122" t="inlineStr"/>
       <c r="R122" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/contapaga</t>
+          <t>https://www.crunchbase.com/organization/lulu-2</t>
         </is>
       </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t>moneto.png</t>
+          <t>lulu-app.png</t>
         </is>
       </c>
       <c r="T122" t="inlineStr"/>
@@ -8481,7 +8489,7 @@
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
@@ -8492,7 +8500,7 @@
       <c r="C123" s="5" t="inlineStr"/>
       <c r="D123" t="inlineStr">
         <is>
-          <t>OrderIn</t>
+          <t>Moneto</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
@@ -8513,20 +8521,16 @@
       </c>
       <c r="N123" t="inlineStr"/>
       <c r="O123" s="5" t="inlineStr"/>
-      <c r="P123" t="inlineStr">
-        <is>
-          <t>Ativa</t>
-        </is>
-      </c>
+      <c r="P123" t="inlineStr"/>
       <c r="Q123" t="inlineStr"/>
       <c r="R123" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/orderin</t>
+          <t>https://www.crunchbase.com/organization/contapaga</t>
         </is>
       </c>
       <c r="S123" t="inlineStr">
         <is>
-          <t>orderin-2026.png</t>
+          <t>moneto.png</t>
         </is>
       </c>
       <c r="T123" t="inlineStr"/>
@@ -8540,7 +8544,7 @@
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>2120</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="B124" s="5" t="inlineStr">
@@ -8551,7 +8555,7 @@
       <c r="C124" s="5" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Scup</t>
+          <t>OrderIn</t>
         </is>
       </c>
       <c r="E124" t="inlineStr"/>
@@ -8572,16 +8576,20 @@
       </c>
       <c r="N124" t="inlineStr"/>
       <c r="O124" s="5" t="inlineStr"/>
-      <c r="P124" t="inlineStr"/>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q124" t="inlineStr"/>
       <c r="R124" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/scup</t>
+          <t>https://www.crunchbase.com/organization/orderin</t>
         </is>
       </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t>scup-2026.png</t>
+          <t>orderin-2026.png</t>
         </is>
       </c>
       <c r="T124" t="inlineStr"/>
@@ -8595,7 +8603,7 @@
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>2120</t>
         </is>
       </c>
       <c r="B125" s="5" t="inlineStr">
@@ -8606,7 +8614,7 @@
       <c r="C125" s="5" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Shoes4you</t>
+          <t>Scup</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -8628,19 +8636,15 @@
       <c r="N125" t="inlineStr"/>
       <c r="O125" s="5" t="inlineStr"/>
       <c r="P125" t="inlineStr"/>
-      <c r="Q125" t="inlineStr">
-        <is>
-          <t>https://shoes4you.com.br/</t>
-        </is>
-      </c>
+      <c r="Q125" t="inlineStr"/>
       <c r="R125" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/shoes4you</t>
+          <t>https://www.crunchbase.com/organization/scup</t>
         </is>
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>shoes4you.png</t>
+          <t>scup-2026.png</t>
         </is>
       </c>
       <c r="T125" t="inlineStr"/>
@@ -8654,7 +8658,7 @@
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>2140</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="B126" s="5" t="inlineStr">
@@ -8665,7 +8669,7 @@
       <c r="C126" s="5" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Siga Seu Time</t>
+          <t>Shoes4you</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -8687,13 +8691,21 @@
       <c r="N126" t="inlineStr"/>
       <c r="O126" s="5" t="inlineStr"/>
       <c r="P126" t="inlineStr"/>
-      <c r="Q126" t="inlineStr"/>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>https://shoes4you.com.br/</t>
+        </is>
+      </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/sigaseutime</t>
-        </is>
-      </c>
-      <c r="S126" t="inlineStr"/>
+          <t>https://www.crunchbase.com/organization/shoes4you</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>shoes4you.png</t>
+        </is>
+      </c>
       <c r="T126" t="inlineStr"/>
       <c r="U126" t="inlineStr"/>
       <c r="V126" t="inlineStr"/>
@@ -8705,7 +8717,7 @@
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2140</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
@@ -8716,7 +8728,7 @@
       <c r="C127" s="5" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
-          <t>youHotel</t>
+          <t>Siga Seu Time</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -8741,14 +8753,10 @@
       <c r="Q127" t="inlineStr"/>
       <c r="R127" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/youhotel</t>
-        </is>
-      </c>
-      <c r="S127" t="inlineStr">
-        <is>
-          <t>youhotel.png</t>
-        </is>
-      </c>
+          <t>https://www.crunchbase.com/organization/sigaseutime</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr"/>
       <c r="T127" t="inlineStr"/>
       <c r="U127" t="inlineStr"/>
       <c r="V127" t="inlineStr"/>
@@ -8757,8 +8765,63 @@
       <c r="Y127" t="inlineStr"/>
       <c r="Z127" t="inlineStr"/>
     </row>
+    <row r="128">
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>2150</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr"/>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>youHotel</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" s="5" t="inlineStr"/>
+      <c r="G128" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H128" s="5" t="inlineStr"/>
+      <c r="I128" s="5" t="inlineStr"/>
+      <c r="J128" s="5" t="inlineStr"/>
+      <c r="K128" s="5" t="inlineStr"/>
+      <c r="L128" t="inlineStr"/>
+      <c r="M128" s="6">
+        <f>IF(L128&lt;&gt;"",L128,_xlfn.TEXTJOIN(" · ",TRUE,IF(F128&lt;&gt;"","Fundador",""),IF(G128&lt;&gt;"","Anjo",""),IF(H128&lt;&gt;"","VC",""),IF(I128&lt;&gt;"","Gestão",""),IF(J128&lt;&gt;"","Conselho",""),IF(K128&lt;&gt;"","Buscapé","")))</f>
+        <v/>
+      </c>
+      <c r="N128" t="inlineStr"/>
+      <c r="O128" s="5" t="inlineStr"/>
+      <c r="P128" t="inlineStr"/>
+      <c r="Q128" t="inlineStr"/>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/youhotel</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>youhotel.png</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr"/>
+      <c r="U128" t="inlineStr"/>
+      <c r="V128" t="inlineStr"/>
+      <c r="W128" t="inlineStr"/>
+      <c r="X128" t="inlineStr"/>
+      <c r="Y128" t="inlineStr"/>
+      <c r="Z128" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z127"/>
+  <autoFilter ref="A1:Z128"/>
   <dataValidations count="2">
     <dataValidation sqref="B2:B2000 F2:F2000 G2:G2000 H2:H2000 I2:I2000 J2:J2000 K2:K2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use x para marcar ou deixe vazio." type="list">
       <formula1>"x"</formula1>

</xml_diff>

<commit_message>
feat(portfolio): anos de Clicksign (2015) e Biosphera (2021); site da Biosphera
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -6334,13 +6334,21 @@
         <v/>
       </c>
       <c r="N85" t="inlineStr"/>
-      <c r="O85" s="5" t="inlineStr"/>
+      <c r="O85" s="5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="P85" t="inlineStr">
         <is>
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q85" t="inlineStr"/>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>https://biosphera.network/en/</t>
+        </is>
+      </c>
       <c r="R85" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/b-partners-6cab</t>
@@ -6359,7 +6367,7 @@
       <c r="Y85" t="inlineStr"/>
       <c r="Z85" t="inlineStr">
         <is>
-          <t>Anjo. Site: bpartners.com.br fora do ar em 28/09/2026; biosphera.io é domínio estacionado.</t>
+          <t>Anjo. Crunchbase ainda aponta o site antigo (bpartners.com.br).</t>
         </is>
       </c>
     </row>
@@ -6515,7 +6523,11 @@
         <v/>
       </c>
       <c r="N88" t="inlineStr"/>
-      <c r="O88" s="5" t="inlineStr"/>
+      <c r="O88" s="5" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
       <c r="P88" t="inlineStr">
         <is>
           <t>Ativa</t>

</xml_diff>

<commit_message>
feat(portfolio): status, notas, carrossel da home e 14 matérias revisados pelo Romero
Edições do Romero na planilha: status de 62 empresas, notas de saída de 20,
nova ordem do carrossel da home (22 logos), Biosphera no conselho, AWL
com site e Canal da Peça exibido como "CWS (Canal da Peça)".

Matérias: o Romero pôs os links; título (como o veículo publicou) e
"fonte · data" preenchidos a partir de cada página, ou da planilha de
mídia quando a peça já estava lá. Normalizados "Saida" → "Saída",
"US$ 1.8 bi" → "US$ 1,8 bi" e "R$ 575m" → "R$ 575M".

Versão em inglês: traduções de status, notas e fontes (mês em inglês,
também na da Repassa); títulos ficam como publicados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -912,7 +912,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1056,9 +1056,21 @@
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>https://fortune.com/2023/07/25/headline-brazil-pismo-visa/</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>How VC Headline notched a 30% stake in Brazil’s biggest startup acquisition in 5 years</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Fortune · jul 2023</t>
+        </is>
+      </c>
       <c r="Z3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -1074,7 +1086,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1108,7 +1120,11 @@
           <t>2013</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q4" t="inlineStr">
         <is>
           <t>https://wellhub.com/pt-br/</t>
@@ -1127,9 +1143,21 @@
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4v8VvLNtaxU</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>#Takeover | Romero Rodrigues &amp; Gympass: a startup brasileira que conquistou o mundo</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Cubo Itaú · set 2020</t>
+        </is>
+      </c>
       <c r="Z4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -1145,7 +1173,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1202,9 +1230,21 @@
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/wayfair-names-romero-rodrigues-to-its-board-of-directors-269021721.html</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Wayfair Names Romero Rodrigues to its Board of Directors</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>PR Newswire · jul 2014</t>
+        </is>
+      </c>
       <c r="Z5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -1220,7 +1260,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1277,9 +1317,21 @@
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>https://www.gazetadopovo.com.br/economia/empreender-pme/fundo-do-fundador-do-buscape-compra-participacao-em-startup-curitibana-9wkf3luxsvvljmo3q7ujely4v/</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Fundo do fundador do Buscapé compra participação em startup curitibana</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Gazeta do Povo · ago 2016</t>
+        </is>
+      </c>
       <c r="Z6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -1295,7 +1347,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1325,7 +1377,11 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr">
         <is>
           <t>https://hotmart.com/en</t>
@@ -1344,9 +1400,21 @@
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>https://startupi.com.br/saiba-como-anda-a-vida-da-hotmart-mais-de-um-ano-depois-de-vencer-o-desafio-buscape/</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Saiba como anda a vida da Hotmart mais de um ano depois de vencer o Desafio Buscapé</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Startupi · fev 2013</t>
+        </is>
+      </c>
       <c r="Z7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -1362,7 +1430,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1415,9 +1483,21 @@
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>https://neofeed.com.br/startups/headline-a-nova-gestora-de-romero-rodrigues-para-investir-em-startups/</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Headline, a nova gestora de Romero Rodrigues para investir em startups</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>NeoFeed · dez 2021</t>
+        </is>
+      </c>
       <c r="Z8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1433,7 +1513,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1482,9 +1562,21 @@
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TuSdKcgnNGA</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Day1 | Acredite no impossível - Romero Rodrigues [Buscapé]</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Endeavor Brasil · nov 2012</t>
+        </is>
+      </c>
       <c r="Z9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1500,7 +1592,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1571,7 +1663,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1599,13 +1691,21 @@
         <f>IF(L11&lt;&gt;"",L11,_xlfn.TEXTJOIN(" · ",TRUE,IF(F11&lt;&gt;"","Fundador",""),IF(G11&lt;&gt;"","Anjo",""),IF(H11&lt;&gt;"","VC",""),IF(I11&lt;&gt;"","Gestão",""),IF(J11&lt;&gt;"","Conselho",""),IF(K11&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Vendida a Riverwood</t>
+        </is>
+      </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
           <t>2004</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q11" t="inlineStr">
         <is>
           <t>https://www.vtex.com/en-us</t>
@@ -1624,9 +1724,21 @@
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>https://fusoesaquisicoes.com/acontece-no-setor/riverwood-compra-participacao-na-vtex/</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>Riverwood compra participação na VTEX da Naspers</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>Fusões &amp; Aquisições · mar 2015</t>
+        </is>
+      </c>
       <c r="Z11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1642,7 +1754,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1680,7 +1792,11 @@
           <t>2010</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q12" t="inlineStr">
         <is>
           <t>https://www.ifood.com.br/</t>
@@ -1725,7 +1841,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1751,7 +1867,11 @@
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" s="5" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q13" t="inlineStr">
         <is>
           <t>https://www.rappi.com.br</t>
@@ -1770,9 +1890,21 @@
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>https://www.wsj.com/articles/colombian-delivery-service-rappi-raising-up-to-145-million-1516327946</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>Colombian Delivery Service Rappi Raising Up to $145 Million</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>Wall Street Journal · jan 2018</t>
+        </is>
+      </c>
       <c r="Z13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1788,7 +1920,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1812,9 +1944,17 @@
         <f>IF(L14&lt;&gt;"",L14,_xlfn.TEXTJOIN(" · ",TRUE,IF(F14&lt;&gt;"","Fundador",""),IF(G14&lt;&gt;"","Anjo",""),IF(H14&lt;&gt;"","VC",""),IF(I14&lt;&gt;"","Gestão",""),IF(J14&lt;&gt;"","Conselho",""),IF(K14&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Vendida ao Itaú</t>
+        </is>
+      </c>
       <c r="O14" s="5" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>R$ 575M · 2019</t>
+        </is>
+      </c>
       <c r="Q14" t="inlineStr">
         <is>
           <t>https://zup.com.br/</t>
@@ -1833,9 +1973,21 @@
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>https://valor.globo.com/financas/noticia/2019/10/31/ita-unibanco-compra-zup-servios-em-tecnologia-por-r-575-milhes.ghtml</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>Itaú Unibanco compra Zup Serviços em Tecnologia por R$ 575 milhões</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>Valor · out 2019</t>
+        </is>
+      </c>
       <c r="Z14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1851,7 +2003,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1875,13 +2027,21 @@
         <f>IF(L15&lt;&gt;"",L15,_xlfn.TEXTJOIN(" · ",TRUE,IF(F15&lt;&gt;"","Fundador",""),IF(G15&lt;&gt;"","Anjo",""),IF(H15&lt;&gt;"","VC",""),IF(I15&lt;&gt;"","Gestão",""),IF(J15&lt;&gt;"","Conselho",""),IF(K15&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Vendida à XP Inc.</t>
+        </is>
+      </c>
       <c r="O15" s="5" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Adquirida · 2018</t>
+        </is>
+      </c>
       <c r="Q15" t="inlineStr">
         <is>
           <t>https://jivemaua.com.br:443/</t>
@@ -1900,9 +2060,21 @@
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>https://braziljournal.com/xp-compra-20-da-jive-uma-gestora-que-compra-e-resolve-problemas/</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>EXCLUSIVO: XP compra 20% da Jive, uma gestora que “compra e resolve problemas”</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>Brazil Journal · jun 2021</t>
+        </is>
+      </c>
       <c r="Z15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1918,7 +2090,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1946,7 +2118,11 @@
         <f>IF(L16&lt;&gt;"",L16,_xlfn.TEXTJOIN(" · ",TRUE,IF(F16&lt;&gt;"","Fundador",""),IF(G16&lt;&gt;"","Anjo",""),IF(H16&lt;&gt;"","VC",""),IF(I16&lt;&gt;"","Gestão",""),IF(J16&lt;&gt;"","Conselho",""),IF(K16&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Vendida a Digital Realty</t>
+        </is>
+      </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
           <t>2013</t>
@@ -1954,7 +2130,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Ativa</t>
+          <t>US$ 1,8 bi · 2018</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1975,9 +2151,21 @@
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>https://www.digitalrealty.com/about/newsroom/press-releases/122893/digital-realty-to-acquire-ascenty</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>Digital Realty To Acquire Ascenty</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>Digital Realty · set 2018</t>
+        </is>
+      </c>
       <c r="Z16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1993,7 +2181,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2019,7 +2207,11 @@
       </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" s="5" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q17" t="inlineStr">
         <is>
           <t>https://recargapay.com.br</t>
@@ -2056,7 +2248,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2123,7 +2315,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2194,7 +2386,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2259,7 +2451,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr"/>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>ABC da Construção</t>
@@ -2555,7 +2751,11 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q25" t="inlineStr">
         <is>
           <t>https://heroseguros.com.br/</t>
@@ -3154,7 +3354,11 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q34" t="inlineStr">
         <is>
           <t>https://revertai.com.br/</t>
@@ -4170,7 +4374,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr"/>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="D50" t="inlineStr">
         <is>
           <t>XP Inc.</t>
@@ -4217,9 +4425,21 @@
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr"/>
-      <c r="W50" t="inlineStr"/>
-      <c r="X50" t="inlineStr"/>
-      <c r="Y50" t="inlineStr"/>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>https://valor.globo.com/financas/noticia/2022/06/09/fundo-de-venture-capital-da-xp-com-a-headline-capta-r-916-mi.ghtml</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>Fundo de venture capital da XP com a Headline capta R$ 916 mi</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>Valor · jun 2022</t>
+        </is>
+      </c>
       <c r="Z50" t="inlineStr"/>
     </row>
     <row r="51">
@@ -4255,7 +4475,11 @@
         <f>IF(L51&lt;&gt;"",L51,_xlfn.TEXTJOIN(" · ",TRUE,IF(F51&lt;&gt;"","Fundador",""),IF(G51&lt;&gt;"","Anjo",""),IF(H51&lt;&gt;"","VC",""),IF(I51&lt;&gt;"","Gestão",""),IF(J51&lt;&gt;"","Conselho",""),IF(K51&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N51" t="inlineStr"/>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Vendida à Creditas</t>
+        </is>
+      </c>
       <c r="O51" s="5" t="inlineStr">
         <is>
           <t>2020</t>
@@ -4318,7 +4542,11 @@
         <f>IF(L52&lt;&gt;"",L52,_xlfn.TEXTJOIN(" · ",TRUE,IF(F52&lt;&gt;"","Fundador",""),IF(G52&lt;&gt;"","Anjo",""),IF(H52&lt;&gt;"","VC",""),IF(I52&lt;&gt;"","Gestão",""),IF(J52&lt;&gt;"","Conselho",""),IF(K52&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N52" t="inlineStr"/>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Vendida à XP Inc.</t>
+        </is>
+      </c>
       <c r="O52" s="5" t="inlineStr">
         <is>
           <t>2019</t>
@@ -4519,7 +4747,11 @@
         <f>IF(L55&lt;&gt;"",L55,_xlfn.TEXTJOIN(" · ",TRUE,IF(F55&lt;&gt;"","Fundador",""),IF(G55&lt;&gt;"","Anjo",""),IF(H55&lt;&gt;"","VC",""),IF(I55&lt;&gt;"","Gestão",""),IF(J55&lt;&gt;"","Conselho",""),IF(K55&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N55" t="inlineStr"/>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Vendida à Renner</t>
+        </is>
+      </c>
       <c r="O55" s="5" t="inlineStr">
         <is>
           <t>2018</t>
@@ -4527,7 +4759,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Adquirida · 2021</t>
+          <t>Saída · 2021</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -4730,7 +4962,11 @@
           <t>2014</t>
         </is>
       </c>
-      <c r="P58" t="inlineStr"/>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q58" t="inlineStr">
         <is>
           <t>https://www.incognia.com/</t>
@@ -4852,14 +5088,22 @@
           <t>2013</t>
         </is>
       </c>
-      <c r="P60" t="inlineStr"/>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr"/>
       <c r="U60" t="inlineStr"/>
       <c r="V60" t="inlineStr"/>
-      <c r="W60" t="inlineStr"/>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>https://retail.economictimes.indiatimes.com/news/e-commerce/e-tailing/ibibo-sells-online-payment-unit-payu-india-to-naspers/30471071</t>
+        </is>
+      </c>
       <c r="X60" t="inlineStr"/>
       <c r="Y60" t="inlineStr"/>
       <c r="Z60" t="inlineStr"/>
@@ -4903,7 +5147,11 @@
           <t>2012</t>
         </is>
       </c>
-      <c r="P61" t="inlineStr"/>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q61" t="inlineStr">
         <is>
           <t>https://www.cuponeria.com.br</t>
@@ -4989,9 +5237,21 @@
       <c r="T62" t="inlineStr"/>
       <c r="U62" t="inlineStr"/>
       <c r="V62" t="inlineStr"/>
-      <c r="W62" t="inlineStr"/>
-      <c r="X62" t="inlineStr"/>
-      <c r="Y62" t="inlineStr"/>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>https://www.nytimes.com/2015/11/11/business/dealbook/redpoint-joint-venture-in-brazil-adds-romero-rodrigues-a-top-entrepreneur.html</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>Redpoint Joint Venture in Brazil Adds Romero Rodrigues, a Top Entrepreneur</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>New York Times · nov 2015</t>
+        </is>
+      </c>
       <c r="Z62" t="inlineStr"/>
     </row>
     <row r="63">
@@ -5033,7 +5293,11 @@
           <t>2012</t>
         </is>
       </c>
-      <c r="P63" t="inlineStr"/>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr">
         <is>
@@ -5092,7 +5356,11 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="P64" t="inlineStr"/>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="inlineStr">
         <is>
@@ -5145,13 +5413,21 @@
         <f>IF(L65&lt;&gt;"",L65,_xlfn.TEXTJOIN(" · ",TRUE,IF(F65&lt;&gt;"","Fundador",""),IF(G65&lt;&gt;"","Anjo",""),IF(H65&lt;&gt;"","VC",""),IF(I65&lt;&gt;"","Gestão",""),IF(J65&lt;&gt;"","Conselho",""),IF(K65&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N65" t="inlineStr"/>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Fundida com PayU</t>
+        </is>
+      </c>
       <c r="O65" s="5" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="P65" t="inlineStr"/>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="inlineStr">
         <is>
@@ -5210,7 +5486,11 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="P66" t="inlineStr"/>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr">
         <is>
@@ -5269,7 +5549,11 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="P67" t="inlineStr"/>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q67" t="inlineStr">
         <is>
           <t>https://modait.com.br/</t>
@@ -5326,13 +5610,21 @@
         <f>IF(L68&lt;&gt;"",L68,_xlfn.TEXTJOIN(" · ",TRUE,IF(F68&lt;&gt;"","Fundador",""),IF(G68&lt;&gt;"","Anjo",""),IF(H68&lt;&gt;"","VC",""),IF(I68&lt;&gt;"","Gestão",""),IF(J68&lt;&gt;"","Conselho",""),IF(K68&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N68" t="inlineStr"/>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>Vendida à Dentsu</t>
+        </is>
+      </c>
       <c r="O68" s="5" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
       </c>
-      <c r="P68" t="inlineStr"/>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Saída · 2015</t>
+        </is>
+      </c>
       <c r="Q68" t="inlineStr">
         <is>
           <t>https://www.navegg.com/br</t>
@@ -5395,7 +5687,11 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="P69" t="inlineStr"/>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q69" t="inlineStr"/>
       <c r="R69" t="inlineStr">
         <is>
@@ -5450,7 +5746,11 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="P70" t="inlineStr"/>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q70" t="inlineStr"/>
       <c r="R70" t="inlineStr">
         <is>
@@ -5503,13 +5803,21 @@
         <f>IF(L71&lt;&gt;"",L71,_xlfn.TEXTJOIN(" · ",TRUE,IF(F71&lt;&gt;"","Fundador",""),IF(G71&lt;&gt;"","Anjo",""),IF(H71&lt;&gt;"","VC",""),IF(I71&lt;&gt;"","Gestão",""),IF(J71&lt;&gt;"","Conselho",""),IF(K71&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N71" t="inlineStr"/>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Fundida com PayU</t>
+        </is>
+      </c>
       <c r="O71" s="5" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="P71" t="inlineStr"/>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q71" t="inlineStr"/>
       <c r="R71" t="inlineStr">
         <is>
@@ -5568,7 +5876,11 @@
           <t>2010</t>
         </is>
       </c>
-      <c r="P72" t="inlineStr"/>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q72" t="inlineStr"/>
       <c r="R72" t="inlineStr">
         <is>
@@ -5627,7 +5939,11 @@
           <t>2010</t>
         </is>
       </c>
-      <c r="P73" t="inlineStr"/>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q73" t="inlineStr"/>
       <c r="R73" t="inlineStr">
         <is>
@@ -5680,13 +5996,21 @@
         <f>IF(L74&lt;&gt;"",L74,_xlfn.TEXTJOIN(" · ",TRUE,IF(F74&lt;&gt;"","Fundador",""),IF(G74&lt;&gt;"","Anjo",""),IF(H74&lt;&gt;"","VC",""),IF(I74&lt;&gt;"","Gestão",""),IF(J74&lt;&gt;"","Conselho",""),IF(K74&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N74" t="inlineStr"/>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>Vendida à A&amp;EIGHT</t>
+        </is>
+      </c>
       <c r="O74" s="5" t="inlineStr">
         <is>
           <t>2009</t>
         </is>
       </c>
-      <c r="P74" t="inlineStr"/>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Saída · 2024</t>
+        </is>
+      </c>
       <c r="Q74" t="inlineStr"/>
       <c r="R74" t="inlineStr">
         <is>
@@ -5743,13 +6067,21 @@
         <f>IF(L75&lt;&gt;"",L75,_xlfn.TEXTJOIN(" · ",TRUE,IF(F75&lt;&gt;"","Fundador",""),IF(G75&lt;&gt;"","Anjo",""),IF(H75&lt;&gt;"","VC",""),IF(I75&lt;&gt;"","Gestão",""),IF(J75&lt;&gt;"","Conselho",""),IF(K75&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N75" t="inlineStr"/>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>Fundida com PayU</t>
+        </is>
+      </c>
       <c r="O75" s="5" t="inlineStr">
         <is>
           <t>2008</t>
         </is>
       </c>
-      <c r="P75" t="inlineStr"/>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q75" t="inlineStr"/>
       <c r="R75" t="inlineStr">
         <is>
@@ -5810,13 +6142,21 @@
         <f>IF(L76&lt;&gt;"",L76,_xlfn.TEXTJOIN(" · ",TRUE,IF(F76&lt;&gt;"","Fundador",""),IF(G76&lt;&gt;"","Anjo",""),IF(H76&lt;&gt;"","VC",""),IF(I76&lt;&gt;"","Gestão",""),IF(J76&lt;&gt;"","Conselho",""),IF(K76&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N76" t="inlineStr"/>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>Fundida com PayU</t>
+        </is>
+      </c>
       <c r="O76" s="5" t="inlineStr">
         <is>
           <t>2008</t>
         </is>
       </c>
-      <c r="P76" t="inlineStr"/>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr">
         <is>
@@ -5869,13 +6209,21 @@
         <f>IF(L77&lt;&gt;"",L77,_xlfn.TEXTJOIN(" · ",TRUE,IF(F77&lt;&gt;"","Fundador",""),IF(G77&lt;&gt;"","Anjo",""),IF(H77&lt;&gt;"","VC",""),IF(I77&lt;&gt;"","Gestão",""),IF(J77&lt;&gt;"","Conselho",""),IF(K77&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N77" t="inlineStr"/>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>Vendida à Nielsen</t>
+        </is>
+      </c>
       <c r="O77" s="5" t="inlineStr">
         <is>
           <t>2007</t>
         </is>
       </c>
-      <c r="P77" t="inlineStr"/>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Saída · 2024</t>
+        </is>
+      </c>
       <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr">
         <is>
@@ -5997,7 +6345,11 @@
           <t>2006</t>
         </is>
       </c>
-      <c r="P79" t="inlineStr"/>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q79" t="inlineStr"/>
       <c r="R79" t="inlineStr">
         <is>
@@ -6056,7 +6408,11 @@
           <t>2006</t>
         </is>
       </c>
-      <c r="P80" t="inlineStr"/>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q80" t="inlineStr">
         <is>
           <t>https://www.quebarato.com.br/</t>
@@ -6113,13 +6469,21 @@
         <f>IF(L81&lt;&gt;"",L81,_xlfn.TEXTJOIN(" · ",TRUE,IF(F81&lt;&gt;"","Fundador",""),IF(G81&lt;&gt;"","Anjo",""),IF(H81&lt;&gt;"","VC",""),IF(I81&lt;&gt;"","Gestão",""),IF(J81&lt;&gt;"","Conselho",""),IF(K81&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N81" t="inlineStr"/>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>Vendida à Locaweb</t>
+        </is>
+      </c>
       <c r="O81" s="5" t="inlineStr">
         <is>
           <t>2004</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr"/>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q81" t="inlineStr"/>
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="inlineStr"/>
@@ -6164,13 +6528,21 @@
         <f>IF(L82&lt;&gt;"",L82,_xlfn.TEXTJOIN(" · ",TRUE,IF(F82&lt;&gt;"","Fundador",""),IF(G82&lt;&gt;"","Anjo",""),IF(H82&lt;&gt;"","VC",""),IF(I82&lt;&gt;"","Gestão",""),IF(J82&lt;&gt;"","Conselho",""),IF(K82&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N82" t="inlineStr"/>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Vendida à JWT</t>
+        </is>
+      </c>
       <c r="O82" s="5" t="inlineStr">
         <is>
           <t>2004</t>
         </is>
       </c>
-      <c r="P82" t="inlineStr"/>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q82" t="inlineStr"/>
       <c r="R82" t="inlineStr">
         <is>
@@ -6233,7 +6605,11 @@
           <t>2004</t>
         </is>
       </c>
-      <c r="P83" t="inlineStr"/>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q83" t="inlineStr"/>
       <c r="R83" t="inlineStr"/>
       <c r="S83" t="inlineStr"/>
@@ -6278,10 +6654,22 @@
         <f>IF(L84&lt;&gt;"",L84,_xlfn.TEXTJOIN(" · ",TRUE,IF(F84&lt;&gt;"","Fundador",""),IF(G84&lt;&gt;"","Anjo",""),IF(H84&lt;&gt;"","VC",""),IF(I84&lt;&gt;"","Gestão",""),IF(J84&lt;&gt;"","Conselho",""),IF(K84&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N84" t="inlineStr"/>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>Vendida à Genstar Capital</t>
+        </is>
+      </c>
       <c r="O84" s="5" t="inlineStr"/>
-      <c r="P84" t="inlineStr"/>
-      <c r="Q84" t="inlineStr"/>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>https://awl.com/</t>
+        </is>
+      </c>
       <c r="R84" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/awl-fee7</t>
@@ -6311,7 +6699,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="C85" s="5" t="inlineStr"/>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="D85" t="inlineStr">
         <is>
           <t>Biosphera (B&amp;Partners)</t>
@@ -6326,7 +6718,11 @@
       </c>
       <c r="H85" s="5" t="inlineStr"/>
       <c r="I85" s="5" t="inlineStr"/>
-      <c r="J85" s="5" t="inlineStr"/>
+      <c r="J85" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K85" s="5" t="inlineStr"/>
       <c r="L85" t="inlineStr"/>
       <c r="M85" s="6">
@@ -6406,7 +6802,11 @@
       </c>
       <c r="N86" t="inlineStr"/>
       <c r="O86" s="5" t="inlineStr"/>
-      <c r="P86" t="inlineStr"/>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q86" t="inlineStr">
         <is>
           <t>https://bovplatform.com/about</t>
@@ -6447,7 +6847,11 @@
           <t>Canal da Peça</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>CWS (Canal da Peça)</t>
+        </is>
+      </c>
       <c r="F87" s="5" t="inlineStr"/>
       <c r="G87" s="5" t="inlineStr">
         <is>
@@ -6465,7 +6869,11 @@
       </c>
       <c r="N87" t="inlineStr"/>
       <c r="O87" s="5" t="inlineStr"/>
-      <c r="P87" t="inlineStr"/>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q87" t="inlineStr">
         <is>
           <t>https://www.canaldapeca.com.br/</t>
@@ -6650,7 +7058,11 @@
       </c>
       <c r="N90" t="inlineStr"/>
       <c r="O90" s="5" t="inlineStr"/>
-      <c r="P90" t="inlineStr"/>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q90" t="inlineStr">
         <is>
           <t>https://www.galena.com</t>
@@ -6709,7 +7121,11 @@
       </c>
       <c r="N91" t="inlineStr"/>
       <c r="O91" s="5" t="inlineStr"/>
-      <c r="P91" t="inlineStr"/>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q91" t="inlineStr"/>
       <c r="R91" t="inlineStr">
         <is>
@@ -6764,7 +7180,11 @@
       </c>
       <c r="N92" t="inlineStr"/>
       <c r="O92" s="5" t="inlineStr"/>
-      <c r="P92" t="inlineStr"/>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q92" t="inlineStr"/>
       <c r="R92" t="inlineStr"/>
       <c r="S92" t="inlineStr">
@@ -6815,7 +7235,11 @@
       </c>
       <c r="N93" t="inlineStr"/>
       <c r="O93" s="5" t="inlineStr"/>
-      <c r="P93" t="inlineStr"/>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q93" t="inlineStr">
         <is>
           <t>https://ingresse.com/</t>
@@ -6939,7 +7363,7 @@
       <c r="O95" s="5" t="inlineStr"/>
       <c r="P95" t="inlineStr">
         <is>
-          <t>Ativa</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
@@ -7000,7 +7424,11 @@
       </c>
       <c r="N96" t="inlineStr"/>
       <c r="O96" s="5" t="inlineStr"/>
-      <c r="P96" t="inlineStr"/>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q96" t="inlineStr">
         <is>
           <t>https://qipu.com.br/</t>
@@ -7116,9 +7544,17 @@
         <f>IF(L98&lt;&gt;"",L98,_xlfn.TEXTJOIN(" · ",TRUE,IF(F98&lt;&gt;"","Fundador",""),IF(G98&lt;&gt;"","Anjo",""),IF(H98&lt;&gt;"","VC",""),IF(I98&lt;&gt;"","Gestão",""),IF(J98&lt;&gt;"","Conselho",""),IF(K98&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N98" t="inlineStr"/>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>Vendida aos gestores</t>
+        </is>
+      </c>
       <c r="O98" s="5" t="inlineStr"/>
-      <c r="P98" t="inlineStr"/>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q98" t="inlineStr">
         <is>
           <t>https://spventures.com.br/</t>
@@ -7177,7 +7613,11 @@
       </c>
       <c r="N99" t="inlineStr"/>
       <c r="O99" s="5" t="inlineStr"/>
-      <c r="P99" t="inlineStr"/>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q99" t="inlineStr">
         <is>
           <t>https://setyou.com.br/</t>
@@ -7234,9 +7674,17 @@
         <f>IF(L100&lt;&gt;"",L100,_xlfn.TEXTJOIN(" · ",TRUE,IF(F100&lt;&gt;"","Fundador",""),IF(G100&lt;&gt;"","Anjo",""),IF(H100&lt;&gt;"","VC",""),IF(I100&lt;&gt;"","Gestão",""),IF(J100&lt;&gt;"","Conselho",""),IF(K100&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N100" t="inlineStr"/>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>Vendida à Decolar</t>
+        </is>
+      </c>
       <c r="O100" s="5" t="inlineStr"/>
-      <c r="P100" t="inlineStr"/>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q100" t="inlineStr"/>
       <c r="R100" t="inlineStr">
         <is>
@@ -8038,7 +8486,11 @@
           <t>2016</t>
         </is>
       </c>
-      <c r="P114" t="inlineStr"/>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q114" t="inlineStr"/>
       <c r="R114" t="inlineStr">
         <is>
@@ -8099,7 +8551,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>Ativa</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr"/>
@@ -8156,7 +8608,11 @@
           <t>2004</t>
         </is>
       </c>
-      <c r="P116" t="inlineStr"/>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q116" t="inlineStr"/>
       <c r="R116" t="inlineStr"/>
       <c r="S116" t="inlineStr">
@@ -8211,7 +8667,11 @@
           <t>2004</t>
         </is>
       </c>
-      <c r="P117" t="inlineStr"/>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q117" t="inlineStr"/>
       <c r="R117" t="inlineStr">
         <is>
@@ -8264,7 +8724,7 @@
       <c r="O118" s="5" t="inlineStr"/>
       <c r="P118" t="inlineStr">
         <is>
-          <t>Ativa</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q118" t="inlineStr"/>
@@ -8317,7 +8777,11 @@
       </c>
       <c r="N119" t="inlineStr"/>
       <c r="O119" s="5" t="inlineStr"/>
-      <c r="P119" t="inlineStr"/>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q119" t="inlineStr"/>
       <c r="R119" t="inlineStr"/>
       <c r="S119" t="inlineStr"/>
@@ -8364,7 +8828,11 @@
       </c>
       <c r="N120" t="inlineStr"/>
       <c r="O120" s="5" t="inlineStr"/>
-      <c r="P120" t="inlineStr"/>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q120" t="inlineStr">
         <is>
           <t>https://jet8.io/</t>
@@ -8419,7 +8887,11 @@
       </c>
       <c r="N121" t="inlineStr"/>
       <c r="O121" s="5" t="inlineStr"/>
-      <c r="P121" t="inlineStr"/>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q121" t="inlineStr">
         <is>
           <t>https://roomorama.com/</t>
@@ -8476,7 +8948,7 @@
       <c r="O122" s="5" t="inlineStr"/>
       <c r="P122" t="inlineStr">
         <is>
-          <t>Adquirida</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q122" t="inlineStr"/>
@@ -8533,7 +9005,11 @@
       </c>
       <c r="N123" t="inlineStr"/>
       <c r="O123" s="5" t="inlineStr"/>
-      <c r="P123" t="inlineStr"/>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q123" t="inlineStr"/>
       <c r="R123" t="inlineStr">
         <is>
@@ -8590,7 +9066,7 @@
       <c r="O124" s="5" t="inlineStr"/>
       <c r="P124" t="inlineStr">
         <is>
-          <t>Ativa</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr"/>
@@ -8645,9 +9121,17 @@
         <f>IF(L125&lt;&gt;"",L125,_xlfn.TEXTJOIN(" · ",TRUE,IF(F125&lt;&gt;"","Fundador",""),IF(G125&lt;&gt;"","Anjo",""),IF(H125&lt;&gt;"","VC",""),IF(I125&lt;&gt;"","Gestão",""),IF(J125&lt;&gt;"","Conselho",""),IF(K125&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N125" t="inlineStr"/>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>Vendida à Sprinkr</t>
+        </is>
+      </c>
       <c r="O125" s="5" t="inlineStr"/>
-      <c r="P125" t="inlineStr"/>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>Saída · 2015</t>
+        </is>
+      </c>
       <c r="Q125" t="inlineStr"/>
       <c r="R125" t="inlineStr">
         <is>
@@ -8702,7 +9186,11 @@
       </c>
       <c r="N126" t="inlineStr"/>
       <c r="O126" s="5" t="inlineStr"/>
-      <c r="P126" t="inlineStr"/>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q126" t="inlineStr">
         <is>
           <t>https://shoes4you.com.br/</t>
@@ -8761,7 +9249,11 @@
       </c>
       <c r="N127" t="inlineStr"/>
       <c r="O127" s="5" t="inlineStr"/>
-      <c r="P127" t="inlineStr"/>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q127" t="inlineStr"/>
       <c r="R127" t="inlineStr">
         <is>
@@ -8812,7 +9304,11 @@
       </c>
       <c r="N128" t="inlineStr"/>
       <c r="O128" s="5" t="inlineStr"/>
-      <c r="P128" t="inlineStr"/>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
       <c r="Q128" t="inlineStr"/>
       <c r="R128" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(portfolio): Arena (VC, via Redpoint) e Cortex (VC e conselho)
Arena: seed de jun 2020 liderada pela Redpoint eventures; Cortex: conselho
desde nov 2015. Perfis no Crunchbase conferidos (site igual e o Romero no
perfil). Sem logo por enquanto: o card mostra o nome.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Empresas'!$A$1:$Z$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Empresas'!$A$1:$Z$130</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -736,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z128"/>
+  <dimension ref="A1:Z130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4374,32 +4374,24 @@
           <t>x</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="C50" s="5" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t>XP Inc.</t>
+          <t>Arena</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="5" t="inlineStr"/>
-      <c r="H50" s="5" t="inlineStr"/>
-      <c r="I50" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr"/>
       <c r="J50" s="5" t="inlineStr"/>
       <c r="K50" s="5" t="inlineStr"/>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>Sócio e executivo</t>
-        </is>
-      </c>
+      <c r="L50" t="inlineStr"/>
       <c r="M50" s="6">
         <f>IF(L50&lt;&gt;"",L50,_xlfn.TEXTJOIN(" · ",TRUE,IF(F50&lt;&gt;"","Fundador",""),IF(G50&lt;&gt;"","Anjo",""),IF(H50&lt;&gt;"","VC",""),IF(I50&lt;&gt;"","Gestão",""),IF(J50&lt;&gt;"","Conselho",""),IF(K50&lt;&gt;"","Buscapé","")))</f>
         <v/>
@@ -4407,45 +4399,41 @@
       <c r="N50" t="inlineStr"/>
       <c r="O50" s="5" t="inlineStr">
         <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>https://arena.im/</t>
+        </is>
+      </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/grupo-xp</t>
-        </is>
-      </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t>xp-inc.png</t>
-        </is>
-      </c>
+          <t>https://www.crunchbase.com/organization/arena-im</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr"/>
-      <c r="W50" t="inlineStr">
-        <is>
-          <t>https://valor.globo.com/financas/noticia/2022/06/09/fundo-de-venture-capital-da-xp-com-a-headline-capta-r-916-mi.ghtml</t>
-        </is>
-      </c>
-      <c r="X50" t="inlineStr">
-        <is>
-          <t>Fundo de venture capital da XP com a Headline capta R$ 916 mi</t>
-        </is>
-      </c>
-      <c r="Y50" t="inlineStr">
-        <is>
-          <t>Valor · jun 2022</t>
-        </is>
-      </c>
-      <c r="Z50" t="inlineStr"/>
+      <c r="W50" t="inlineStr"/>
+      <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr"/>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>Via Redpoint eventures (seed de jun 2020).</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>490</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -4453,66 +4441,78 @@
           <t>x</t>
         </is>
       </c>
-      <c r="C51" s="5" t="inlineStr"/>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Kzas</t>
+          <t>XP Inc.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" s="5" t="inlineStr"/>
       <c r="G51" s="5" t="inlineStr"/>
-      <c r="H51" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="I51" s="5" t="inlineStr"/>
+      <c r="H51" s="5" t="inlineStr"/>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J51" s="5" t="inlineStr"/>
       <c r="K51" s="5" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Sócio e executivo</t>
+        </is>
+      </c>
       <c r="M51" s="6">
         <f>IF(L51&lt;&gt;"",L51,_xlfn.TEXTJOIN(" · ",TRUE,IF(F51&lt;&gt;"","Fundador",""),IF(G51&lt;&gt;"","Anjo",""),IF(H51&lt;&gt;"","VC",""),IF(I51&lt;&gt;"","Gestão",""),IF(J51&lt;&gt;"","Conselho",""),IF(K51&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>Vendida à Creditas</t>
-        </is>
-      </c>
+      <c r="N51" t="inlineStr"/>
       <c r="O51" s="5" t="inlineStr">
         <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/kzas-ai</t>
+          <t>https://www.crunchbase.com/organization/grupo-xp</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>kzas.png</t>
+          <t>xp-inc.png</t>
         </is>
       </c>
       <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr"/>
-      <c r="W51" t="inlineStr"/>
-      <c r="X51" t="inlineStr"/>
-      <c r="Y51" t="inlineStr"/>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>https://valor.globo.com/financas/noticia/2022/06/09/fundo-de-venture-capital-da-xp-com-a-headline-capta-r-916-mi.ghtml</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>Fundo de venture capital da XP com a Headline capta R$ 916 mi</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>Valor · jun 2022</t>
+        </is>
+      </c>
       <c r="Z51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>500</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
@@ -4523,7 +4523,7 @@
       <c r="C52" s="5" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Antecipa</t>
+          <t>Kzas</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -4544,12 +4544,12 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>Vendida à XP Inc.</t>
+          <t>Vendida à Creditas</t>
         </is>
       </c>
       <c r="O52" s="5" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -4557,19 +4557,15 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr">
-        <is>
-          <t>https://antecipa.com/</t>
-        </is>
-      </c>
+      <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/antecipa</t>
+          <t>https://www.crunchbase.com/organization/kzas-ai</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>antecipa.png</t>
+          <t>kzas.png</t>
         </is>
       </c>
       <c r="T52" t="inlineStr"/>
@@ -4583,7 +4579,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>510</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -4594,7 +4590,7 @@
       <c r="C53" s="5" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>GigU</t>
+          <t>Antecipa</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -4613,7 +4609,11 @@
         <f>IF(L53&lt;&gt;"",L53,_xlfn.TEXTJOIN(" · ",TRUE,IF(F53&lt;&gt;"","Fundador",""),IF(G53&lt;&gt;"","Anjo",""),IF(H53&lt;&gt;"","VC",""),IF(I53&lt;&gt;"","Gestão",""),IF(J53&lt;&gt;"","Conselho",""),IF(K53&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N53" t="inlineStr"/>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Vendida à XP Inc.</t>
+        </is>
+      </c>
       <c r="O53" s="5" t="inlineStr">
         <is>
           <t>2019</t>
@@ -4621,22 +4621,22 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>Ativa</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>https://site.stopclub.com.br/</t>
+          <t>https://antecipa.com/</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/stopclub</t>
+          <t>https://www.crunchbase.com/organization/antecipa</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>gigu.png</t>
+          <t>antecipa.png</t>
         </is>
       </c>
       <c r="T53" t="inlineStr"/>
@@ -4650,7 +4650,7 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>520</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
@@ -4661,7 +4661,7 @@
       <c r="C54" s="5" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Vittude</t>
+          <t>GigU</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -4693,17 +4693,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>https://vittude.com/</t>
+          <t>https://site.stopclub.com.br/</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/vittude</t>
+          <t>https://www.crunchbase.com/organization/stopclub</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>vittude.png</t>
+          <t>gigu.png</t>
         </is>
       </c>
       <c r="T54" t="inlineStr"/>
@@ -4717,7 +4717,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>530</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
@@ -4728,7 +4728,7 @@
       <c r="C55" s="5" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Repassa</t>
+          <t>Vittude</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -4747,60 +4747,44 @@
         <f>IF(L55&lt;&gt;"",L55,_xlfn.TEXTJOIN(" · ",TRUE,IF(F55&lt;&gt;"","Fundador",""),IF(G55&lt;&gt;"","Anjo",""),IF(H55&lt;&gt;"","VC",""),IF(I55&lt;&gt;"","Gestão",""),IF(J55&lt;&gt;"","Conselho",""),IF(K55&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>Vendida à Renner</t>
-        </is>
-      </c>
+      <c r="N55" t="inlineStr"/>
       <c r="O55" s="5" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Saída · 2021</t>
+          <t>Ativa</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>https://www.repassa.com.br</t>
+          <t>https://vittude.com/</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/repassa</t>
+          <t>https://www.crunchbase.com/organization/vittude</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>repassa.png</t>
+          <t>vittude.png</t>
         </is>
       </c>
       <c r="T55" t="inlineStr"/>
       <c r="U55" t="inlineStr"/>
       <c r="V55" t="inlineStr"/>
-      <c r="W55" t="inlineStr">
-        <is>
-          <t>https://braziljournal.com/renner-compra-repassa-e-entra-no-mercado-de-usados/</t>
-        </is>
-      </c>
-      <c r="X55" t="inlineStr">
-        <is>
-          <t>Renner compra a Repassa</t>
-        </is>
-      </c>
-      <c r="Y55" t="inlineStr">
-        <is>
-          <t>Brazil Journal · jul 2021</t>
-        </is>
-      </c>
+      <c r="W55" t="inlineStr"/>
+      <c r="X55" t="inlineStr"/>
+      <c r="Y55" t="inlineStr"/>
       <c r="Z55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>540</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
@@ -4811,59 +4795,79 @@
       <c r="C56" s="5" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ABFintechs</t>
+          <t>Repassa</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" s="5" t="inlineStr"/>
       <c r="G56" s="5" t="inlineStr"/>
-      <c r="H56" s="5" t="inlineStr"/>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I56" s="5" t="inlineStr"/>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J56" s="5" t="inlineStr"/>
       <c r="K56" s="5" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
       <c r="M56" s="6">
         <f>IF(L56&lt;&gt;"",L56,_xlfn.TEXTJOIN(" · ",TRUE,IF(F56&lt;&gt;"","Fundador",""),IF(G56&lt;&gt;"","Anjo",""),IF(H56&lt;&gt;"","VC",""),IF(I56&lt;&gt;"","Gestão",""),IF(J56&lt;&gt;"","Conselho",""),IF(K56&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N56" t="inlineStr"/>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Vendida à Renner</t>
+        </is>
+      </c>
       <c r="O56" s="5" t="inlineStr">
         <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="P56" t="inlineStr"/>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Saída · 2021</t>
+        </is>
+      </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>https://www.abfintechs.com.br/</t>
+          <t>https://www.repassa.com.br</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/abfintechs</t>
+          <t>https://www.crunchbase.com/organization/repassa</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>abfintechs.png</t>
+          <t>repassa.png</t>
         </is>
       </c>
       <c r="T56" t="inlineStr"/>
       <c r="U56" t="inlineStr"/>
       <c r="V56" t="inlineStr"/>
-      <c r="W56" t="inlineStr"/>
-      <c r="X56" t="inlineStr"/>
-      <c r="Y56" t="inlineStr"/>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>https://braziljournal.com/renner-compra-repassa-e-entra-no-mercado-de-usados/</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>Renner compra a Repassa</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>Brazil Journal · jul 2021</t>
+        </is>
+      </c>
       <c r="Z56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>560</t>
+          <t>550</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
@@ -4874,19 +4878,19 @@
       <c r="C57" s="5" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Consulta do Bem</t>
+          <t>ABFintechs</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" s="5" t="inlineStr"/>
       <c r="G57" s="5" t="inlineStr"/>
-      <c r="H57" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H57" s="5" t="inlineStr"/>
       <c r="I57" s="5" t="inlineStr"/>
-      <c r="J57" s="5" t="inlineStr"/>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K57" s="5" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
       <c r="M57" s="6">
@@ -4896,23 +4900,23 @@
       <c r="N57" t="inlineStr"/>
       <c r="O57" s="5" t="inlineStr">
         <is>
-          <t>2016</t>
-        </is>
-      </c>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>Encerrada</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr"/>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>https://www.abfintechs.com.br/</t>
+        </is>
+      </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/consulta-do-bem</t>
+          <t>https://www.crunchbase.com/organization/abfintechs</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>consulta-do-bem.png</t>
+          <t>abfintechs.png</t>
         </is>
       </c>
       <c r="T57" t="inlineStr"/>
@@ -4926,7 +4930,7 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>620</t>
+          <t>560</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
@@ -4937,20 +4941,20 @@
       <c r="C58" s="5" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>In Loco</t>
+          <t>Consulta do Bem</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" s="5" t="inlineStr"/>
       <c r="G58" s="5" t="inlineStr"/>
-      <c r="H58" s="5" t="inlineStr"/>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I58" s="5" t="inlineStr"/>
       <c r="J58" s="5" t="inlineStr"/>
-      <c r="K58" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K58" s="5" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
       <c r="M58" s="6">
         <f>IF(L58&lt;&gt;"",L58,_xlfn.TEXTJOIN(" · ",TRUE,IF(F58&lt;&gt;"","Fundador",""),IF(G58&lt;&gt;"","Anjo",""),IF(H58&lt;&gt;"","VC",""),IF(I58&lt;&gt;"","Gestão",""),IF(J58&lt;&gt;"","Conselho",""),IF(K58&lt;&gt;"","Buscapé","")))</f>
@@ -4959,7 +4963,7 @@
       <c r="N58" t="inlineStr"/>
       <c r="O58" s="5" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -4967,19 +4971,15 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q58" t="inlineStr">
-        <is>
-          <t>https://www.incognia.com/</t>
-        </is>
-      </c>
+      <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/ubee</t>
+          <t>https://www.crunchbase.com/organization/consulta-do-bem</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>in-loco.png</t>
+          <t>consulta-do-bem.png</t>
         </is>
       </c>
       <c r="T58" t="inlineStr"/>
@@ -4993,7 +4993,7 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>570</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -5004,13 +5004,17 @@
       <c r="C59" s="5" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>PayU</t>
+          <t>Cortex</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" s="5" t="inlineStr"/>
       <c r="G59" s="5" t="inlineStr"/>
-      <c r="H59" s="5" t="inlineStr"/>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I59" s="5" t="inlineStr"/>
       <c r="J59" s="5" t="inlineStr">
         <is>
@@ -5026,44 +5030,52 @@
       <c r="N59" t="inlineStr"/>
       <c r="O59" s="5" t="inlineStr">
         <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="P59" t="inlineStr"/>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>https://corporate.payu.com</t>
+          <t>https://www.cortex-intelligence.com/en/</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/payu</t>
-        </is>
-      </c>
-      <c r="S59" t="inlineStr">
-        <is>
-          <t>payu.png</t>
-        </is>
-      </c>
+          <t>https://www.crunchbase.com/organization/cortex-intelligence</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr"/>
       <c r="U59" t="inlineStr"/>
       <c r="V59" t="inlineStr"/>
       <c r="W59" t="inlineStr"/>
       <c r="X59" t="inlineStr"/>
       <c r="Y59" t="inlineStr"/>
-      <c r="Z59" t="inlineStr"/>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>Via Redpoint eventures; conselho desde nov 2015 (Crunchbase).</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>720</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr"/>
+          <t>620</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="C60" s="5" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Btarget</t>
+          <t>In Loco</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -5085,7 +5097,7 @@
       <c r="N60" t="inlineStr"/>
       <c r="O60" s="5" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -5093,17 +5105,25 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>https://www.incognia.com/</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/ubee</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>in-loco.png</t>
+        </is>
+      </c>
       <c r="T60" t="inlineStr"/>
       <c r="U60" t="inlineStr"/>
       <c r="V60" t="inlineStr"/>
-      <c r="W60" t="inlineStr">
-        <is>
-          <t>https://retail.economictimes.indiatimes.com/news/e-commerce/e-tailing/ibibo-sells-online-payment-unit-payu-india-to-naspers/30471071</t>
-        </is>
-      </c>
+      <c r="W60" t="inlineStr"/>
       <c r="X60" t="inlineStr"/>
       <c r="Y60" t="inlineStr"/>
       <c r="Z60" t="inlineStr"/>
@@ -5111,7 +5131,7 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>640</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
@@ -5122,7 +5142,7 @@
       <c r="C61" s="5" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Cuponeria</t>
+          <t>PayU</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -5130,12 +5150,12 @@
       <c r="G61" s="5" t="inlineStr"/>
       <c r="H61" s="5" t="inlineStr"/>
       <c r="I61" s="5" t="inlineStr"/>
-      <c r="J61" s="5" t="inlineStr"/>
-      <c r="K61" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K61" s="5" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>
       <c r="M61" s="6">
         <f>IF(L61&lt;&gt;"",L61,_xlfn.TEXTJOIN(" · ",TRUE,IF(F61&lt;&gt;"","Fundador",""),IF(G61&lt;&gt;"","Anjo",""),IF(H61&lt;&gt;"","VC",""),IF(I61&lt;&gt;"","Gestão",""),IF(J61&lt;&gt;"","Conselho",""),IF(K61&lt;&gt;"","Buscapé","")))</f>
@@ -5144,27 +5164,23 @@
       <c r="N61" t="inlineStr"/>
       <c r="O61" s="5" t="inlineStr">
         <is>
-          <t>2012</t>
-        </is>
-      </c>
-      <c r="P61" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr"/>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>https://www.cuponeria.com.br</t>
+          <t>https://corporate.payu.com</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/cuponeria</t>
+          <t>https://www.crunchbase.com/organization/payu</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>cuponeria.png</t>
+          <t>payu.png</t>
         </is>
       </c>
       <c r="T61" t="inlineStr"/>
@@ -5178,36 +5194,28 @@
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>740</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>720</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr"/>
       <c r="C62" s="5" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Redpoint e.ventures</t>
+          <t>Btarget</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" s="5" t="inlineStr"/>
       <c r="G62" s="5" t="inlineStr"/>
       <c r="H62" s="5" t="inlineStr"/>
-      <c r="I62" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I62" s="5" t="inlineStr"/>
       <c r="J62" s="5" t="inlineStr"/>
-      <c r="K62" s="5" t="inlineStr"/>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>Sócio de Gestora</t>
-        </is>
-      </c>
+      <c r="K62" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr"/>
       <c r="M62" s="6">
         <f>IF(L62&lt;&gt;"",L62,_xlfn.TEXTJOIN(" · ",TRUE,IF(F62&lt;&gt;"","Fundador",""),IF(G62&lt;&gt;"","Anjo",""),IF(H62&lt;&gt;"","VC",""),IF(I62&lt;&gt;"","Gestão",""),IF(J62&lt;&gt;"","Conselho",""),IF(K62&lt;&gt;"","Buscapé","")))</f>
         <v/>
@@ -5215,49 +5223,33 @@
       <c r="N62" t="inlineStr"/>
       <c r="O62" s="5" t="inlineStr">
         <is>
-          <t>2012</t>
-        </is>
-      </c>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr">
-        <is>
-          <t>https://rpev.com.br/</t>
-        </is>
-      </c>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/redpoint-eventures</t>
-        </is>
-      </c>
-      <c r="S62" t="inlineStr">
-        <is>
-          <t>redpoint-eventures.png</t>
-        </is>
-      </c>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr"/>
       <c r="U62" t="inlineStr"/>
       <c r="V62" t="inlineStr"/>
       <c r="W62" t="inlineStr">
         <is>
-          <t>https://www.nytimes.com/2015/11/11/business/dealbook/redpoint-joint-venture-in-brazil-adds-romero-rodrigues-a-top-entrepreneur.html</t>
-        </is>
-      </c>
-      <c r="X62" t="inlineStr">
-        <is>
-          <t>Redpoint Joint Venture in Brazil Adds Romero Rodrigues, a Top Entrepreneur</t>
-        </is>
-      </c>
-      <c r="Y62" t="inlineStr">
-        <is>
-          <t>New York Times · nov 2015</t>
-        </is>
-      </c>
+          <t>https://retail.economictimes.indiatimes.com/news/e-commerce/e-tailing/ibibo-sells-online-payment-unit-payu-india-to-naspers/30471071</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr"/>
+      <c r="Y62" t="inlineStr"/>
       <c r="Z62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>750</t>
+          <t>730</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
@@ -5268,7 +5260,7 @@
       <c r="C63" s="5" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Shopcliq</t>
+          <t>Cuponeria</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -5295,18 +5287,22 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>Encerrada</t>
-        </is>
-      </c>
-      <c r="Q63" t="inlineStr"/>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>https://www.cuponeria.com.br</t>
+        </is>
+      </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/shopcliq</t>
+          <t>https://www.crunchbase.com/organization/cuponeria</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>shopcliq.png</t>
+          <t>cuponeria.png</t>
         </is>
       </c>
       <c r="T63" t="inlineStr"/>
@@ -5320,7 +5316,7 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>760</t>
+          <t>740</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
@@ -5331,21 +5327,25 @@
       <c r="C64" s="5" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Brandsclub</t>
+          <t>Redpoint e.ventures</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" s="5" t="inlineStr"/>
       <c r="G64" s="5" t="inlineStr"/>
       <c r="H64" s="5" t="inlineStr"/>
-      <c r="I64" s="5" t="inlineStr"/>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J64" s="5" t="inlineStr"/>
-      <c r="K64" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr"/>
+      <c r="K64" s="5" t="inlineStr"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Sócio de Gestora</t>
+        </is>
+      </c>
       <c r="M64" s="6">
         <f>IF(L64&lt;&gt;"",L64,_xlfn.TEXTJOIN(" · ",TRUE,IF(F64&lt;&gt;"","Fundador",""),IF(G64&lt;&gt;"","Anjo",""),IF(H64&lt;&gt;"","VC",""),IF(I64&lt;&gt;"","Gestão",""),IF(J64&lt;&gt;"","Conselho",""),IF(K64&lt;&gt;"","Buscapé","")))</f>
         <v/>
@@ -5353,37 +5353,49 @@
       <c r="N64" t="inlineStr"/>
       <c r="O64" s="5" t="inlineStr">
         <is>
-          <t>2011</t>
-        </is>
-      </c>
-      <c r="P64" t="inlineStr">
-        <is>
-          <t>Encerrada</t>
-        </is>
-      </c>
-      <c r="Q64" t="inlineStr"/>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>https://rpev.com.br/</t>
+        </is>
+      </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/brandsclub</t>
+          <t>https://www.crunchbase.com/organization/redpoint-eventures</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>brandsclub.png</t>
+          <t>redpoint-eventures.png</t>
         </is>
       </c>
       <c r="T64" t="inlineStr"/>
       <c r="U64" t="inlineStr"/>
       <c r="V64" t="inlineStr"/>
-      <c r="W64" t="inlineStr"/>
-      <c r="X64" t="inlineStr"/>
-      <c r="Y64" t="inlineStr"/>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>https://www.nytimes.com/2015/11/11/business/dealbook/redpoint-joint-venture-in-brazil-adds-romero-rodrigues-a-top-entrepreneur.html</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>Redpoint Joint Venture in Brazil Adds Romero Rodrigues, a Top Entrepreneur</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>New York Times · nov 2015</t>
+        </is>
+      </c>
       <c r="Z64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>770</t>
+          <t>750</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
@@ -5394,7 +5406,7 @@
       <c r="C65" s="5" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>DineroMail</t>
+          <t>Shopcliq</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -5413,30 +5425,26 @@
         <f>IF(L65&lt;&gt;"",L65,_xlfn.TEXTJOIN(" · ",TRUE,IF(F65&lt;&gt;"","Fundador",""),IF(G65&lt;&gt;"","Anjo",""),IF(H65&lt;&gt;"","VC",""),IF(I65&lt;&gt;"","Gestão",""),IF(J65&lt;&gt;"","Conselho",""),IF(K65&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>Fundida com PayU</t>
-        </is>
-      </c>
+      <c r="N65" t="inlineStr"/>
       <c r="O65" s="5" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2012</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/dineromail</t>
+          <t>https://www.crunchbase.com/organization/shopcliq</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>dineromail.png</t>
+          <t>shopcliq.png</t>
         </is>
       </c>
       <c r="T65" t="inlineStr"/>
@@ -5450,7 +5458,7 @@
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>780</t>
+          <t>760</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
@@ -5461,7 +5469,7 @@
       <c r="C66" s="5" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>MeuCarrinho</t>
+          <t>Brandsclub</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -5494,12 +5502,12 @@
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/meucarrinho</t>
+          <t>https://www.crunchbase.com/organization/brandsclub</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>meucarrinho.png</t>
+          <t>brandsclub.png</t>
         </is>
       </c>
       <c r="T66" t="inlineStr"/>
@@ -5513,7 +5521,7 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>790</t>
+          <t>770</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -5524,7 +5532,7 @@
       <c r="C67" s="5" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Moda It</t>
+          <t>DineroMail</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -5543,7 +5551,11 @@
         <f>IF(L67&lt;&gt;"",L67,_xlfn.TEXTJOIN(" · ",TRUE,IF(F67&lt;&gt;"","Fundador",""),IF(G67&lt;&gt;"","Anjo",""),IF(H67&lt;&gt;"","VC",""),IF(I67&lt;&gt;"","Gestão",""),IF(J67&lt;&gt;"","Conselho",""),IF(K67&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N67" t="inlineStr"/>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>Fundida com PayU</t>
+        </is>
+      </c>
       <c r="O67" s="5" t="inlineStr">
         <is>
           <t>2011</t>
@@ -5551,22 +5563,18 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>Encerrada</t>
-        </is>
-      </c>
-      <c r="Q67" t="inlineStr">
-        <is>
-          <t>https://modait.com.br/</t>
-        </is>
-      </c>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr"/>
       <c r="R67" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/moda-it</t>
+          <t>https://www.crunchbase.com/organization/dineromail</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>moda-it.png</t>
+          <t>dineromail.png</t>
         </is>
       </c>
       <c r="T67" t="inlineStr"/>
@@ -5580,7 +5588,7 @@
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>780</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
@@ -5591,7 +5599,7 @@
       <c r="C68" s="5" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Navegg</t>
+          <t>MeuCarrinho</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -5610,11 +5618,7 @@
         <f>IF(L68&lt;&gt;"",L68,_xlfn.TEXTJOIN(" · ",TRUE,IF(F68&lt;&gt;"","Fundador",""),IF(G68&lt;&gt;"","Anjo",""),IF(H68&lt;&gt;"","VC",""),IF(I68&lt;&gt;"","Gestão",""),IF(J68&lt;&gt;"","Conselho",""),IF(K68&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>Vendida à Dentsu</t>
-        </is>
-      </c>
+      <c r="N68" t="inlineStr"/>
       <c r="O68" s="5" t="inlineStr">
         <is>
           <t>2011</t>
@@ -5622,22 +5626,18 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Saída · 2015</t>
-        </is>
-      </c>
-      <c r="Q68" t="inlineStr">
-        <is>
-          <t>https://www.navegg.com/br</t>
-        </is>
-      </c>
+          <t>Encerrada</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/navegg</t>
+          <t>https://www.crunchbase.com/organization/meucarrinho</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>navegg.png</t>
+          <t>meucarrinho.png</t>
         </is>
       </c>
       <c r="T68" t="inlineStr"/>
@@ -5651,7 +5651,7 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>810</t>
+          <t>790</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
@@ -5662,7 +5662,7 @@
       <c r="C69" s="5" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Recomind.net</t>
+          <t>Moda It</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -5692,13 +5692,21 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>https://modait.com.br/</t>
+        </is>
+      </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/recomind-net</t>
-        </is>
-      </c>
-      <c r="S69" t="inlineStr"/>
+          <t>https://www.crunchbase.com/organization/moda-it</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>moda-it.png</t>
+        </is>
+      </c>
       <c r="T69" t="inlineStr"/>
       <c r="U69" t="inlineStr"/>
       <c r="V69" t="inlineStr"/>
@@ -5710,7 +5718,7 @@
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>820</t>
+          <t>800</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
@@ -5721,7 +5729,7 @@
       <c r="C70" s="5" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Urbanizo</t>
+          <t>Navegg</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -5740,7 +5748,11 @@
         <f>IF(L70&lt;&gt;"",L70,_xlfn.TEXTJOIN(" · ",TRUE,IF(F70&lt;&gt;"","Fundador",""),IF(G70&lt;&gt;"","Anjo",""),IF(H70&lt;&gt;"","VC",""),IF(I70&lt;&gt;"","Gestão",""),IF(J70&lt;&gt;"","Conselho",""),IF(K70&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N70" t="inlineStr"/>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Vendida à Dentsu</t>
+        </is>
+      </c>
       <c r="O70" s="5" t="inlineStr">
         <is>
           <t>2011</t>
@@ -5748,18 +5760,22 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>Encerrada</t>
-        </is>
-      </c>
-      <c r="Q70" t="inlineStr"/>
+          <t>Saída · 2015</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>https://www.navegg.com/br</t>
+        </is>
+      </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/urbanizo</t>
+          <t>https://www.crunchbase.com/organization/navegg</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>urbanizo.png</t>
+          <t>navegg.png</t>
         </is>
       </c>
       <c r="T70" t="inlineStr"/>
@@ -5773,7 +5789,7 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>830</t>
+          <t>810</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
@@ -5784,7 +5800,7 @@
       <c r="C71" s="5" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>PagosOnline</t>
+          <t>Recomind.net</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -5803,32 +5819,24 @@
         <f>IF(L71&lt;&gt;"",L71,_xlfn.TEXTJOIN(" · ",TRUE,IF(F71&lt;&gt;"","Fundador",""),IF(G71&lt;&gt;"","Anjo",""),IF(H71&lt;&gt;"","VC",""),IF(I71&lt;&gt;"","Gestão",""),IF(J71&lt;&gt;"","Conselho",""),IF(K71&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N71" t="inlineStr">
-        <is>
-          <t>Fundida com PayU</t>
-        </is>
-      </c>
+      <c r="N71" t="inlineStr"/>
       <c r="O71" s="5" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr"/>
       <c r="R71" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/pagosonline</t>
-        </is>
-      </c>
-      <c r="S71" t="inlineStr">
-        <is>
-          <t>pagosonline.png</t>
-        </is>
-      </c>
+          <t>https://www.crunchbase.com/organization/recomind-net</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr"/>
       <c r="T71" t="inlineStr"/>
       <c r="U71" t="inlineStr"/>
       <c r="V71" t="inlineStr"/>
@@ -5840,7 +5848,7 @@
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>840</t>
+          <t>820</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
@@ -5851,7 +5859,7 @@
       <c r="C72" s="5" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
-          <t>SaveMe</t>
+          <t>Urbanizo</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -5873,7 +5881,7 @@
       <c r="N72" t="inlineStr"/>
       <c r="O72" s="5" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
@@ -5884,12 +5892,12 @@
       <c r="Q72" t="inlineStr"/>
       <c r="R72" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/saveme</t>
+          <t>https://www.crunchbase.com/organization/urbanizo</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>saveme-2026.png</t>
+          <t>urbanizo.png</t>
         </is>
       </c>
       <c r="T72" t="inlineStr"/>
@@ -5903,7 +5911,7 @@
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>850</t>
+          <t>830</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
@@ -5914,7 +5922,7 @@
       <c r="C73" s="5" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
-          <t>eBehavior</t>
+          <t>PagosOnline</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
@@ -5933,7 +5941,11 @@
         <f>IF(L73&lt;&gt;"",L73,_xlfn.TEXTJOIN(" · ",TRUE,IF(F73&lt;&gt;"","Fundador",""),IF(G73&lt;&gt;"","Anjo",""),IF(H73&lt;&gt;"","VC",""),IF(I73&lt;&gt;"","Gestão",""),IF(J73&lt;&gt;"","Conselho",""),IF(K73&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N73" t="inlineStr"/>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>Fundida com PayU</t>
+        </is>
+      </c>
       <c r="O73" s="5" t="inlineStr">
         <is>
           <t>2010</t>
@@ -5941,18 +5953,18 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Encerrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr"/>
       <c r="R73" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/ebehavior-b888</t>
+          <t>https://www.crunchbase.com/organization/pagosonline</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>ebehavior.png</t>
+          <t>pagosonline.png</t>
         </is>
       </c>
       <c r="T73" t="inlineStr"/>
@@ -5966,7 +5978,7 @@
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>860</t>
+          <t>840</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
@@ -5977,7 +5989,7 @@
       <c r="C74" s="5" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Lomadee</t>
+          <t>SaveMe</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -5996,30 +6008,26 @@
         <f>IF(L74&lt;&gt;"",L74,_xlfn.TEXTJOIN(" · ",TRUE,IF(F74&lt;&gt;"","Fundador",""),IF(G74&lt;&gt;"","Anjo",""),IF(H74&lt;&gt;"","VC",""),IF(I74&lt;&gt;"","Gestão",""),IF(J74&lt;&gt;"","Conselho",""),IF(K74&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N74" t="inlineStr">
-        <is>
-          <t>Vendida à A&amp;EIGHT</t>
-        </is>
-      </c>
+      <c r="N74" t="inlineStr"/>
       <c r="O74" s="5" t="inlineStr">
         <is>
-          <t>2009</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>Saída · 2024</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr"/>
       <c r="R74" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/lomadee</t>
+          <t>https://www.crunchbase.com/organization/saveme</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>lomadee.png</t>
+          <t>saveme-2026.png</t>
         </is>
       </c>
       <c r="T74" t="inlineStr"/>
@@ -6033,7 +6041,7 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>870</t>
+          <t>850</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
@@ -6044,14 +6052,10 @@
       <c r="C75" s="5" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Bcash / Pagamento Digital</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Bcash</t>
-        </is>
-      </c>
+          <t>eBehavior</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
       <c r="F75" s="5" t="inlineStr"/>
       <c r="G75" s="5" t="inlineStr"/>
       <c r="H75" s="5" t="inlineStr"/>
@@ -6067,43 +6071,31 @@
         <f>IF(L75&lt;&gt;"",L75,_xlfn.TEXTJOIN(" · ",TRUE,IF(F75&lt;&gt;"","Fundador",""),IF(G75&lt;&gt;"","Anjo",""),IF(H75&lt;&gt;"","VC",""),IF(I75&lt;&gt;"","Gestão",""),IF(J75&lt;&gt;"","Conselho",""),IF(K75&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N75" t="inlineStr">
-        <is>
-          <t>Fundida com PayU</t>
-        </is>
-      </c>
+      <c r="N75" t="inlineStr"/>
       <c r="O75" s="5" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr"/>
       <c r="R75" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/pagamento-digital</t>
+          <t>https://www.crunchbase.com/organization/ebehavior-b888</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>pagamento-digital.png</t>
+          <t>ebehavior.png</t>
         </is>
       </c>
       <c r="T75" t="inlineStr"/>
-      <c r="U75" t="inlineStr">
-        <is>
-          <t>Bcash</t>
-        </is>
-      </c>
-      <c r="V75" t="inlineStr">
-        <is>
-          <t>Pagamento Digital</t>
-        </is>
-      </c>
+      <c r="U75" t="inlineStr"/>
+      <c r="V75" t="inlineStr"/>
       <c r="W75" t="inlineStr"/>
       <c r="X75" t="inlineStr"/>
       <c r="Y75" t="inlineStr"/>
@@ -6112,7 +6104,7 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>880</t>
+          <t>860</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
@@ -6123,7 +6115,7 @@
       <c r="C76" s="5" t="inlineStr"/>
       <c r="D76" t="inlineStr">
         <is>
-          <t>FControl</t>
+          <t>Lomadee</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -6144,28 +6136,28 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>Fundida com PayU</t>
+          <t>Vendida à A&amp;EIGHT</t>
         </is>
       </c>
       <c r="O76" s="5" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>2009</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Saída · 2024</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/f-control</t>
+          <t>https://www.crunchbase.com/organization/lomadee</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>fcontrol.png</t>
+          <t>lomadee.png</t>
         </is>
       </c>
       <c r="T76" t="inlineStr"/>
@@ -6179,7 +6171,7 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>890</t>
+          <t>870</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
@@ -6190,10 +6182,14 @@
       <c r="C77" s="5" t="inlineStr"/>
       <c r="D77" t="inlineStr">
         <is>
-          <t>E-bit</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr"/>
+          <t>Bcash / Pagamento Digital</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Bcash</t>
+        </is>
+      </c>
       <c r="F77" s="5" t="inlineStr"/>
       <c r="G77" s="5" t="inlineStr"/>
       <c r="H77" s="5" t="inlineStr"/>
@@ -6211,33 +6207,41 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>Vendida à Nielsen</t>
+          <t>Fundida com PayU</t>
         </is>
       </c>
       <c r="O77" s="5" t="inlineStr">
         <is>
-          <t>2007</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>Saída · 2024</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/e-bit</t>
+          <t>https://www.crunchbase.com/organization/pagamento-digital</t>
         </is>
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>e-bit.png</t>
+          <t>pagamento-digital.png</t>
         </is>
       </c>
       <c r="T77" t="inlineStr"/>
-      <c r="U77" t="inlineStr"/>
-      <c r="V77" t="inlineStr"/>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>Bcash</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>Pagamento Digital</t>
+        </is>
+      </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
       <c r="Y77" t="inlineStr"/>
@@ -6246,7 +6250,7 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>880</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
@@ -6257,7 +6261,7 @@
       <c r="C78" s="5" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Bondfaro</t>
+          <t>FControl</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -6276,26 +6280,30 @@
         <f>IF(L78&lt;&gt;"",L78,_xlfn.TEXTJOIN(" · ",TRUE,IF(F78&lt;&gt;"","Fundador",""),IF(G78&lt;&gt;"","Anjo",""),IF(H78&lt;&gt;"","VC",""),IF(I78&lt;&gt;"","Gestão",""),IF(J78&lt;&gt;"","Conselho",""),IF(K78&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N78" t="inlineStr"/>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>Fundida com PayU</t>
+        </is>
+      </c>
       <c r="O78" s="5" t="inlineStr">
         <is>
-          <t>2006</t>
-        </is>
-      </c>
-      <c r="P78" t="inlineStr"/>
-      <c r="Q78" t="inlineStr">
-        <is>
-          <t>https://www.bondfaro.com.br/</t>
-        </is>
-      </c>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr"/>
       <c r="R78" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/bondfaro</t>
+          <t>https://www.crunchbase.com/organization/f-control</t>
         </is>
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>bondfaro-2026.png</t>
+          <t>fcontrol.png</t>
         </is>
       </c>
       <c r="T78" t="inlineStr"/>
@@ -6309,7 +6317,7 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>910</t>
+          <t>890</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
@@ -6320,7 +6328,7 @@
       <c r="C79" s="5" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
-          <t>CortaContas</t>
+          <t>E-bit</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -6339,26 +6347,30 @@
         <f>IF(L79&lt;&gt;"",L79,_xlfn.TEXTJOIN(" · ",TRUE,IF(F79&lt;&gt;"","Fundador",""),IF(G79&lt;&gt;"","Anjo",""),IF(H79&lt;&gt;"","VC",""),IF(I79&lt;&gt;"","Gestão",""),IF(J79&lt;&gt;"","Conselho",""),IF(K79&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N79" t="inlineStr"/>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>Vendida à Nielsen</t>
+        </is>
+      </c>
       <c r="O79" s="5" t="inlineStr">
         <is>
-          <t>2006</t>
+          <t>2007</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>Encerrada</t>
+          <t>Saída · 2024</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr"/>
       <c r="R79" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/cortacontas</t>
+          <t>https://www.crunchbase.com/organization/e-bit</t>
         </is>
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>cortacontas.png</t>
+          <t>e-bit.png</t>
         </is>
       </c>
       <c r="T79" t="inlineStr"/>
@@ -6372,7 +6384,7 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>920</t>
+          <t>900</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
@@ -6383,7 +6395,7 @@
       <c r="C80" s="5" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
-          <t>QueBarato!</t>
+          <t>Bondfaro</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -6408,24 +6420,20 @@
           <t>2006</t>
         </is>
       </c>
-      <c r="P80" t="inlineStr">
-        <is>
-          <t>Encerrada</t>
-        </is>
-      </c>
+      <c r="P80" t="inlineStr"/>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>https://www.quebarato.com.br/</t>
+          <t>https://www.bondfaro.com.br/</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/quebarato</t>
+          <t>https://www.crunchbase.com/organization/bondfaro</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>quebarato.png</t>
+          <t>bondfaro-2026.png</t>
         </is>
       </c>
       <c r="T80" t="inlineStr"/>
@@ -6439,7 +6447,7 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>910</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
@@ -6450,43 +6458,47 @@
       <c r="C81" s="5" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
-          <t>All in</t>
+          <t>CortaContas</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" s="5" t="inlineStr"/>
-      <c r="G81" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G81" s="5" t="inlineStr"/>
       <c r="H81" s="5" t="inlineStr"/>
       <c r="I81" s="5" t="inlineStr"/>
       <c r="J81" s="5" t="inlineStr"/>
-      <c r="K81" s="5" t="inlineStr"/>
+      <c r="K81" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L81" t="inlineStr"/>
       <c r="M81" s="6">
         <f>IF(L81&lt;&gt;"",L81,_xlfn.TEXTJOIN(" · ",TRUE,IF(F81&lt;&gt;"","Fundador",""),IF(G81&lt;&gt;"","Anjo",""),IF(H81&lt;&gt;"","VC",""),IF(I81&lt;&gt;"","Gestão",""),IF(J81&lt;&gt;"","Conselho",""),IF(K81&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N81" t="inlineStr">
-        <is>
-          <t>Vendida à Locaweb</t>
-        </is>
-      </c>
+      <c r="N81" t="inlineStr"/>
       <c r="O81" s="5" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>2006</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr"/>
-      <c r="R81" t="inlineStr"/>
-      <c r="S81" t="inlineStr"/>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/cortacontas</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>cortacontas.png</t>
+        </is>
+      </c>
       <c r="T81" t="inlineStr"/>
       <c r="U81" t="inlineStr"/>
       <c r="V81" t="inlineStr"/>
@@ -6498,7 +6510,7 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>960</t>
+          <t>920</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
@@ -6509,49 +6521,49 @@
       <c r="C82" s="5" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Mídia Digital / Mirum</t>
+          <t>QueBarato!</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" s="5" t="inlineStr"/>
-      <c r="G82" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G82" s="5" t="inlineStr"/>
       <c r="H82" s="5" t="inlineStr"/>
       <c r="I82" s="5" t="inlineStr"/>
       <c r="J82" s="5" t="inlineStr"/>
-      <c r="K82" s="5" t="inlineStr"/>
+      <c r="K82" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L82" t="inlineStr"/>
       <c r="M82" s="6">
         <f>IF(L82&lt;&gt;"",L82,_xlfn.TEXTJOIN(" · ",TRUE,IF(F82&lt;&gt;"","Fundador",""),IF(G82&lt;&gt;"","Anjo",""),IF(H82&lt;&gt;"","VC",""),IF(I82&lt;&gt;"","Gestão",""),IF(J82&lt;&gt;"","Conselho",""),IF(K82&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N82" t="inlineStr">
-        <is>
-          <t>Vendida à JWT</t>
-        </is>
-      </c>
+      <c r="N82" t="inlineStr"/>
       <c r="O82" s="5" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>2006</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="Q82" t="inlineStr"/>
+          <t>Encerrada</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>https://www.quebarato.com.br/</t>
+        </is>
+      </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/mirum-agency; https://www.crunchbase.com/organization/m%C3%ADdia-digital</t>
+          <t>https://www.crunchbase.com/organization/quebarato</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>mirum.png</t>
+          <t>quebarato.png</t>
         </is>
       </c>
       <c r="T82" t="inlineStr"/>
@@ -6565,7 +6577,7 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>980</t>
+          <t>930</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
@@ -6576,30 +6588,30 @@
       <c r="C83" s="5" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
-          <t>i-Equities</t>
+          <t>All in</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" s="5" t="inlineStr"/>
-      <c r="G83" s="5" t="inlineStr"/>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H83" s="5" t="inlineStr"/>
-      <c r="I83" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I83" s="5" t="inlineStr"/>
       <c r="J83" s="5" t="inlineStr"/>
       <c r="K83" s="5" t="inlineStr"/>
-      <c r="L83" t="inlineStr">
-        <is>
-          <t>Holding</t>
-        </is>
-      </c>
+      <c r="L83" t="inlineStr"/>
       <c r="M83" s="6">
         <f>IF(L83&lt;&gt;"",L83,_xlfn.TEXTJOIN(" · ",TRUE,IF(F83&lt;&gt;"","Fundador",""),IF(G83&lt;&gt;"","Anjo",""),IF(H83&lt;&gt;"","VC",""),IF(I83&lt;&gt;"","Gestão",""),IF(J83&lt;&gt;"","Conselho",""),IF(K83&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N83" t="inlineStr"/>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>Vendida à Locaweb</t>
+        </is>
+      </c>
       <c r="O83" s="5" t="inlineStr">
         <is>
           <t>2004</t>
@@ -6607,7 +6619,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>Encerrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr"/>
@@ -6624,7 +6636,7 @@
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>960</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
@@ -6635,7 +6647,7 @@
       <c r="C84" s="5" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
-          <t>AWL Leads</t>
+          <t>Mídia Digital / Mirum</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -6656,28 +6668,28 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>Vendida à Genstar Capital</t>
-        </is>
-      </c>
-      <c r="O84" s="5" t="inlineStr"/>
+          <t>Vendida à JWT</t>
+        </is>
+      </c>
+      <c r="O84" s="5" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
       <c r="P84" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q84" t="inlineStr">
-        <is>
-          <t>https://awl.com/</t>
-        </is>
-      </c>
+      <c r="Q84" t="inlineStr"/>
       <c r="R84" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/awl-fee7</t>
+          <t>https://www.crunchbase.com/organization/mirum-agency; https://www.crunchbase.com/organization/m%C3%ADdia-digital</t>
         </is>
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>awl-leads.png</t>
+          <t>mirum.png</t>
         </is>
       </c>
       <c r="T84" t="inlineStr"/>
@@ -6691,7 +6703,7 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>1005</t>
+          <t>980</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -6699,32 +6711,28 @@
           <t>x</t>
         </is>
       </c>
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="C85" s="5" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Biosphera (B&amp;Partners)</t>
+          <t>i-Equities</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" s="5" t="inlineStr"/>
-      <c r="G85" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G85" s="5" t="inlineStr"/>
       <c r="H85" s="5" t="inlineStr"/>
-      <c r="I85" s="5" t="inlineStr"/>
-      <c r="J85" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J85" s="5" t="inlineStr"/>
       <c r="K85" s="5" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Holding</t>
+        </is>
+      </c>
       <c r="M85" s="6">
         <f>IF(L85&lt;&gt;"",L85,_xlfn.TEXTJOIN(" · ",TRUE,IF(F85&lt;&gt;"","Fundador",""),IF(G85&lt;&gt;"","Anjo",""),IF(H85&lt;&gt;"","VC",""),IF(I85&lt;&gt;"","Gestão",""),IF(J85&lt;&gt;"","Conselho",""),IF(K85&lt;&gt;"","Buscapé","")))</f>
         <v/>
@@ -6732,45 +6740,29 @@
       <c r="N85" t="inlineStr"/>
       <c r="O85" s="5" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2004</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>Ativa</t>
-        </is>
-      </c>
-      <c r="Q85" t="inlineStr">
-        <is>
-          <t>https://biosphera.network/en/</t>
-        </is>
-      </c>
-      <c r="R85" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/b-partners-6cab</t>
-        </is>
-      </c>
-      <c r="S85" t="inlineStr">
-        <is>
-          <t>biosphera.png</t>
-        </is>
-      </c>
+          <t>Encerrada</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr"/>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr"/>
       <c r="T85" t="inlineStr"/>
       <c r="U85" t="inlineStr"/>
       <c r="V85" t="inlineStr"/>
       <c r="W85" t="inlineStr"/>
       <c r="X85" t="inlineStr"/>
       <c r="Y85" t="inlineStr"/>
-      <c r="Z85" t="inlineStr">
-        <is>
-          <t>Anjo. Crunchbase ainda aponta o site antigo (bpartners.com.br).</t>
-        </is>
-      </c>
+      <c r="Z85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>1010</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
@@ -6781,7 +6773,7 @@
       <c r="C86" s="5" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
-          <t>BovControl</t>
+          <t>AWL Leads</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -6800,26 +6792,30 @@
         <f>IF(L86&lt;&gt;"",L86,_xlfn.TEXTJOIN(" · ",TRUE,IF(F86&lt;&gt;"","Fundador",""),IF(G86&lt;&gt;"","Anjo",""),IF(H86&lt;&gt;"","VC",""),IF(I86&lt;&gt;"","Gestão",""),IF(J86&lt;&gt;"","Conselho",""),IF(K86&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N86" t="inlineStr"/>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>Vendida à Genstar Capital</t>
+        </is>
+      </c>
       <c r="O86" s="5" t="inlineStr"/>
       <c r="P86" t="inlineStr">
         <is>
-          <t>Ativa</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>https://bovplatform.com/about</t>
+          <t>https://awl.com/</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/bovcontrol</t>
+          <t>https://www.crunchbase.com/organization/awl-fee7</t>
         </is>
       </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t>bovcontrol.png</t>
+          <t>awl-leads.png</t>
         </is>
       </c>
       <c r="T86" t="inlineStr"/>
@@ -6833,7 +6829,7 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>1020</t>
+          <t>1005</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -6841,17 +6837,17 @@
           <t>x</t>
         </is>
       </c>
-      <c r="C87" s="5" t="inlineStr"/>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Canal da Peça</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>CWS (Canal da Peça)</t>
-        </is>
-      </c>
+          <t>Biosphera (B&amp;Partners)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
       <c r="F87" s="5" t="inlineStr"/>
       <c r="G87" s="5" t="inlineStr">
         <is>
@@ -6860,7 +6856,11 @@
       </c>
       <c r="H87" s="5" t="inlineStr"/>
       <c r="I87" s="5" t="inlineStr"/>
-      <c r="J87" s="5" t="inlineStr"/>
+      <c r="J87" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K87" s="5" t="inlineStr"/>
       <c r="L87" t="inlineStr"/>
       <c r="M87" s="6">
@@ -6868,7 +6868,11 @@
         <v/>
       </c>
       <c r="N87" t="inlineStr"/>
-      <c r="O87" s="5" t="inlineStr"/>
+      <c r="O87" s="5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="P87" t="inlineStr">
         <is>
           <t>Ativa</t>
@@ -6876,17 +6880,17 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>https://www.canaldapeca.com.br/</t>
+          <t>https://biosphera.network/en/</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/canal-da-pe%C3%A7a</t>
+          <t>https://www.crunchbase.com/organization/b-partners-6cab</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>canal-da-peca.png</t>
+          <t>biosphera.png</t>
         </is>
       </c>
       <c r="T87" t="inlineStr"/>
@@ -6895,12 +6899,16 @@
       <c r="W87" t="inlineStr"/>
       <c r="X87" t="inlineStr"/>
       <c r="Y87" t="inlineStr"/>
-      <c r="Z87" t="inlineStr"/>
+      <c r="Z87" t="inlineStr">
+        <is>
+          <t>Anjo. Crunchbase ainda aponta o site antigo (bpartners.com.br).</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>1030</t>
+          <t>1010</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
@@ -6911,7 +6919,7 @@
       <c r="C88" s="5" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Clicksign</t>
+          <t>BovControl</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -6931,11 +6939,7 @@
         <v/>
       </c>
       <c r="N88" t="inlineStr"/>
-      <c r="O88" s="5" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
-      </c>
+      <c r="O88" s="5" t="inlineStr"/>
       <c r="P88" t="inlineStr">
         <is>
           <t>Ativa</t>
@@ -6943,17 +6947,17 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>https://www.clicksign.com</t>
+          <t>https://bovplatform.com/about</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/clicksign</t>
+          <t>https://www.crunchbase.com/organization/bovcontrol</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>clicksign.png</t>
+          <t>bovcontrol.png</t>
         </is>
       </c>
       <c r="T88" t="inlineStr"/>
@@ -6967,7 +6971,7 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>1040</t>
+          <t>1020</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
@@ -6978,10 +6982,14 @@
       <c r="C89" s="5" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
-          <t>DirectTalk</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr"/>
+          <t>Canal da Peça</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>CWS (Canal da Peça)</t>
+        </is>
+      </c>
       <c r="F89" s="5" t="inlineStr"/>
       <c r="G89" s="5" t="inlineStr">
         <is>
@@ -7004,15 +7012,19 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q89" t="inlineStr"/>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>https://www.canaldapeca.com.br/</t>
+        </is>
+      </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/hi-platform</t>
+          <t>https://www.crunchbase.com/organization/canal-da-pe%C3%A7a</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>directtalk.png</t>
+          <t>canal-da-peca.png</t>
         </is>
       </c>
       <c r="T89" t="inlineStr"/>
@@ -7026,7 +7038,7 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>1050</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
@@ -7037,7 +7049,7 @@
       <c r="C90" s="5" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Galena</t>
+          <t>Clicksign</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -7057,7 +7069,11 @@
         <v/>
       </c>
       <c r="N90" t="inlineStr"/>
-      <c r="O90" s="5" t="inlineStr"/>
+      <c r="O90" s="5" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
       <c r="P90" t="inlineStr">
         <is>
           <t>Ativa</t>
@@ -7065,17 +7081,17 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>https://www.galena.com</t>
+          <t>https://www.clicksign.com</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/galena-c08c</t>
+          <t>https://www.crunchbase.com/organization/clicksign</t>
         </is>
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>galena.png</t>
+          <t>clicksign.png</t>
         </is>
       </c>
       <c r="T90" t="inlineStr"/>
@@ -7089,7 +7105,7 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>1060</t>
+          <t>1040</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -7100,7 +7116,7 @@
       <c r="C91" s="5" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Grubster / ChefsClub</t>
+          <t>DirectTalk</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -7123,18 +7139,18 @@
       <c r="O91" s="5" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
-          <t>Encerrada</t>
+          <t>Ativa</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr"/>
       <c r="R91" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/grubster</t>
+          <t>https://www.crunchbase.com/organization/hi-platform</t>
         </is>
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>chefsclub-grubster.png</t>
+          <t>directtalk.png</t>
         </is>
       </c>
       <c r="T91" t="inlineStr"/>
@@ -7148,7 +7164,7 @@
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>1070</t>
+          <t>1050</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
@@ -7159,7 +7175,7 @@
       <c r="C92" s="5" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Humortadela</t>
+          <t>Galena</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -7182,14 +7198,22 @@
       <c r="O92" s="5" t="inlineStr"/>
       <c r="P92" t="inlineStr">
         <is>
-          <t>Encerrada</t>
-        </is>
-      </c>
-      <c r="Q92" t="inlineStr"/>
-      <c r="R92" t="inlineStr"/>
+          <t>Ativa</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>https://www.galena.com</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/galena-c08c</t>
+        </is>
+      </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t>humortadela.png</t>
+          <t>galena.png</t>
         </is>
       </c>
       <c r="T92" t="inlineStr"/>
@@ -7203,7 +7227,7 @@
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>1080</t>
+          <t>1060</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -7214,7 +7238,7 @@
       <c r="C93" s="5" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Ingresse</t>
+          <t>Grubster / ChefsClub</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -7237,22 +7261,18 @@
       <c r="O93" s="5" t="inlineStr"/>
       <c r="P93" t="inlineStr">
         <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="Q93" t="inlineStr">
-        <is>
-          <t>https://ingresse.com/</t>
-        </is>
-      </c>
+          <t>Encerrada</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr"/>
       <c r="R93" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/ingresse</t>
+          <t>https://www.crunchbase.com/organization/grubster</t>
         </is>
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>ingresse.png</t>
+          <t>chefsclub-grubster.png</t>
         </is>
       </c>
       <c r="T93" t="inlineStr"/>
@@ -7266,7 +7286,7 @@
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>1090</t>
+          <t>1070</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
@@ -7277,7 +7297,7 @@
       <c r="C94" s="5" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Lema21</t>
+          <t>Humortadela</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -7296,26 +7316,18 @@
         <f>IF(L94&lt;&gt;"",L94,_xlfn.TEXTJOIN(" · ",TRUE,IF(F94&lt;&gt;"","Fundador",""),IF(G94&lt;&gt;"","Anjo",""),IF(H94&lt;&gt;"","VC",""),IF(I94&lt;&gt;"","Gestão",""),IF(J94&lt;&gt;"","Conselho",""),IF(K94&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N94" t="inlineStr">
-        <is>
-          <t>Vendida à Essilor</t>
-        </is>
-      </c>
+      <c r="N94" t="inlineStr"/>
       <c r="O94" s="5" t="inlineStr"/>
       <c r="P94" t="inlineStr">
         <is>
-          <t>Adquirida</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr"/>
-      <c r="R94" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/lema21</t>
-        </is>
-      </c>
+      <c r="R94" t="inlineStr"/>
       <c r="S94" t="inlineStr">
         <is>
-          <t>lema21.png</t>
+          <t>humortadela.png</t>
         </is>
       </c>
       <c r="T94" t="inlineStr"/>
@@ -7329,7 +7341,7 @@
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>1080</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -7340,7 +7352,7 @@
       <c r="C95" s="5" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Prontmed</t>
+          <t>Ingresse</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -7363,22 +7375,22 @@
       <c r="O95" s="5" t="inlineStr"/>
       <c r="P95" t="inlineStr">
         <is>
-          <t>Encerrada</t>
+          <t>Saída</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>https://www.prontmed.com</t>
+          <t>https://ingresse.com/</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/prontmed</t>
+          <t>https://www.crunchbase.com/organization/ingresse</t>
         </is>
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>prontmed.png</t>
+          <t>ingresse.png</t>
         </is>
       </c>
       <c r="T95" t="inlineStr"/>
@@ -7392,7 +7404,7 @@
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>1110</t>
+          <t>1090</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
@@ -7403,7 +7415,7 @@
       <c r="C96" s="5" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Qipu / MEI Grátis</t>
+          <t>Lema21</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -7422,26 +7434,26 @@
         <f>IF(L96&lt;&gt;"",L96,_xlfn.TEXTJOIN(" · ",TRUE,IF(F96&lt;&gt;"","Fundador",""),IF(G96&lt;&gt;"","Anjo",""),IF(H96&lt;&gt;"","VC",""),IF(I96&lt;&gt;"","Gestão",""),IF(J96&lt;&gt;"","Conselho",""),IF(K96&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N96" t="inlineStr"/>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>Vendida à Essilor</t>
+        </is>
+      </c>
       <c r="O96" s="5" t="inlineStr"/>
       <c r="P96" t="inlineStr">
         <is>
-          <t>Ativa</t>
-        </is>
-      </c>
-      <c r="Q96" t="inlineStr">
-        <is>
-          <t>https://qipu.com.br/</t>
-        </is>
-      </c>
+          <t>Adquirida</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr"/>
       <c r="R96" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/qipu</t>
+          <t>https://www.crunchbase.com/organization/lema21</t>
         </is>
       </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t>qipu-mei-gratis.png</t>
+          <t>lema21.png</t>
         </is>
       </c>
       <c r="T96" t="inlineStr"/>
@@ -7455,7 +7467,7 @@
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>1120</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -7466,7 +7478,7 @@
       <c r="C97" s="5" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Quero Educação</t>
+          <t>Prontmed</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -7489,18 +7501,22 @@
       <c r="O97" s="5" t="inlineStr"/>
       <c r="P97" t="inlineStr">
         <is>
-          <t>Ativa</t>
-        </is>
-      </c>
-      <c r="Q97" t="inlineStr"/>
+          <t>Encerrada</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>https://www.prontmed.com</t>
+        </is>
+      </c>
       <c r="R97" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/quero-education</t>
+          <t>https://www.crunchbase.com/organization/prontmed</t>
         </is>
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>quero-educacao.png</t>
+          <t>prontmed.png</t>
         </is>
       </c>
       <c r="T97" t="inlineStr"/>
@@ -7514,7 +7530,7 @@
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>1130</t>
+          <t>1110</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
@@ -7525,7 +7541,7 @@
       <c r="C98" s="5" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
-          <t>SP Ventures</t>
+          <t>Qipu / MEI Grátis</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -7544,30 +7560,26 @@
         <f>IF(L98&lt;&gt;"",L98,_xlfn.TEXTJOIN(" · ",TRUE,IF(F98&lt;&gt;"","Fundador",""),IF(G98&lt;&gt;"","Anjo",""),IF(H98&lt;&gt;"","VC",""),IF(I98&lt;&gt;"","Gestão",""),IF(J98&lt;&gt;"","Conselho",""),IF(K98&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N98" t="inlineStr">
-        <is>
-          <t>Vendida aos gestores</t>
-        </is>
-      </c>
+      <c r="N98" t="inlineStr"/>
       <c r="O98" s="5" t="inlineStr"/>
       <c r="P98" t="inlineStr">
         <is>
-          <t>Saída</t>
+          <t>Ativa</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>https://spventures.com.br/</t>
+          <t>https://qipu.com.br/</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/sp-ventures</t>
+          <t>https://www.crunchbase.com/organization/qipu</t>
         </is>
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>sp-ventures-2026.png</t>
+          <t>qipu-mei-gratis.png</t>
         </is>
       </c>
       <c r="T98" t="inlineStr"/>
@@ -7581,7 +7593,7 @@
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>1140</t>
+          <t>1120</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -7592,7 +7604,7 @@
       <c r="C99" s="5" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
-          <t>SetYou</t>
+          <t>Quero Educação</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -7618,19 +7630,15 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q99" t="inlineStr">
-        <is>
-          <t>https://setyou.com.br/</t>
-        </is>
-      </c>
+      <c r="Q99" t="inlineStr"/>
       <c r="R99" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/set-you</t>
+          <t>https://www.crunchbase.com/organization/quero-education</t>
         </is>
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t>setyou.png</t>
+          <t>quero-educacao.png</t>
         </is>
       </c>
       <c r="T99" t="inlineStr"/>
@@ -7644,7 +7652,7 @@
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>1150</t>
+          <t>1130</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
@@ -7655,17 +7663,17 @@
       <c r="C100" s="5" t="inlineStr"/>
       <c r="D100" t="inlineStr">
         <is>
-          <t>ViajaNet</t>
+          <t>SP Ventures</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" s="5" t="inlineStr"/>
-      <c r="G100" s="5" t="inlineStr"/>
-      <c r="H100" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H100" s="5" t="inlineStr"/>
       <c r="I100" s="5" t="inlineStr"/>
       <c r="J100" s="5" t="inlineStr"/>
       <c r="K100" s="5" t="inlineStr"/>
@@ -7676,7 +7684,7 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>Vendida à Decolar</t>
+          <t>Vendida aos gestores</t>
         </is>
       </c>
       <c r="O100" s="5" t="inlineStr"/>
@@ -7685,15 +7693,19 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q100" t="inlineStr"/>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>https://spventures.com.br/</t>
+        </is>
+      </c>
       <c r="R100" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/viajanet</t>
+          <t>https://www.crunchbase.com/organization/sp-ventures</t>
         </is>
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>viajanet.png</t>
+          <t>sp-ventures-2026.png</t>
         </is>
       </c>
       <c r="T100" t="inlineStr"/>
@@ -7707,7 +7719,7 @@
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>1140</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -7718,45 +7730,45 @@
       <c r="C101" s="5" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Ceneo</t>
+          <t>SetYou</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" s="5" t="inlineStr"/>
-      <c r="G101" s="5" t="inlineStr"/>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H101" s="5" t="inlineStr"/>
       <c r="I101" s="5" t="inlineStr"/>
       <c r="J101" s="5" t="inlineStr"/>
-      <c r="K101" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K101" s="5" t="inlineStr"/>
       <c r="L101" t="inlineStr"/>
       <c r="M101" s="6">
         <f>IF(L101&lt;&gt;"",L101,_xlfn.TEXTJOIN(" · ",TRUE,IF(F101&lt;&gt;"","Fundador",""),IF(G101&lt;&gt;"","Anjo",""),IF(H101&lt;&gt;"","VC",""),IF(I101&lt;&gt;"","Gestão",""),IF(J101&lt;&gt;"","Conselho",""),IF(K101&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
       <c r="N101" t="inlineStr"/>
-      <c r="O101" s="5" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="P101" t="inlineStr"/>
+      <c r="O101" s="5" t="inlineStr"/>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>https://www.ceneo.pl/</t>
+          <t>https://setyou.com.br/</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/ceneo</t>
+          <t>https://www.crunchbase.com/organization/set-you</t>
         </is>
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>ceneo.png</t>
+          <t>setyou.png</t>
         </is>
       </c>
       <c r="T101" t="inlineStr"/>
@@ -7770,7 +7782,7 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>1901</t>
+          <t>1150</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
@@ -7781,37 +7793,45 @@
       <c r="C102" s="5" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Compari</t>
+          <t>ViajaNet</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" s="5" t="inlineStr"/>
       <c r="G102" s="5" t="inlineStr"/>
-      <c r="H102" s="5" t="inlineStr"/>
+      <c r="H102" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I102" s="5" t="inlineStr"/>
       <c r="J102" s="5" t="inlineStr"/>
-      <c r="K102" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K102" s="5" t="inlineStr"/>
       <c r="L102" t="inlineStr"/>
       <c r="M102" s="6">
         <f>IF(L102&lt;&gt;"",L102,_xlfn.TEXTJOIN(" · ",TRUE,IF(F102&lt;&gt;"","Fundador",""),IF(G102&lt;&gt;"","Anjo",""),IF(H102&lt;&gt;"","VC",""),IF(I102&lt;&gt;"","Gestão",""),IF(J102&lt;&gt;"","Conselho",""),IF(K102&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N102" t="inlineStr"/>
-      <c r="O102" s="5" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="P102" t="inlineStr"/>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>Vendida à Decolar</t>
+        </is>
+      </c>
+      <c r="O102" s="5" t="inlineStr"/>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
       <c r="Q102" t="inlineStr"/>
-      <c r="R102" t="inlineStr"/>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/viajanet</t>
+        </is>
+      </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>compari.png</t>
+          <t>viajanet.png</t>
         </is>
       </c>
       <c r="T102" t="inlineStr"/>
@@ -7825,7 +7845,7 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
@@ -7836,7 +7856,7 @@
       <c r="C103" s="5" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Drezzi</t>
+          <t>Ceneo</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -7862,13 +7882,21 @@
         </is>
       </c>
       <c r="P103" t="inlineStr"/>
-      <c r="Q103" t="inlineStr"/>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>https://www.ceneo.pl/</t>
+        </is>
+      </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/drezzy</t>
-        </is>
-      </c>
-      <c r="S103" t="inlineStr"/>
+          <t>https://www.crunchbase.com/organization/ceneo</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>ceneo.png</t>
+        </is>
+      </c>
       <c r="T103" t="inlineStr"/>
       <c r="U103" t="inlineStr"/>
       <c r="V103" t="inlineStr"/>
@@ -7880,7 +7908,7 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
@@ -7891,7 +7919,7 @@
       <c r="C104" s="5" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Heureka</t>
+          <t>Compari</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -7918,14 +7946,10 @@
       </c>
       <c r="P104" t="inlineStr"/>
       <c r="Q104" t="inlineStr"/>
-      <c r="R104" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/heureka-group</t>
-        </is>
-      </c>
+      <c r="R104" t="inlineStr"/>
       <c r="S104" t="inlineStr">
         <is>
-          <t>heureka.png</t>
+          <t>compari.png</t>
         </is>
       </c>
       <c r="T104" t="inlineStr"/>
@@ -7939,31 +7963,31 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>1904</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="inlineStr"/>
+          <t>1902</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="C105" s="5" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Misshobby</t>
+          <t>Drezzi</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" s="5" t="inlineStr"/>
       <c r="G105" s="5" t="inlineStr"/>
       <c r="H105" s="5" t="inlineStr"/>
-      <c r="I105" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J105" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K105" s="5" t="inlineStr"/>
+      <c r="I105" s="5" t="inlineStr"/>
+      <c r="J105" s="5" t="inlineStr"/>
+      <c r="K105" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L105" t="inlineStr"/>
       <c r="M105" s="6">
         <f>IF(L105&lt;&gt;"",L105,_xlfn.TEXTJOIN(" · ",TRUE,IF(F105&lt;&gt;"","Fundador",""),IF(G105&lt;&gt;"","Anjo",""),IF(H105&lt;&gt;"","VC",""),IF(I105&lt;&gt;"","Gestão",""),IF(J105&lt;&gt;"","Conselho",""),IF(K105&lt;&gt;"","Buscapé","")))</f>
@@ -7976,17 +8000,13 @@
         </is>
       </c>
       <c r="P105" t="inlineStr"/>
-      <c r="Q105" t="inlineStr">
-        <is>
-          <t>https://www.misshobby.com/it</t>
-        </is>
-      </c>
-      <c r="R105" t="inlineStr"/>
-      <c r="S105" t="inlineStr">
-        <is>
-          <t>misshobby.png</t>
-        </is>
-      </c>
+      <c r="Q105" t="inlineStr"/>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/drezzy</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr"/>
       <c r="T105" t="inlineStr"/>
       <c r="U105" t="inlineStr"/>
       <c r="V105" t="inlineStr"/>
@@ -7998,7 +8018,7 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>1905</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
@@ -8009,7 +8029,7 @@
       <c r="C106" s="5" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Pazaruvaj</t>
+          <t>Heureka</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -8036,10 +8056,14 @@
       </c>
       <c r="P106" t="inlineStr"/>
       <c r="Q106" t="inlineStr"/>
-      <c r="R106" t="inlineStr"/>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/heureka-group</t>
+        </is>
+      </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>pazaruvaj.png</t>
+          <t>heureka.png</t>
         </is>
       </c>
       <c r="T106" t="inlineStr"/>
@@ -8053,31 +8077,31 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>1906</t>
-        </is>
-      </c>
-      <c r="B107" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1904</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr"/>
       <c r="C107" s="5" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
-          <t>PriceCheck</t>
+          <t>Misshobby</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" s="5" t="inlineStr"/>
       <c r="G107" s="5" t="inlineStr"/>
       <c r="H107" s="5" t="inlineStr"/>
-      <c r="I107" s="5" t="inlineStr"/>
-      <c r="J107" s="5" t="inlineStr"/>
-      <c r="K107" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I107" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J107" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K107" s="5" t="inlineStr"/>
       <c r="L107" t="inlineStr"/>
       <c r="M107" s="6">
         <f>IF(L107&lt;&gt;"",L107,_xlfn.TEXTJOIN(" · ",TRUE,IF(F107&lt;&gt;"","Fundador",""),IF(G107&lt;&gt;"","Anjo",""),IF(H107&lt;&gt;"","VC",""),IF(I107&lt;&gt;"","Gestão",""),IF(J107&lt;&gt;"","Conselho",""),IF(K107&lt;&gt;"","Buscapé","")))</f>
@@ -8090,15 +8114,15 @@
         </is>
       </c>
       <c r="P107" t="inlineStr"/>
-      <c r="Q107" t="inlineStr"/>
-      <c r="R107" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/pricecheck</t>
-        </is>
-      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>https://www.misshobby.com/it</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr"/>
       <c r="S107" t="inlineStr">
         <is>
-          <t>pricecheck.png</t>
+          <t>misshobby.png</t>
         </is>
       </c>
       <c r="T107" t="inlineStr"/>
@@ -8112,7 +8136,7 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1905</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
@@ -8123,7 +8147,7 @@
       <c r="C108" s="5" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
-          <t>ShoppyDoo</t>
+          <t>Pazaruvaj</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -8149,19 +8173,11 @@
         </is>
       </c>
       <c r="P108" t="inlineStr"/>
-      <c r="Q108" t="inlineStr">
-        <is>
-          <t>https://www.shoppydoo.it/</t>
-        </is>
-      </c>
-      <c r="R108" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/shoppydoo</t>
-        </is>
-      </c>
+      <c r="Q108" t="inlineStr"/>
+      <c r="R108" t="inlineStr"/>
       <c r="S108" t="inlineStr">
         <is>
-          <t>shoppydoo.png</t>
+          <t>pazaruvaj.png</t>
         </is>
       </c>
       <c r="T108" t="inlineStr"/>
@@ -8175,7 +8191,7 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
@@ -8186,7 +8202,7 @@
       <c r="C109" s="5" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Trovaprezzi</t>
+          <t>PriceCheck</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -8215,12 +8231,12 @@
       <c r="Q109" t="inlineStr"/>
       <c r="R109" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/trovaprezzi-it-d087</t>
+          <t>https://www.crunchbase.com/organization/pricecheck</t>
         </is>
       </c>
       <c r="S109" t="inlineStr">
         <is>
-          <t>trovaprezzi.png</t>
+          <t>pricecheck.png</t>
         </is>
       </c>
       <c r="T109" t="inlineStr"/>
@@ -8234,7 +8250,7 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
@@ -8245,7 +8261,7 @@
       <c r="C110" s="5" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Ucuzu</t>
+          <t>ShoppyDoo</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
@@ -8271,9 +8287,21 @@
         </is>
       </c>
       <c r="P110" t="inlineStr"/>
-      <c r="Q110" t="inlineStr"/>
-      <c r="R110" t="inlineStr"/>
-      <c r="S110" t="inlineStr"/>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>https://www.shoppydoo.it/</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/shoppydoo</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>shoppydoo.png</t>
+        </is>
+      </c>
       <c r="T110" t="inlineStr"/>
       <c r="U110" t="inlineStr"/>
       <c r="V110" t="inlineStr"/>
@@ -8285,7 +8313,7 @@
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
@@ -8296,7 +8324,7 @@
       <c r="C111" s="5" t="inlineStr"/>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Vcene</t>
+          <t>Trovaprezzi</t>
         </is>
       </c>
       <c r="E111" t="inlineStr"/>
@@ -8325,10 +8353,14 @@
       <c r="Q111" t="inlineStr"/>
       <c r="R111" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/vcene</t>
-        </is>
-      </c>
-      <c r="S111" t="inlineStr"/>
+          <t>https://www.crunchbase.com/organization/trovaprezzi-it-d087</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>trovaprezzi.png</t>
+        </is>
+      </c>
       <c r="T111" t="inlineStr"/>
       <c r="U111" t="inlineStr"/>
       <c r="V111" t="inlineStr"/>
@@ -8340,7 +8372,7 @@
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
@@ -8351,7 +8383,7 @@
       <c r="C112" s="5" t="inlineStr"/>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Árukereső</t>
+          <t>Ucuzu</t>
         </is>
       </c>
       <c r="E112" t="inlineStr"/>
@@ -8378,16 +8410,8 @@
       </c>
       <c r="P112" t="inlineStr"/>
       <c r="Q112" t="inlineStr"/>
-      <c r="R112" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/%C3%A1rukeres%C5%91</t>
-        </is>
-      </c>
-      <c r="S112" t="inlineStr">
-        <is>
-          <t>arukereso.png</t>
-        </is>
-      </c>
+      <c r="R112" t="inlineStr"/>
+      <c r="S112" t="inlineStr"/>
       <c r="T112" t="inlineStr"/>
       <c r="U112" t="inlineStr"/>
       <c r="V112" t="inlineStr"/>
@@ -8399,7 +8423,7 @@
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
@@ -8410,20 +8434,20 @@
       <c r="C113" s="5" t="inlineStr"/>
       <c r="D113" t="inlineStr">
         <is>
-          <t>FocoSoft</t>
+          <t>Vcene</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
-      <c r="F113" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="F113" s="5" t="inlineStr"/>
       <c r="G113" s="5" t="inlineStr"/>
       <c r="H113" s="5" t="inlineStr"/>
       <c r="I113" s="5" t="inlineStr"/>
       <c r="J113" s="5" t="inlineStr"/>
-      <c r="K113" s="5" t="inlineStr"/>
+      <c r="K113" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L113" t="inlineStr"/>
       <c r="M113" s="6">
         <f>IF(L113&lt;&gt;"",L113,_xlfn.TEXTJOIN(" · ",TRUE,IF(F113&lt;&gt;"","Fundador",""),IF(G113&lt;&gt;"","Anjo",""),IF(H113&lt;&gt;"","VC",""),IF(I113&lt;&gt;"","Gestão",""),IF(J113&lt;&gt;"","Conselho",""),IF(K113&lt;&gt;"","Buscapé","")))</f>
@@ -8432,12 +8456,16 @@
       <c r="N113" t="inlineStr"/>
       <c r="O113" s="5" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="P113" t="inlineStr"/>
       <c r="Q113" t="inlineStr"/>
-      <c r="R113" t="inlineStr"/>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/vcene</t>
+        </is>
+      </c>
       <c r="S113" t="inlineStr"/>
       <c r="T113" t="inlineStr"/>
       <c r="U113" t="inlineStr"/>
@@ -8450,7 +8478,7 @@
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="B114" s="5" t="inlineStr">
@@ -8461,20 +8489,20 @@
       <c r="C114" s="5" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Curupira</t>
+          <t>Árukereső</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" s="5" t="inlineStr"/>
-      <c r="G114" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G114" s="5" t="inlineStr"/>
       <c r="H114" s="5" t="inlineStr"/>
       <c r="I114" s="5" t="inlineStr"/>
       <c r="J114" s="5" t="inlineStr"/>
-      <c r="K114" s="5" t="inlineStr"/>
+      <c r="K114" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L114" t="inlineStr"/>
       <c r="M114" s="6">
         <f>IF(L114&lt;&gt;"",L114,_xlfn.TEXTJOIN(" · ",TRUE,IF(F114&lt;&gt;"","Fundador",""),IF(G114&lt;&gt;"","Anjo",""),IF(H114&lt;&gt;"","VC",""),IF(I114&lt;&gt;"","Gestão",""),IF(J114&lt;&gt;"","Conselho",""),IF(K114&lt;&gt;"","Buscapé","")))</f>
@@ -8483,23 +8511,19 @@
       <c r="N114" t="inlineStr"/>
       <c r="O114" s="5" t="inlineStr">
         <is>
-          <t>2016</t>
-        </is>
-      </c>
-      <c r="P114" t="inlineStr">
-        <is>
-          <t>Encerrada</t>
-        </is>
-      </c>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr"/>
       <c r="Q114" t="inlineStr"/>
       <c r="R114" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/curupira</t>
+          <t>https://www.crunchbase.com/organization/%C3%A1rukeres%C5%91</t>
         </is>
       </c>
       <c r="S114" t="inlineStr">
         <is>
-          <t>curupira.png</t>
+          <t>arukereso.png</t>
         </is>
       </c>
       <c r="T114" t="inlineStr"/>
@@ -8513,7 +8537,7 @@
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
@@ -8524,16 +8548,16 @@
       <c r="C115" s="5" t="inlineStr"/>
       <c r="D115" t="inlineStr">
         <is>
-          <t>CyberCook / Vila Mulher</t>
+          <t>FocoSoft</t>
         </is>
       </c>
       <c r="E115" t="inlineStr"/>
-      <c r="F115" s="5" t="inlineStr"/>
-      <c r="G115" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr"/>
       <c r="H115" s="5" t="inlineStr"/>
       <c r="I115" s="5" t="inlineStr"/>
       <c r="J115" s="5" t="inlineStr"/>
@@ -8546,21 +8570,13 @@
       <c r="N115" t="inlineStr"/>
       <c r="O115" s="5" t="inlineStr">
         <is>
-          <t>2004</t>
-        </is>
-      </c>
-      <c r="P115" t="inlineStr">
-        <is>
-          <t>Encerrada</t>
-        </is>
-      </c>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr"/>
       <c r="Q115" t="inlineStr"/>
       <c r="R115" t="inlineStr"/>
-      <c r="S115" t="inlineStr">
-        <is>
-          <t>cybercook.png</t>
-        </is>
-      </c>
+      <c r="S115" t="inlineStr"/>
       <c r="T115" t="inlineStr"/>
       <c r="U115" t="inlineStr"/>
       <c r="V115" t="inlineStr"/>
@@ -8572,7 +8588,7 @@
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>2030</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="B116" s="5" t="inlineStr">
@@ -8583,7 +8599,7 @@
       <c r="C116" s="5" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Loteria Brasil</t>
+          <t>Curupira</t>
         </is>
       </c>
       <c r="E116" t="inlineStr"/>
@@ -8605,7 +8621,7 @@
       <c r="N116" t="inlineStr"/>
       <c r="O116" s="5" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -8614,10 +8630,14 @@
         </is>
       </c>
       <c r="Q116" t="inlineStr"/>
-      <c r="R116" t="inlineStr"/>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/curupira</t>
+        </is>
+      </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>loteria-brasil.png</t>
+          <t>curupira.png</t>
         </is>
       </c>
       <c r="T116" t="inlineStr"/>
@@ -8631,7 +8651,7 @@
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>2040</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="B117" s="5" t="inlineStr">
@@ -8642,7 +8662,7 @@
       <c r="C117" s="5" t="inlineStr"/>
       <c r="D117" t="inlineStr">
         <is>
-          <t>eHub</t>
+          <t>CyberCook / Vila Mulher</t>
         </is>
       </c>
       <c r="E117" t="inlineStr"/>
@@ -8673,12 +8693,12 @@
         </is>
       </c>
       <c r="Q117" t="inlineStr"/>
-      <c r="R117" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/ehub</t>
-        </is>
-      </c>
-      <c r="S117" t="inlineStr"/>
+      <c r="R117" t="inlineStr"/>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>cybercook.png</t>
+        </is>
+      </c>
       <c r="T117" t="inlineStr"/>
       <c r="U117" t="inlineStr"/>
       <c r="V117" t="inlineStr"/>
@@ -8690,7 +8710,7 @@
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>2030</t>
         </is>
       </c>
       <c r="B118" s="5" t="inlineStr">
@@ -8701,7 +8721,7 @@
       <c r="C118" s="5" t="inlineStr"/>
       <c r="D118" t="inlineStr">
         <is>
-          <t>ContaPaga</t>
+          <t>Loteria Brasil</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -8721,19 +8741,23 @@
         <v/>
       </c>
       <c r="N118" t="inlineStr"/>
-      <c r="O118" s="5" t="inlineStr"/>
+      <c r="O118" s="5" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
       <c r="P118" t="inlineStr">
         <is>
           <t>Encerrada</t>
         </is>
       </c>
       <c r="Q118" t="inlineStr"/>
-      <c r="R118" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/contapaga</t>
-        </is>
-      </c>
-      <c r="S118" t="inlineStr"/>
+      <c r="R118" t="inlineStr"/>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t>loteria-brasil.png</t>
+        </is>
+      </c>
       <c r="T118" t="inlineStr"/>
       <c r="U118" t="inlineStr"/>
       <c r="V118" t="inlineStr"/>
@@ -8745,7 +8769,7 @@
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>2060</t>
+          <t>2040</t>
         </is>
       </c>
       <c r="B119" s="5" t="inlineStr">
@@ -8756,7 +8780,7 @@
       <c r="C119" s="5" t="inlineStr"/>
       <c r="D119" t="inlineStr">
         <is>
-          <t>HospedeVIP</t>
+          <t>eHub</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -8776,14 +8800,22 @@
         <v/>
       </c>
       <c r="N119" t="inlineStr"/>
-      <c r="O119" s="5" t="inlineStr"/>
+      <c r="O119" s="5" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
       <c r="P119" t="inlineStr">
         <is>
           <t>Encerrada</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr"/>
-      <c r="R119" t="inlineStr"/>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/ehub</t>
+        </is>
+      </c>
       <c r="S119" t="inlineStr"/>
       <c r="T119" t="inlineStr"/>
       <c r="U119" t="inlineStr"/>
@@ -8796,7 +8828,7 @@
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>2070</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="B120" s="5" t="inlineStr">
@@ -8807,7 +8839,7 @@
       <c r="C120" s="5" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Jet8</t>
+          <t>ContaPaga</t>
         </is>
       </c>
       <c r="E120" t="inlineStr"/>
@@ -8833,17 +8865,13 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q120" t="inlineStr">
-        <is>
-          <t>https://jet8.io/</t>
-        </is>
-      </c>
-      <c r="R120" t="inlineStr"/>
-      <c r="S120" t="inlineStr">
-        <is>
-          <t>jet8-2026.png</t>
-        </is>
-      </c>
+      <c r="Q120" t="inlineStr"/>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/contapaga</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr"/>
       <c r="T120" t="inlineStr"/>
       <c r="U120" t="inlineStr"/>
       <c r="V120" t="inlineStr"/>
@@ -8855,7 +8883,7 @@
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>2080</t>
+          <t>2060</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
@@ -8866,7 +8894,7 @@
       <c r="C121" s="5" t="inlineStr"/>
       <c r="D121" t="inlineStr">
         <is>
-          <t>LOFTY / ROOMORAMA</t>
+          <t>HospedeVIP</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -8892,16 +8920,8 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q121" t="inlineStr">
-        <is>
-          <t>https://roomorama.com/</t>
-        </is>
-      </c>
-      <c r="R121" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/roomorama; https://www.crunchbase.com/organization/lofty-ai</t>
-        </is>
-      </c>
+      <c r="Q121" t="inlineStr"/>
+      <c r="R121" t="inlineStr"/>
       <c r="S121" t="inlineStr"/>
       <c r="T121" t="inlineStr"/>
       <c r="U121" t="inlineStr"/>
@@ -8914,7 +8934,7 @@
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>2090</t>
+          <t>2070</t>
         </is>
       </c>
       <c r="B122" s="5" t="inlineStr">
@@ -8925,7 +8945,7 @@
       <c r="C122" s="5" t="inlineStr"/>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Lulu App</t>
+          <t>Jet8</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -8951,15 +8971,15 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q122" t="inlineStr"/>
-      <c r="R122" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/lulu-2</t>
-        </is>
-      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>https://jet8.io/</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr"/>
       <c r="S122" t="inlineStr">
         <is>
-          <t>lulu-app.png</t>
+          <t>jet8-2026.png</t>
         </is>
       </c>
       <c r="T122" t="inlineStr"/>
@@ -8973,7 +8993,7 @@
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>2080</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
@@ -8984,7 +9004,7 @@
       <c r="C123" s="5" t="inlineStr"/>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Moneto</t>
+          <t>LOFTY / ROOMORAMA</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
@@ -9010,17 +9030,17 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q123" t="inlineStr"/>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>https://roomorama.com/</t>
+        </is>
+      </c>
       <c r="R123" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/contapaga</t>
-        </is>
-      </c>
-      <c r="S123" t="inlineStr">
-        <is>
-          <t>moneto.png</t>
-        </is>
-      </c>
+          <t>https://www.crunchbase.com/organization/roomorama; https://www.crunchbase.com/organization/lofty-ai</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr"/>
       <c r="T123" t="inlineStr"/>
       <c r="U123" t="inlineStr"/>
       <c r="V123" t="inlineStr"/>
@@ -9032,7 +9052,7 @@
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>2090</t>
         </is>
       </c>
       <c r="B124" s="5" t="inlineStr">
@@ -9043,7 +9063,7 @@
       <c r="C124" s="5" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
-          <t>OrderIn</t>
+          <t>Lulu App</t>
         </is>
       </c>
       <c r="E124" t="inlineStr"/>
@@ -9072,12 +9092,12 @@
       <c r="Q124" t="inlineStr"/>
       <c r="R124" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/orderin</t>
+          <t>https://www.crunchbase.com/organization/lulu-2</t>
         </is>
       </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t>orderin-2026.png</t>
+          <t>lulu-app.png</t>
         </is>
       </c>
       <c r="T124" t="inlineStr"/>
@@ -9091,7 +9111,7 @@
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>2120</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="B125" s="5" t="inlineStr">
@@ -9102,7 +9122,7 @@
       <c r="C125" s="5" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Scup</t>
+          <t>Moneto</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -9121,26 +9141,22 @@
         <f>IF(L125&lt;&gt;"",L125,_xlfn.TEXTJOIN(" · ",TRUE,IF(F125&lt;&gt;"","Fundador",""),IF(G125&lt;&gt;"","Anjo",""),IF(H125&lt;&gt;"","VC",""),IF(I125&lt;&gt;"","Gestão",""),IF(J125&lt;&gt;"","Conselho",""),IF(K125&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N125" t="inlineStr">
-        <is>
-          <t>Vendida à Sprinkr</t>
-        </is>
-      </c>
+      <c r="N125" t="inlineStr"/>
       <c r="O125" s="5" t="inlineStr"/>
       <c r="P125" t="inlineStr">
         <is>
-          <t>Saída · 2015</t>
+          <t>Encerrada</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr"/>
       <c r="R125" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/scup</t>
+          <t>https://www.crunchbase.com/organization/contapaga</t>
         </is>
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>scup-2026.png</t>
+          <t>moneto.png</t>
         </is>
       </c>
       <c r="T125" t="inlineStr"/>
@@ -9154,7 +9170,7 @@
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="B126" s="5" t="inlineStr">
@@ -9165,7 +9181,7 @@
       <c r="C126" s="5" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Shoes4you</t>
+          <t>OrderIn</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -9191,19 +9207,15 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q126" t="inlineStr">
-        <is>
-          <t>https://shoes4you.com.br/</t>
-        </is>
-      </c>
+      <c r="Q126" t="inlineStr"/>
       <c r="R126" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/shoes4you</t>
+          <t>https://www.crunchbase.com/organization/orderin</t>
         </is>
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>shoes4you.png</t>
+          <t>orderin-2026.png</t>
         </is>
       </c>
       <c r="T126" t="inlineStr"/>
@@ -9217,7 +9229,7 @@
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>2140</t>
+          <t>2120</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
@@ -9228,7 +9240,7 @@
       <c r="C127" s="5" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Siga Seu Time</t>
+          <t>Scup</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -9247,20 +9259,28 @@
         <f>IF(L127&lt;&gt;"",L127,_xlfn.TEXTJOIN(" · ",TRUE,IF(F127&lt;&gt;"","Fundador",""),IF(G127&lt;&gt;"","Anjo",""),IF(H127&lt;&gt;"","VC",""),IF(I127&lt;&gt;"","Gestão",""),IF(J127&lt;&gt;"","Conselho",""),IF(K127&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N127" t="inlineStr"/>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>Vendida à Sprinkr</t>
+        </is>
+      </c>
       <c r="O127" s="5" t="inlineStr"/>
       <c r="P127" t="inlineStr">
         <is>
-          <t>Encerrada</t>
+          <t>Saída · 2015</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr"/>
       <c r="R127" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/sigaseutime</t>
-        </is>
-      </c>
-      <c r="S127" t="inlineStr"/>
+          <t>https://www.crunchbase.com/organization/scup</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>scup-2026.png</t>
+        </is>
+      </c>
       <c r="T127" t="inlineStr"/>
       <c r="U127" t="inlineStr"/>
       <c r="V127" t="inlineStr"/>
@@ -9272,7 +9292,7 @@
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="B128" s="5" t="inlineStr">
@@ -9283,7 +9303,7 @@
       <c r="C128" s="5" t="inlineStr"/>
       <c r="D128" t="inlineStr">
         <is>
-          <t>youHotel</t>
+          <t>Shoes4you</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -9309,15 +9329,19 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q128" t="inlineStr"/>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>https://shoes4you.com.br/</t>
+        </is>
+      </c>
       <c r="R128" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/youhotel</t>
+          <t>https://www.crunchbase.com/organization/shoes4you</t>
         </is>
       </c>
       <c r="S128" t="inlineStr">
         <is>
-          <t>youhotel.png</t>
+          <t>shoes4you.png</t>
         </is>
       </c>
       <c r="T128" t="inlineStr"/>
@@ -9328,8 +9352,122 @@
       <c r="Y128" t="inlineStr"/>
       <c r="Z128" t="inlineStr"/>
     </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>2140</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr"/>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Siga Seu Time</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" s="5" t="inlineStr"/>
+      <c r="G129" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H129" s="5" t="inlineStr"/>
+      <c r="I129" s="5" t="inlineStr"/>
+      <c r="J129" s="5" t="inlineStr"/>
+      <c r="K129" s="5" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
+      <c r="M129" s="6">
+        <f>IF(L129&lt;&gt;"",L129,_xlfn.TEXTJOIN(" · ",TRUE,IF(F129&lt;&gt;"","Fundador",""),IF(G129&lt;&gt;"","Anjo",""),IF(H129&lt;&gt;"","VC",""),IF(I129&lt;&gt;"","Gestão",""),IF(J129&lt;&gt;"","Conselho",""),IF(K129&lt;&gt;"","Buscapé","")))</f>
+        <v/>
+      </c>
+      <c r="N129" t="inlineStr"/>
+      <c r="O129" s="5" t="inlineStr"/>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr"/>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/sigaseutime</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr"/>
+      <c r="T129" t="inlineStr"/>
+      <c r="U129" t="inlineStr"/>
+      <c r="V129" t="inlineStr"/>
+      <c r="W129" t="inlineStr"/>
+      <c r="X129" t="inlineStr"/>
+      <c r="Y129" t="inlineStr"/>
+      <c r="Z129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="inlineStr">
+        <is>
+          <t>2150</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr"/>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>youHotel</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" s="5" t="inlineStr"/>
+      <c r="G130" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H130" s="5" t="inlineStr"/>
+      <c r="I130" s="5" t="inlineStr"/>
+      <c r="J130" s="5" t="inlineStr"/>
+      <c r="K130" s="5" t="inlineStr"/>
+      <c r="L130" t="inlineStr"/>
+      <c r="M130" s="6">
+        <f>IF(L130&lt;&gt;"",L130,_xlfn.TEXTJOIN(" · ",TRUE,IF(F130&lt;&gt;"","Fundador",""),IF(G130&lt;&gt;"","Anjo",""),IF(H130&lt;&gt;"","VC",""),IF(I130&lt;&gt;"","Gestão",""),IF(J130&lt;&gt;"","Conselho",""),IF(K130&lt;&gt;"","Buscapé","")))</f>
+        <v/>
+      </c>
+      <c r="N130" t="inlineStr"/>
+      <c r="O130" s="5" t="inlineStr"/>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr"/>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/youhotel</t>
+        </is>
+      </c>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>youhotel.png</t>
+        </is>
+      </c>
+      <c r="T130" t="inlineStr"/>
+      <c r="U130" t="inlineStr"/>
+      <c r="V130" t="inlineStr"/>
+      <c r="W130" t="inlineStr"/>
+      <c r="X130" t="inlineStr"/>
+      <c r="Y130" t="inlineStr"/>
+      <c r="Z130" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z128"/>
+  <autoFilter ref="A1:Z130"/>
   <dataValidations count="2">
     <dataValidation sqref="B2:B2000 F2:F2000 G2:G2000 H2:H2000 I2:I2000 J2:J2000 K2:K2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use x para marcar ou deixe vazio." type="list">
       <formula1>"x"</formula1>

</xml_diff>

<commit_message>
feat(portfolio): logos da Arena e da Cortex
Arena veio em SVG branco (para fundo escuro): renderizado em escuro sobre
transparente. Cortex já vinha com fundo transparente.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -4417,7 +4417,11 @@
           <t>https://www.crunchbase.com/organization/arena-im</t>
         </is>
       </c>
-      <c r="S50" t="inlineStr"/>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>arena.png</t>
+        </is>
+      </c>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr"/>
@@ -5048,7 +5052,11 @@
           <t>https://www.crunchbase.com/organization/cortex-intelligence</t>
         </is>
       </c>
-      <c r="S59" t="inlineStr"/>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>cortex.png</t>
+        </is>
+      </c>
       <c r="T59" t="inlineStr"/>
       <c r="U59" t="inlineStr"/>
       <c r="V59" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(portfolio): filtros Saídas e Acima de US$ 1 bi, ordenação; Poli-USP na Trajetória
- Planilha ganha as colunas Saída e US$ 1 bi+ (x), pré-preenchidas: 26
  saídas (status e notas de venda, fusão ou saída) e as 9 empresas acima
  de US$ 1 bi que o site já cita.
- Página: botões Saídas e Acima de US$ 1 bi, que combinam com as abas de
  relação e a busca (clicar de novo desliga), e ordenação por destaque,
  nome ou ano (segundo clique inverte). Sem ano vai para o fim.
- Versão em inglês: Exits, Over $1b, Featured, Name, Year.
- Trajetória: logo da Poli-USP no marco de 2002 (formatura).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Empresas'!$A$1:$Z$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Empresas'!$A$1:$AB$130</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -257,50 +257,60 @@
     </comment>
     <comment ref="Q1" authorId="0" shapeId="0">
       <text>
-        <t>URL do site. Vazio = card sem link.</t>
+        <t>x = teve exit (venda, fusão, saída da participação). Alimenta o filtro Saídas do portfólio.</t>
       </text>
     </comment>
     <comment ref="R1" authorId="0" shapeId="0">
       <text>
-        <t>Opcional. Perfis da empresa em outros sites (Crunchbase, Wikidata, LinkedIn), separados por ';'. Não aparecem no card: vão para os dados estruturados (sameAs), que ligam a empresa à mesma empresa nesses sites.</t>
+        <t>x = passou de US$ 1 bilhão de valor. Alimenta o filtro Acima de US$ 1 bi do portfólio.</t>
       </text>
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
       <text>
-        <t>Arquivo em assets/img/logos/. Vazio = mostra o nome em texto.</t>
+        <t>URL do site. Vazio = card sem link.</t>
       </text>
     </comment>
     <comment ref="T1" authorId="0" shapeId="0">
       <text>
-        <t>Opcional. Segundo logo empilhado (ex.: Movile + iFood).</t>
+        <t>Opcional. Perfis da empresa em outros sites (Crunchbase, Wikidata, LinkedIn), separados por ';'. Não aparecem no card: vão para os dados estruturados (sameAs), que ligam a empresa à mesma empresa nesses sites.</t>
       </text>
     </comment>
     <comment ref="U1" authorId="0" shapeId="0">
       <text>
-        <t>Opcional. Texto mostrado antes do logo (ex.: Bcash). Sem logo, o nome já aparece em texto.</t>
+        <t>Arquivo em assets/img/logos/. Vazio = mostra o nome em texto.</t>
       </text>
     </comment>
     <comment ref="V1" authorId="0" shapeId="0">
       <text>
-        <t>Opcional. Textos alternativos separados por ';', na ordem dos logos. Vazio = Nome.</t>
+        <t>Opcional. Segundo logo empilhado (ex.: Movile + iFood).</t>
       </text>
     </comment>
     <comment ref="W1" authorId="0" shapeId="0">
       <text>
-        <t>Link de uma matéria sobre a empresa.</t>
+        <t>Opcional. Texto mostrado antes do logo (ex.: Bcash). Sem logo, o nome já aparece em texto.</t>
       </text>
     </comment>
     <comment ref="X1" authorId="0" shapeId="0">
       <text>
-        <t>Título exibido no card.</t>
+        <t>Opcional. Textos alternativos separados por ';', na ordem dos logos. Vazio = Nome.</t>
       </text>
     </comment>
     <comment ref="Y1" authorId="0" shapeId="0">
       <text>
+        <t>Link de uma matéria sobre a empresa.</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <t>Título exibido no card.</t>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
         <t>Ex.: 'Brazil Journal · jul 2021'.</t>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
+    <comment ref="AB1" authorId="0" shapeId="0">
       <text>
         <t>Não vai para o site.</t>
       </text>
@@ -598,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -690,36 +700,43 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Perfis: links da empresa no Crunchbase, Wikidata ou LinkedIn, separados por ';'. Não aparecem no card;</t>
+          <t>Saída e US$ 1 bi+: marque x. Alimentam os filtros Saídas e Acima de US$ 1 bi da página (combinam com as abas).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  entram nos dados estruturados da página, para o Google e as IAs ligarem a empresa ao seu portfólio.</t>
+          <t>Perfis: links da empresa no Crunchbase, Wikidata ou LinkedIn, separados por ';'. Não aparecem no card;</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t xml:space="preserve">  entram nos dados estruturados da página, para o Google e as IAs ligarem a empresa ao seu portfólio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Observações internas não vão para o site.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Passe o mouse no cabeçalho de cada coluna para ver a explicação.</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
+        <is>
+          <t>Passe o mouse no cabeçalho de cada coluna para ver a explicação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Não renomeie os cabeçalhos da aba Empresas: o script procura as colunas pelo nome.</t>
         </is>
@@ -736,7 +753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z130"/>
+  <dimension ref="A1:AB130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -755,16 +772,18 @@
     <col width="26" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
-    <col width="40" customWidth="1" min="18" max="18"/>
-    <col width="17" customWidth="1" min="19" max="19"/>
-    <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="22" customWidth="1" min="22" max="22"/>
-    <col width="34" customWidth="1" min="23" max="23"/>
-    <col width="28" customWidth="1" min="24" max="24"/>
-    <col width="22" customWidth="1" min="25" max="25"/>
-    <col width="36" customWidth="1" min="26" max="26"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="34" customWidth="1" min="25" max="25"/>
+    <col width="28" customWidth="1" min="26" max="26"/>
+    <col width="22" customWidth="1" min="27" max="27"/>
+    <col width="36" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -848,52 +867,62 @@
           <t>Status</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>US$ 1 bi+</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Site</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>Perfis</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>Logo</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>Logo 2</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>Logo em texto</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
         <is>
           <t>Alt dos logos</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>Matéria (link)</t>
         </is>
       </c>
-      <c r="X1" s="3" t="inlineStr">
+      <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>Matéria (título)</t>
         </is>
       </c>
-      <c r="Y1" s="3" t="inlineStr">
+      <c r="AA1" s="3" t="inlineStr">
         <is>
           <t>Matéria (fonte · data)</t>
         </is>
       </c>
-      <c r="Z1" s="3" t="inlineStr">
+      <c r="AB1" s="3" t="inlineStr">
         <is>
           <t>Observações internas</t>
         </is>
@@ -959,28 +988,34 @@
           <t>US$ 374M · 2009</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
         <is>
           <t>https://www.buscape.com.br</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/buscap-company</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>buscape-2026.png</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -1038,40 +1073,50 @@
           <t>US$ 1 bi · 2024</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>https://www.pismo.io/</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/pismo</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>pismo.png</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr">
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr">
         <is>
           <t>https://fortune.com/2023/07/25/headline-brazil-pismo-visa/</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>How VC Headline notched a 30% stake in Brazil’s biggest startup acquisition in 5 years</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>Fortune · jul 2023</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1125,40 +1170,46 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q4" s="5" t="inlineStr"/>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
         <is>
           <t>https://wellhub.com/pt-br/</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/gympass</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>wellhub.png</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr">
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=4v8VvLNtaxU</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>#Takeover | Romero Rodrigues &amp; Gympass: a startup brasileira que conquistou o mundo</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>Cubo Itaú · set 2020</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1212,40 +1263,46 @@
           <t>Listada na NYSE</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr"/>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
         <is>
           <t>https://www.wayfair.com</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/wayfair</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>wayfair.png</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr">
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/wayfair-names-romero-rodrigues-to-its-board-of-directors-269021721.html</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>Wayfair Names Romero Rodrigues to its Board of Directors</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>PR Newswire · jul 2014</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1299,40 +1356,46 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q6" s="5" t="inlineStr"/>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
         <is>
           <t>https://olist.com</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/olist</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>olist.png</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr">
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr">
         <is>
           <t>https://www.gazetadopovo.com.br/economia/empreender-pme/fundo-do-fundador-do-buscape-compra-participacao-em-startup-curitibana-9wkf3luxsvvljmo3q7ujely4v/</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>Fundo do fundador do Buscapé compra participação em startup curitibana</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="AA6" t="inlineStr">
         <is>
           <t>Gazeta do Povo · ago 2016</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1382,40 +1445,50 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
         <is>
           <t>https://hotmart.com/en</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/hotmart</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>hotmart.png</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr">
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr">
         <is>
           <t>https://startupi.com.br/saiba-como-anda-a-vida-da-hotmart-mais-de-um-ano-depois-de-vencer-o-desafio-buscape/</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>Saiba como anda a vida da Hotmart mais de um ano depois de vencer o Desafio Buscapé</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="AA7" t="inlineStr">
         <is>
           <t>Startupi · fev 2013</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1465,40 +1538,42 @@
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr">
+      <c r="Q8" s="5" t="inlineStr"/>
+      <c r="R8" s="5" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
         <is>
           <t>https://headline.com</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/headlinevc</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>headline-brasil.png</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr">
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr">
         <is>
           <t>https://neofeed.com.br/startups/headline-a-nova-gestora-de-romero-rodrigues-para-investir-em-startups/</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t>Headline, a nova gestora de Romero Rodrigues para investir em startups</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="AA8" t="inlineStr">
         <is>
           <t>NeoFeed · dez 2021</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1544,40 +1619,42 @@
         </is>
       </c>
       <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr">
+      <c r="Q9" s="5" t="inlineStr"/>
+      <c r="R9" s="5" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
         <is>
           <t>https://brasil.endeavor.org/</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/endeavor-brasil</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>endeavor-brasil.png</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr">
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=TuSdKcgnNGA</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t>Day1 | Acredite no impossível - Romero Rodrigues [Buscapé]</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="AA9" t="inlineStr">
         <is>
           <t>Endeavor Brasil · nov 2012</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1627,28 +1704,30 @@
           <t>Listada na B3</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="Q10" s="5" t="inlineStr"/>
+      <c r="R10" s="5" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
         <is>
           <t>https://www.totvs.com</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/totvs</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>totvs.png</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1706,40 +1785,50 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
         <is>
           <t>https://www.vtex.com/en-us</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/vtex</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>vtex.png</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr">
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr">
         <is>
           <t>https://fusoesaquisicoes.com/acontece-no-setor/riverwood-compra-participacao-na-vtex/</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
+      <c r="Z11" t="inlineStr">
         <is>
           <t>Riverwood compra participação na VTEX da Naspers</t>
         </is>
       </c>
-      <c r="Y11" t="inlineStr">
+      <c r="AA11" t="inlineStr">
         <is>
           <t>Fusões &amp; Aquisições · mar 2015</t>
         </is>
       </c>
-      <c r="Z11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1797,36 +1886,42 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="Q12" s="5" t="inlineStr"/>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
         <is>
           <t>https://www.ifood.com.br/</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/movile-latin-america</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>movile.png</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>ifood.png</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr">
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr">
         <is>
           <t>Movile; iFood</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1872,40 +1967,46 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="Q13" s="5" t="inlineStr"/>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
         <is>
           <t>https://www.rappi.com.br</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/rappi</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>rappi.png</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr">
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr">
         <is>
           <t>https://www.wsj.com/articles/colombian-delivery-service-rappi-raising-up-to-145-million-1516327946</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="Z13" t="inlineStr">
         <is>
           <t>Colombian Delivery Service Rappi Raising Up to $145 Million</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="AA13" t="inlineStr">
         <is>
           <t>Wall Street Journal · jan 2018</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1955,40 +2056,46 @@
           <t>R$ 575M · 2019</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
         <is>
           <t>https://zup.com.br/</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/zup-it-innovation</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>zup.png</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr">
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr">
         <is>
           <t>https://valor.globo.com/financas/noticia/2019/10/31/ita-unibanco-compra-zup-servios-em-tecnologia-por-r-575-milhes.ghtml</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
+      <c r="Z14" t="inlineStr">
         <is>
           <t>Itaú Unibanco compra Zup Serviços em Tecnologia por R$ 575 milhões</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
+      <c r="AA14" t="inlineStr">
         <is>
           <t>Valor · out 2019</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -2042,40 +2149,46 @@
           <t>Adquirida · 2018</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
         <is>
           <t>https://jivemaua.com.br:443/</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/jive-investments</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>jive.png</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr">
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr">
         <is>
           <t>https://braziljournal.com/xp-compra-20-da-jive-uma-gestora-que-compra-e-resolve-problemas/</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="Z15" t="inlineStr">
         <is>
           <t>EXCLUSIVO: XP compra 20% da Jive, uma gestora que “compra e resolve problemas”</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="AA15" t="inlineStr">
         <is>
           <t>Brazil Journal · jun 2021</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2133,40 +2246,50 @@
           <t>US$ 1,8 bi · 2018</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
         <is>
           <t>https://ascenty.com/</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/ascenty</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>ascenty.png</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr">
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr">
         <is>
           <t>https://www.digitalrealty.com/about/newsroom/press-releases/122893/digital-realty-to-acquire-ascenty</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
+      <c r="Z16" t="inlineStr">
         <is>
           <t>Digital Realty To Acquire Ascenty</t>
         </is>
       </c>
-      <c r="Y16" t="inlineStr">
+      <c r="AA16" t="inlineStr">
         <is>
           <t>Digital Realty · set 2018</t>
         </is>
       </c>
-      <c r="Z16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -2212,28 +2335,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="Q17" s="5" t="inlineStr"/>
+      <c r="R17" s="5" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
         <is>
           <t>https://recargapay.com.br</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/recargapay</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>recargapay.png</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2279,28 +2404,30 @@
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr">
+      <c r="Q18" s="5" t="inlineStr"/>
+      <c r="R18" s="5" t="inlineStr"/>
+      <c r="S18" t="inlineStr">
         <is>
           <t>https://www.prosus.com</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/naspers</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>naspers-prosus.png</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -2350,28 +2477,30 @@
           <t>Listada na B3</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
+      <c r="Q19" s="5" t="inlineStr"/>
+      <c r="R19" s="5" t="inlineStr"/>
+      <c r="S19" t="inlineStr">
         <is>
           <t>https://neogrid.com</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/neogrid</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>neogrid.png</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -2417,28 +2546,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr">
+      <c r="Q20" s="5" t="inlineStr"/>
+      <c r="R20" s="5" t="inlineStr"/>
+      <c r="S20" t="inlineStr">
         <is>
           <t>https://www.viagogo.com/</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/viagogo</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>viagogo.png</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr"/>
       <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -2488,28 +2619,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
+      <c r="Q21" s="5" t="inlineStr"/>
+      <c r="R21" s="5" t="inlineStr"/>
+      <c r="S21" t="inlineStr">
         <is>
           <t>https://www.abcdaconstrucao.com.br/</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/abc-da-constru%C3%A7%C3%A3o</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>abc-da-construcao.png</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -2555,28 +2688,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr">
+      <c r="Q22" s="5" t="inlineStr"/>
+      <c r="R22" s="5" t="inlineStr"/>
+      <c r="S22" t="inlineStr">
         <is>
           <t>https://www.blips.com.br</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="T22" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/blips</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr">
+      <c r="U22" t="inlineStr">
         <is>
           <t>blips.png</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -2622,28 +2757,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr">
+      <c r="Q23" s="5" t="inlineStr"/>
+      <c r="R23" s="5" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
         <is>
           <t>https://avenia.io</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="T23" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/brla-digital</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr">
+      <c r="U23" t="inlineStr">
         <is>
           <t>avenia.png</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2689,28 +2826,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
+      <c r="Q24" s="5" t="inlineStr"/>
+      <c r="R24" s="5" t="inlineStr"/>
+      <c r="S24" t="inlineStr">
         <is>
           <t>https://condoconta.com.br</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="T24" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/condoconta</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="U24" t="inlineStr">
         <is>
           <t>condoconta.png</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr"/>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -2756,28 +2895,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr">
+      <c r="Q25" s="5" t="inlineStr"/>
+      <c r="R25" s="5" t="inlineStr"/>
+      <c r="S25" t="inlineStr">
         <is>
           <t>https://heroseguros.com.br/</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
+      <c r="T25" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/hero-seguros</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr">
+      <c r="U25" t="inlineStr">
         <is>
           <t>hero-seguros.png</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -2823,28 +2964,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
+      <c r="Q26" s="5" t="inlineStr"/>
+      <c r="R26" s="5" t="inlineStr"/>
+      <c r="S26" t="inlineStr">
         <is>
           <t>https://mercadoderecebiveis.com.br/</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="T26" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/mercado-de-receb%C3%ADveis</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="U26" t="inlineStr">
         <is>
           <t>mercado-de-recebiveis.png</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr"/>
       <c r="X26" t="inlineStr"/>
       <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -2890,28 +3033,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="Q27" s="5" t="inlineStr"/>
+      <c r="R27" s="5" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
         <is>
           <t>https://neurogram.com/</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
+      <c r="T27" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/neurogram</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr">
+      <c r="U27" t="inlineStr">
         <is>
           <t>neurogram.png</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
       <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -2957,28 +3102,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr">
+      <c r="Q28" s="5" t="inlineStr"/>
+      <c r="R28" s="5" t="inlineStr"/>
+      <c r="S28" t="inlineStr">
         <is>
           <t>https://housi.com</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
+      <c r="T28" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/housi</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr">
+      <c r="U28" t="inlineStr">
         <is>
           <t>housi.png</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -3024,28 +3171,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
+      <c r="Q29" s="5" t="inlineStr"/>
+      <c r="R29" s="5" t="inlineStr"/>
+      <c r="S29" t="inlineStr">
         <is>
           <t>https://vaas.com.br/</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
+      <c r="T29" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/vaas-1dc0</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>vaas.png</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
       <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -3091,28 +3240,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr">
+      <c r="Q30" s="5" t="inlineStr"/>
+      <c r="R30" s="5" t="inlineStr"/>
+      <c r="S30" t="inlineStr">
         <is>
           <t>https://www.tembici.com.br/pt/</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
+      <c r="T30" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/tem-bici</t>
         </is>
       </c>
-      <c r="S30" t="inlineStr">
+      <c r="U30" t="inlineStr">
         <is>
           <t>tembici.png</t>
         </is>
       </c>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr"/>
       <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -3158,28 +3309,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr">
+      <c r="Q31" s="5" t="inlineStr"/>
+      <c r="R31" s="5" t="inlineStr"/>
+      <c r="S31" t="inlineStr">
         <is>
           <t>https://eureciclo.com.br/</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
+      <c r="T31" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/eureciclo</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr">
+      <c r="U31" t="inlineStr">
         <is>
           <t>eureciclo.png</t>
         </is>
       </c>
-      <c r="T31" t="inlineStr"/>
-      <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
       <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -3225,28 +3378,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr">
+      <c r="Q32" s="5" t="inlineStr"/>
+      <c r="R32" s="5" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
         <is>
           <t>https://marketup.com</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
+      <c r="T32" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/marketup</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr">
+      <c r="U32" t="inlineStr">
         <is>
           <t>marketup.png</t>
         </is>
       </c>
-      <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr"/>
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -3292,28 +3447,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr">
+      <c r="Q33" s="5" t="inlineStr"/>
+      <c r="R33" s="5" t="inlineStr"/>
+      <c r="S33" t="inlineStr">
         <is>
           <t>https://www.delfos.energy/</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
+      <c r="T33" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/delfos-intelligent-maintenance</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr">
+      <c r="U33" t="inlineStr">
         <is>
           <t>delfos.png</t>
         </is>
       </c>
-      <c r="T33" t="inlineStr"/>
-      <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr"/>
       <c r="X33" t="inlineStr"/>
       <c r="Y33" t="inlineStr"/>
       <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -3359,24 +3516,26 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr">
+      <c r="Q34" s="5" t="inlineStr"/>
+      <c r="R34" s="5" t="inlineStr"/>
+      <c r="S34" t="inlineStr">
         <is>
           <t>https://revertai.com.br/</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr">
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr">
         <is>
           <t>revert.png</t>
         </is>
       </c>
-      <c r="T34" t="inlineStr"/>
-      <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr"/>
       <c r="W34" t="inlineStr"/>
       <c r="X34" t="inlineStr"/>
       <c r="Y34" t="inlineStr"/>
       <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr"/>
+      <c r="AB34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -3422,28 +3581,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr">
+      <c r="Q35" s="5" t="inlineStr"/>
+      <c r="R35" s="5" t="inlineStr"/>
+      <c r="S35" t="inlineStr">
         <is>
           <t>https://alia.do</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr">
+      <c r="T35" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/aliado-1328</t>
         </is>
       </c>
-      <c r="S35" t="inlineStr">
+      <c r="U35" t="inlineStr">
         <is>
           <t>alia-do.png</t>
         </is>
       </c>
-      <c r="T35" t="inlineStr"/>
-      <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr"/>
       <c r="W35" t="inlineStr"/>
       <c r="X35" t="inlineStr"/>
       <c r="Y35" t="inlineStr"/>
       <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr"/>
+      <c r="AB35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -3489,28 +3650,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr">
+      <c r="Q36" s="5" t="inlineStr"/>
+      <c r="R36" s="5" t="inlineStr"/>
+      <c r="S36" t="inlineStr">
         <is>
           <t>https://celero.com.br</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
+      <c r="T36" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/celero-534d</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
+      <c r="U36" t="inlineStr">
         <is>
           <t>celero.png</t>
         </is>
       </c>
-      <c r="T36" t="inlineStr"/>
-      <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="inlineStr"/>
       <c r="X36" t="inlineStr"/>
       <c r="Y36" t="inlineStr"/>
       <c r="Z36" t="inlineStr"/>
+      <c r="AA36" t="inlineStr"/>
+      <c r="AB36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -3556,28 +3719,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr">
+      <c r="Q37" s="5" t="inlineStr"/>
+      <c r="R37" s="5" t="inlineStr"/>
+      <c r="S37" t="inlineStr">
         <is>
           <t>https://doc9.com.br/</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
+      <c r="T37" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/doc9</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr">
+      <c r="U37" t="inlineStr">
         <is>
           <t>doc9.png</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr"/>
-      <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr"/>
       <c r="X37" t="inlineStr"/>
       <c r="Y37" t="inlineStr"/>
       <c r="Z37" t="inlineStr"/>
+      <c r="AA37" t="inlineStr"/>
+      <c r="AB37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -3623,24 +3788,26 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr">
+      <c r="Q38" s="5" t="inlineStr"/>
+      <c r="R38" s="5" t="inlineStr"/>
+      <c r="S38" t="inlineStr">
         <is>
           <t>https://jumpad.ai/</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr">
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr">
         <is>
           <t>jumpad.png</t>
         </is>
       </c>
-      <c r="T38" t="inlineStr"/>
-      <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr"/>
       <c r="X38" t="inlineStr"/>
       <c r="Y38" t="inlineStr"/>
       <c r="Z38" t="inlineStr"/>
+      <c r="AA38" t="inlineStr"/>
+      <c r="AB38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -3686,28 +3853,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr">
+      <c r="Q39" s="5" t="inlineStr"/>
+      <c r="R39" s="5" t="inlineStr"/>
+      <c r="S39" t="inlineStr">
         <is>
           <t>https://pipeimob.com.br/</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr">
+      <c r="T39" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/pipeimob</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr">
+      <c r="U39" t="inlineStr">
         <is>
           <t>pipeimob.png</t>
         </is>
       </c>
-      <c r="T39" t="inlineStr"/>
-      <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr"/>
       <c r="W39" t="inlineStr"/>
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
+      <c r="AA39" t="inlineStr"/>
+      <c r="AB39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -3753,28 +3922,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr">
+      <c r="Q40" s="5" t="inlineStr"/>
+      <c r="R40" s="5" t="inlineStr"/>
+      <c r="S40" t="inlineStr">
         <is>
           <t>https://www.horuss.ai/</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
+      <c r="T40" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/horuss-ai</t>
         </is>
       </c>
-      <c r="S40" t="inlineStr">
+      <c r="U40" t="inlineStr">
         <is>
           <t>horuss.png</t>
         </is>
       </c>
-      <c r="T40" t="inlineStr"/>
-      <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr"/>
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="inlineStr"/>
       <c r="Z40" t="inlineStr"/>
+      <c r="AA40" t="inlineStr"/>
+      <c r="AB40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -3820,28 +3991,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr">
+      <c r="Q41" s="5" t="inlineStr"/>
+      <c r="R41" s="5" t="inlineStr"/>
+      <c r="S41" t="inlineStr">
         <is>
           <t>https://turn2c.com</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr">
+      <c r="T41" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/turn2c</t>
         </is>
       </c>
-      <c r="S41" t="inlineStr">
+      <c r="U41" t="inlineStr">
         <is>
           <t>turn2c.png</t>
         </is>
       </c>
-      <c r="T41" t="inlineStr"/>
-      <c r="U41" t="inlineStr"/>
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr"/>
       <c r="X41" t="inlineStr"/>
       <c r="Y41" t="inlineStr"/>
       <c r="Z41" t="inlineStr"/>
+      <c r="AA41" t="inlineStr"/>
+      <c r="AB41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -3887,24 +4060,26 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr">
+      <c r="Q42" s="5" t="inlineStr"/>
+      <c r="R42" s="5" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/cycles-nutrition</t>
         </is>
       </c>
-      <c r="S42" t="inlineStr">
+      <c r="U42" t="inlineStr">
         <is>
           <t>cycles.png</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr"/>
-      <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="inlineStr"/>
       <c r="X42" t="inlineStr"/>
       <c r="Y42" t="inlineStr"/>
       <c r="Z42" t="inlineStr"/>
+      <c r="AA42" t="inlineStr"/>
+      <c r="AB42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -3950,28 +4125,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr">
+      <c r="Q43" s="5" t="inlineStr"/>
+      <c r="R43" s="5" t="inlineStr"/>
+      <c r="S43" t="inlineStr">
         <is>
           <t>https://fiibo.com.br</t>
         </is>
       </c>
-      <c r="R43" t="inlineStr">
+      <c r="T43" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/fiibo</t>
         </is>
       </c>
-      <c r="S43" t="inlineStr">
+      <c r="U43" t="inlineStr">
         <is>
           <t>fiibo.png</t>
         </is>
       </c>
-      <c r="T43" t="inlineStr"/>
-      <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr"/>
       <c r="W43" t="inlineStr"/>
       <c r="X43" t="inlineStr"/>
       <c r="Y43" t="inlineStr"/>
       <c r="Z43" t="inlineStr"/>
+      <c r="AA43" t="inlineStr"/>
+      <c r="AB43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -4017,24 +4194,26 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr">
+      <c r="Q44" s="5" t="inlineStr"/>
+      <c r="R44" s="5" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/fin-x</t>
         </is>
       </c>
-      <c r="S44" t="inlineStr">
+      <c r="U44" t="inlineStr">
         <is>
           <t>fin-x.png</t>
         </is>
       </c>
-      <c r="T44" t="inlineStr"/>
-      <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr"/>
       <c r="W44" t="inlineStr"/>
       <c r="X44" t="inlineStr"/>
       <c r="Y44" t="inlineStr"/>
       <c r="Z44" t="inlineStr"/>
+      <c r="AA44" t="inlineStr"/>
+      <c r="AB44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -4080,28 +4259,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr">
+      <c r="Q45" s="5" t="inlineStr"/>
+      <c r="R45" s="5" t="inlineStr"/>
+      <c r="S45" t="inlineStr">
         <is>
           <t>https://hubii.com.br/</t>
         </is>
       </c>
-      <c r="R45" t="inlineStr">
+      <c r="T45" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/hubii-7288</t>
         </is>
       </c>
-      <c r="S45" t="inlineStr">
+      <c r="U45" t="inlineStr">
         <is>
           <t>hubii.png</t>
         </is>
       </c>
-      <c r="T45" t="inlineStr"/>
-      <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr"/>
       <c r="W45" t="inlineStr"/>
       <c r="X45" t="inlineStr"/>
       <c r="Y45" t="inlineStr"/>
       <c r="Z45" t="inlineStr"/>
+      <c r="AA45" t="inlineStr"/>
+      <c r="AB45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -4147,28 +4328,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr">
+      <c r="Q46" s="5" t="inlineStr"/>
+      <c r="R46" s="5" t="inlineStr"/>
+      <c r="S46" t="inlineStr">
         <is>
           <t>https://missionbrasil.com.br/</t>
         </is>
       </c>
-      <c r="R46" t="inlineStr">
+      <c r="T46" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/mission-brasil</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr">
+      <c r="U46" t="inlineStr">
         <is>
           <t>mission-brasil.png</t>
         </is>
       </c>
-      <c r="T46" t="inlineStr"/>
-      <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr"/>
       <c r="W46" t="inlineStr"/>
       <c r="X46" t="inlineStr"/>
       <c r="Y46" t="inlineStr"/>
       <c r="Z46" t="inlineStr"/>
+      <c r="AA46" t="inlineStr"/>
+      <c r="AB46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -4214,28 +4397,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr">
+      <c r="Q47" s="5" t="inlineStr"/>
+      <c r="R47" s="5" t="inlineStr"/>
+      <c r="S47" t="inlineStr">
         <is>
           <t>https://trinus.co</t>
         </is>
       </c>
-      <c r="R47" t="inlineStr">
+      <c r="T47" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/trinus-co</t>
         </is>
       </c>
-      <c r="S47" t="inlineStr">
+      <c r="U47" t="inlineStr">
         <is>
           <t>trinus.png</t>
         </is>
       </c>
-      <c r="T47" t="inlineStr"/>
-      <c r="U47" t="inlineStr"/>
       <c r="V47" t="inlineStr"/>
       <c r="W47" t="inlineStr"/>
       <c r="X47" t="inlineStr"/>
       <c r="Y47" t="inlineStr"/>
       <c r="Z47" t="inlineStr"/>
+      <c r="AA47" t="inlineStr"/>
+      <c r="AB47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -4281,24 +4466,26 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr">
+      <c r="Q48" s="5" t="inlineStr"/>
+      <c r="R48" s="5" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/upik</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr">
+      <c r="U48" t="inlineStr">
         <is>
           <t>upik.png</t>
         </is>
       </c>
-      <c r="T48" t="inlineStr"/>
-      <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr"/>
       <c r="W48" t="inlineStr"/>
       <c r="X48" t="inlineStr"/>
       <c r="Y48" t="inlineStr"/>
       <c r="Z48" t="inlineStr"/>
+      <c r="AA48" t="inlineStr"/>
+      <c r="AB48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
@@ -4344,24 +4531,26 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr">
+      <c r="Q49" s="5" t="inlineStr"/>
+      <c r="R49" s="5" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/smart-break</t>
         </is>
       </c>
-      <c r="S49" t="inlineStr">
+      <c r="U49" t="inlineStr">
         <is>
           <t>smart-break.png</t>
         </is>
       </c>
-      <c r="T49" t="inlineStr"/>
-      <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr"/>
       <c r="W49" t="inlineStr"/>
       <c r="X49" t="inlineStr"/>
       <c r="Y49" t="inlineStr"/>
       <c r="Z49" t="inlineStr"/>
+      <c r="AA49" t="inlineStr"/>
+      <c r="AB49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -4407,28 +4596,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q50" t="inlineStr">
+      <c r="Q50" s="5" t="inlineStr"/>
+      <c r="R50" s="5" t="inlineStr"/>
+      <c r="S50" t="inlineStr">
         <is>
           <t>https://arena.im/</t>
         </is>
       </c>
-      <c r="R50" t="inlineStr">
+      <c r="T50" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/arena-im</t>
         </is>
       </c>
-      <c r="S50" t="inlineStr">
+      <c r="U50" t="inlineStr">
         <is>
           <t>arena.png</t>
         </is>
       </c>
-      <c r="T50" t="inlineStr"/>
-      <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr"/>
       <c r="W50" t="inlineStr"/>
       <c r="X50" t="inlineStr"/>
       <c r="Y50" t="inlineStr"/>
-      <c r="Z50" t="inlineStr">
+      <c r="Z50" t="inlineStr"/>
+      <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr">
         <is>
           <t>Via Redpoint eventures (seed de jun 2020).</t>
         </is>
@@ -4482,36 +4673,38 @@
         </is>
       </c>
       <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr">
+      <c r="Q51" s="5" t="inlineStr"/>
+      <c r="R51" s="5" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/grupo-xp</t>
         </is>
       </c>
-      <c r="S51" t="inlineStr">
+      <c r="U51" t="inlineStr">
         <is>
           <t>xp-inc.png</t>
         </is>
       </c>
-      <c r="T51" t="inlineStr"/>
-      <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr"/>
-      <c r="W51" t="inlineStr">
+      <c r="W51" t="inlineStr"/>
+      <c r="X51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr">
         <is>
           <t>https://valor.globo.com/financas/noticia/2022/06/09/fundo-de-venture-capital-da-xp-com-a-headline-capta-r-916-mi.ghtml</t>
         </is>
       </c>
-      <c r="X51" t="inlineStr">
+      <c r="Z51" t="inlineStr">
         <is>
           <t>Fundo de venture capital da XP com a Headline capta R$ 916 mi</t>
         </is>
       </c>
-      <c r="Y51" t="inlineStr">
+      <c r="AA51" t="inlineStr">
         <is>
           <t>Valor · jun 2022</t>
         </is>
       </c>
-      <c r="Z51" t="inlineStr"/>
+      <c r="AB51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -4561,24 +4754,30 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr">
+      <c r="Q52" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R52" s="5" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/kzas-ai</t>
         </is>
       </c>
-      <c r="S52" t="inlineStr">
+      <c r="U52" t="inlineStr">
         <is>
           <t>kzas.png</t>
         </is>
       </c>
-      <c r="T52" t="inlineStr"/>
-      <c r="U52" t="inlineStr"/>
       <c r="V52" t="inlineStr"/>
       <c r="W52" t="inlineStr"/>
       <c r="X52" t="inlineStr"/>
       <c r="Y52" t="inlineStr"/>
       <c r="Z52" t="inlineStr"/>
+      <c r="AA52" t="inlineStr"/>
+      <c r="AB52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -4628,28 +4827,34 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q53" t="inlineStr">
+      <c r="Q53" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R53" s="5" t="inlineStr"/>
+      <c r="S53" t="inlineStr">
         <is>
           <t>https://antecipa.com/</t>
         </is>
       </c>
-      <c r="R53" t="inlineStr">
+      <c r="T53" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/antecipa</t>
         </is>
       </c>
-      <c r="S53" t="inlineStr">
+      <c r="U53" t="inlineStr">
         <is>
           <t>antecipa.png</t>
         </is>
       </c>
-      <c r="T53" t="inlineStr"/>
-      <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr"/>
       <c r="W53" t="inlineStr"/>
       <c r="X53" t="inlineStr"/>
       <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="inlineStr"/>
+      <c r="AA53" t="inlineStr"/>
+      <c r="AB53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -4695,28 +4900,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q54" t="inlineStr">
+      <c r="Q54" s="5" t="inlineStr"/>
+      <c r="R54" s="5" t="inlineStr"/>
+      <c r="S54" t="inlineStr">
         <is>
           <t>https://site.stopclub.com.br/</t>
         </is>
       </c>
-      <c r="R54" t="inlineStr">
+      <c r="T54" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/stopclub</t>
         </is>
       </c>
-      <c r="S54" t="inlineStr">
+      <c r="U54" t="inlineStr">
         <is>
           <t>gigu.png</t>
         </is>
       </c>
-      <c r="T54" t="inlineStr"/>
-      <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr"/>
       <c r="W54" t="inlineStr"/>
       <c r="X54" t="inlineStr"/>
       <c r="Y54" t="inlineStr"/>
       <c r="Z54" t="inlineStr"/>
+      <c r="AA54" t="inlineStr"/>
+      <c r="AB54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
@@ -4762,28 +4969,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q55" t="inlineStr">
+      <c r="Q55" s="5" t="inlineStr"/>
+      <c r="R55" s="5" t="inlineStr"/>
+      <c r="S55" t="inlineStr">
         <is>
           <t>https://vittude.com/</t>
         </is>
       </c>
-      <c r="R55" t="inlineStr">
+      <c r="T55" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/vittude</t>
         </is>
       </c>
-      <c r="S55" t="inlineStr">
+      <c r="U55" t="inlineStr">
         <is>
           <t>vittude.png</t>
         </is>
       </c>
-      <c r="T55" t="inlineStr"/>
-      <c r="U55" t="inlineStr"/>
       <c r="V55" t="inlineStr"/>
       <c r="W55" t="inlineStr"/>
       <c r="X55" t="inlineStr"/>
       <c r="Y55" t="inlineStr"/>
       <c r="Z55" t="inlineStr"/>
+      <c r="AA55" t="inlineStr"/>
+      <c r="AB55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
@@ -4833,40 +5042,46 @@
           <t>Saída · 2021</t>
         </is>
       </c>
-      <c r="Q56" t="inlineStr">
+      <c r="Q56" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R56" s="5" t="inlineStr"/>
+      <c r="S56" t="inlineStr">
         <is>
           <t>https://www.repassa.com.br</t>
         </is>
       </c>
-      <c r="R56" t="inlineStr">
+      <c r="T56" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/repassa</t>
         </is>
       </c>
-      <c r="S56" t="inlineStr">
+      <c r="U56" t="inlineStr">
         <is>
           <t>repassa.png</t>
         </is>
       </c>
-      <c r="T56" t="inlineStr"/>
-      <c r="U56" t="inlineStr"/>
       <c r="V56" t="inlineStr"/>
-      <c r="W56" t="inlineStr">
+      <c r="W56" t="inlineStr"/>
+      <c r="X56" t="inlineStr"/>
+      <c r="Y56" t="inlineStr">
         <is>
           <t>https://braziljournal.com/renner-compra-repassa-e-entra-no-mercado-de-usados/</t>
         </is>
       </c>
-      <c r="X56" t="inlineStr">
+      <c r="Z56" t="inlineStr">
         <is>
           <t>Renner compra a Repassa</t>
         </is>
       </c>
-      <c r="Y56" t="inlineStr">
+      <c r="AA56" t="inlineStr">
         <is>
           <t>Brazil Journal · jul 2021</t>
         </is>
       </c>
-      <c r="Z56" t="inlineStr"/>
+      <c r="AB56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
@@ -4908,28 +5123,30 @@
         </is>
       </c>
       <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr">
+      <c r="Q57" s="5" t="inlineStr"/>
+      <c r="R57" s="5" t="inlineStr"/>
+      <c r="S57" t="inlineStr">
         <is>
           <t>https://www.abfintechs.com.br/</t>
         </is>
       </c>
-      <c r="R57" t="inlineStr">
+      <c r="T57" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/abfintechs</t>
         </is>
       </c>
-      <c r="S57" t="inlineStr">
+      <c r="U57" t="inlineStr">
         <is>
           <t>abfintechs.png</t>
         </is>
       </c>
-      <c r="T57" t="inlineStr"/>
-      <c r="U57" t="inlineStr"/>
       <c r="V57" t="inlineStr"/>
       <c r="W57" t="inlineStr"/>
       <c r="X57" t="inlineStr"/>
       <c r="Y57" t="inlineStr"/>
       <c r="Z57" t="inlineStr"/>
+      <c r="AA57" t="inlineStr"/>
+      <c r="AB57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
@@ -4975,24 +5192,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q58" t="inlineStr"/>
-      <c r="R58" t="inlineStr">
+      <c r="Q58" s="5" t="inlineStr"/>
+      <c r="R58" s="5" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/consulta-do-bem</t>
         </is>
       </c>
-      <c r="S58" t="inlineStr">
+      <c r="U58" t="inlineStr">
         <is>
           <t>consulta-do-bem.png</t>
         </is>
       </c>
-      <c r="T58" t="inlineStr"/>
-      <c r="U58" t="inlineStr"/>
       <c r="V58" t="inlineStr"/>
       <c r="W58" t="inlineStr"/>
       <c r="X58" t="inlineStr"/>
       <c r="Y58" t="inlineStr"/>
       <c r="Z58" t="inlineStr"/>
+      <c r="AA58" t="inlineStr"/>
+      <c r="AB58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
@@ -5042,28 +5261,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q59" t="inlineStr">
+      <c r="Q59" s="5" t="inlineStr"/>
+      <c r="R59" s="5" t="inlineStr"/>
+      <c r="S59" t="inlineStr">
         <is>
           <t>https://www.cortex-intelligence.com/en/</t>
         </is>
       </c>
-      <c r="R59" t="inlineStr">
+      <c r="T59" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/cortex-intelligence</t>
         </is>
       </c>
-      <c r="S59" t="inlineStr">
+      <c r="U59" t="inlineStr">
         <is>
           <t>cortex.png</t>
         </is>
       </c>
-      <c r="T59" t="inlineStr"/>
-      <c r="U59" t="inlineStr"/>
       <c r="V59" t="inlineStr"/>
       <c r="W59" t="inlineStr"/>
       <c r="X59" t="inlineStr"/>
       <c r="Y59" t="inlineStr"/>
-      <c r="Z59" t="inlineStr">
+      <c r="Z59" t="inlineStr"/>
+      <c r="AA59" t="inlineStr"/>
+      <c r="AB59" t="inlineStr">
         <is>
           <t>Via Redpoint eventures; conselho desde nov 2015 (Crunchbase).</t>
         </is>
@@ -5113,28 +5334,30 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q60" t="inlineStr">
+      <c r="Q60" s="5" t="inlineStr"/>
+      <c r="R60" s="5" t="inlineStr"/>
+      <c r="S60" t="inlineStr">
         <is>
           <t>https://www.incognia.com/</t>
         </is>
       </c>
-      <c r="R60" t="inlineStr">
+      <c r="T60" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/ubee</t>
         </is>
       </c>
-      <c r="S60" t="inlineStr">
+      <c r="U60" t="inlineStr">
         <is>
           <t>in-loco.png</t>
         </is>
       </c>
-      <c r="T60" t="inlineStr"/>
-      <c r="U60" t="inlineStr"/>
       <c r="V60" t="inlineStr"/>
       <c r="W60" t="inlineStr"/>
       <c r="X60" t="inlineStr"/>
       <c r="Y60" t="inlineStr"/>
       <c r="Z60" t="inlineStr"/>
+      <c r="AA60" t="inlineStr"/>
+      <c r="AB60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
@@ -5176,28 +5399,30 @@
         </is>
       </c>
       <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr">
+      <c r="Q61" s="5" t="inlineStr"/>
+      <c r="R61" s="5" t="inlineStr"/>
+      <c r="S61" t="inlineStr">
         <is>
           <t>https://corporate.payu.com</t>
         </is>
       </c>
-      <c r="R61" t="inlineStr">
+      <c r="T61" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/payu</t>
         </is>
       </c>
-      <c r="S61" t="inlineStr">
+      <c r="U61" t="inlineStr">
         <is>
           <t>payu.png</t>
         </is>
       </c>
-      <c r="T61" t="inlineStr"/>
-      <c r="U61" t="inlineStr"/>
       <c r="V61" t="inlineStr"/>
       <c r="W61" t="inlineStr"/>
       <c r="X61" t="inlineStr"/>
       <c r="Y61" t="inlineStr"/>
       <c r="Z61" t="inlineStr"/>
+      <c r="AA61" t="inlineStr"/>
+      <c r="AB61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -5239,20 +5464,22 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr"/>
+      <c r="Q62" s="5" t="inlineStr"/>
+      <c r="R62" s="5" t="inlineStr"/>
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr"/>
       <c r="U62" t="inlineStr"/>
       <c r="V62" t="inlineStr"/>
-      <c r="W62" t="inlineStr">
+      <c r="W62" t="inlineStr"/>
+      <c r="X62" t="inlineStr"/>
+      <c r="Y62" t="inlineStr">
         <is>
           <t>https://retail.economictimes.indiatimes.com/news/e-commerce/e-tailing/ibibo-sells-online-payment-unit-payu-india-to-naspers/30471071</t>
         </is>
       </c>
-      <c r="X62" t="inlineStr"/>
-      <c r="Y62" t="inlineStr"/>
       <c r="Z62" t="inlineStr"/>
+      <c r="AA62" t="inlineStr"/>
+      <c r="AB62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
@@ -5298,28 +5525,34 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q63" t="inlineStr">
+      <c r="Q63" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R63" s="5" t="inlineStr"/>
+      <c r="S63" t="inlineStr">
         <is>
           <t>https://www.cuponeria.com.br</t>
         </is>
       </c>
-      <c r="R63" t="inlineStr">
+      <c r="T63" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/cuponeria</t>
         </is>
       </c>
-      <c r="S63" t="inlineStr">
+      <c r="U63" t="inlineStr">
         <is>
           <t>cuponeria.png</t>
         </is>
       </c>
-      <c r="T63" t="inlineStr"/>
-      <c r="U63" t="inlineStr"/>
       <c r="V63" t="inlineStr"/>
       <c r="W63" t="inlineStr"/>
       <c r="X63" t="inlineStr"/>
       <c r="Y63" t="inlineStr"/>
       <c r="Z63" t="inlineStr"/>
+      <c r="AA63" t="inlineStr"/>
+      <c r="AB63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -5365,40 +5598,42 @@
         </is>
       </c>
       <c r="P64" t="inlineStr"/>
-      <c r="Q64" t="inlineStr">
+      <c r="Q64" s="5" t="inlineStr"/>
+      <c r="R64" s="5" t="inlineStr"/>
+      <c r="S64" t="inlineStr">
         <is>
           <t>https://rpev.com.br/</t>
         </is>
       </c>
-      <c r="R64" t="inlineStr">
+      <c r="T64" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/redpoint-eventures</t>
         </is>
       </c>
-      <c r="S64" t="inlineStr">
+      <c r="U64" t="inlineStr">
         <is>
           <t>redpoint-eventures.png</t>
         </is>
       </c>
-      <c r="T64" t="inlineStr"/>
-      <c r="U64" t="inlineStr"/>
       <c r="V64" t="inlineStr"/>
-      <c r="W64" t="inlineStr">
+      <c r="W64" t="inlineStr"/>
+      <c r="X64" t="inlineStr"/>
+      <c r="Y64" t="inlineStr">
         <is>
           <t>https://www.nytimes.com/2015/11/11/business/dealbook/redpoint-joint-venture-in-brazil-adds-romero-rodrigues-a-top-entrepreneur.html</t>
         </is>
       </c>
-      <c r="X64" t="inlineStr">
+      <c r="Z64" t="inlineStr">
         <is>
           <t>Redpoint Joint Venture in Brazil Adds Romero Rodrigues, a Top Entrepreneur</t>
         </is>
       </c>
-      <c r="Y64" t="inlineStr">
+      <c r="AA64" t="inlineStr">
         <is>
           <t>New York Times · nov 2015</t>
         </is>
       </c>
-      <c r="Z64" t="inlineStr"/>
+      <c r="AB64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
@@ -5444,24 +5679,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q65" t="inlineStr"/>
-      <c r="R65" t="inlineStr">
+      <c r="Q65" s="5" t="inlineStr"/>
+      <c r="R65" s="5" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
+      <c r="T65" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/shopcliq</t>
         </is>
       </c>
-      <c r="S65" t="inlineStr">
+      <c r="U65" t="inlineStr">
         <is>
           <t>shopcliq.png</t>
         </is>
       </c>
-      <c r="T65" t="inlineStr"/>
-      <c r="U65" t="inlineStr"/>
       <c r="V65" t="inlineStr"/>
       <c r="W65" t="inlineStr"/>
       <c r="X65" t="inlineStr"/>
       <c r="Y65" t="inlineStr"/>
       <c r="Z65" t="inlineStr"/>
+      <c r="AA65" t="inlineStr"/>
+      <c r="AB65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -5507,24 +5744,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q66" t="inlineStr"/>
-      <c r="R66" t="inlineStr">
+      <c r="Q66" s="5" t="inlineStr"/>
+      <c r="R66" s="5" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/brandsclub</t>
         </is>
       </c>
-      <c r="S66" t="inlineStr">
+      <c r="U66" t="inlineStr">
         <is>
           <t>brandsclub.png</t>
         </is>
       </c>
-      <c r="T66" t="inlineStr"/>
-      <c r="U66" t="inlineStr"/>
       <c r="V66" t="inlineStr"/>
       <c r="W66" t="inlineStr"/>
       <c r="X66" t="inlineStr"/>
       <c r="Y66" t="inlineStr"/>
       <c r="Z66" t="inlineStr"/>
+      <c r="AA66" t="inlineStr"/>
+      <c r="AB66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
@@ -5574,24 +5813,30 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q67" t="inlineStr"/>
-      <c r="R67" t="inlineStr">
+      <c r="Q67" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R67" s="5" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/dineromail</t>
         </is>
       </c>
-      <c r="S67" t="inlineStr">
+      <c r="U67" t="inlineStr">
         <is>
           <t>dineromail.png</t>
         </is>
       </c>
-      <c r="T67" t="inlineStr"/>
-      <c r="U67" t="inlineStr"/>
       <c r="V67" t="inlineStr"/>
       <c r="W67" t="inlineStr"/>
       <c r="X67" t="inlineStr"/>
       <c r="Y67" t="inlineStr"/>
       <c r="Z67" t="inlineStr"/>
+      <c r="AA67" t="inlineStr"/>
+      <c r="AB67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -5637,24 +5882,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q68" t="inlineStr"/>
-      <c r="R68" t="inlineStr">
+      <c r="Q68" s="5" t="inlineStr"/>
+      <c r="R68" s="5" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/meucarrinho</t>
         </is>
       </c>
-      <c r="S68" t="inlineStr">
+      <c r="U68" t="inlineStr">
         <is>
           <t>meucarrinho.png</t>
         </is>
       </c>
-      <c r="T68" t="inlineStr"/>
-      <c r="U68" t="inlineStr"/>
       <c r="V68" t="inlineStr"/>
       <c r="W68" t="inlineStr"/>
       <c r="X68" t="inlineStr"/>
       <c r="Y68" t="inlineStr"/>
       <c r="Z68" t="inlineStr"/>
+      <c r="AA68" t="inlineStr"/>
+      <c r="AB68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
@@ -5700,28 +5947,30 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q69" t="inlineStr">
+      <c r="Q69" s="5" t="inlineStr"/>
+      <c r="R69" s="5" t="inlineStr"/>
+      <c r="S69" t="inlineStr">
         <is>
           <t>https://modait.com.br/</t>
         </is>
       </c>
-      <c r="R69" t="inlineStr">
+      <c r="T69" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/moda-it</t>
         </is>
       </c>
-      <c r="S69" t="inlineStr">
+      <c r="U69" t="inlineStr">
         <is>
           <t>moda-it.png</t>
         </is>
       </c>
-      <c r="T69" t="inlineStr"/>
-      <c r="U69" t="inlineStr"/>
       <c r="V69" t="inlineStr"/>
       <c r="W69" t="inlineStr"/>
       <c r="X69" t="inlineStr"/>
       <c r="Y69" t="inlineStr"/>
       <c r="Z69" t="inlineStr"/>
+      <c r="AA69" t="inlineStr"/>
+      <c r="AB69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -5771,28 +6020,34 @@
           <t>Saída · 2015</t>
         </is>
       </c>
-      <c r="Q70" t="inlineStr">
+      <c r="Q70" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R70" s="5" t="inlineStr"/>
+      <c r="S70" t="inlineStr">
         <is>
           <t>https://www.navegg.com/br</t>
         </is>
       </c>
-      <c r="R70" t="inlineStr">
+      <c r="T70" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/navegg</t>
         </is>
       </c>
-      <c r="S70" t="inlineStr">
+      <c r="U70" t="inlineStr">
         <is>
           <t>navegg.png</t>
         </is>
       </c>
-      <c r="T70" t="inlineStr"/>
-      <c r="U70" t="inlineStr"/>
       <c r="V70" t="inlineStr"/>
       <c r="W70" t="inlineStr"/>
       <c r="X70" t="inlineStr"/>
       <c r="Y70" t="inlineStr"/>
       <c r="Z70" t="inlineStr"/>
+      <c r="AA70" t="inlineStr"/>
+      <c r="AB70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
@@ -5838,20 +6093,22 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q71" t="inlineStr"/>
-      <c r="R71" t="inlineStr">
+      <c r="Q71" s="5" t="inlineStr"/>
+      <c r="R71" s="5" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/recomind-net</t>
         </is>
       </c>
-      <c r="S71" t="inlineStr"/>
-      <c r="T71" t="inlineStr"/>
       <c r="U71" t="inlineStr"/>
       <c r="V71" t="inlineStr"/>
       <c r="W71" t="inlineStr"/>
       <c r="X71" t="inlineStr"/>
       <c r="Y71" t="inlineStr"/>
       <c r="Z71" t="inlineStr"/>
+      <c r="AA71" t="inlineStr"/>
+      <c r="AB71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -5897,24 +6154,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr">
+      <c r="Q72" s="5" t="inlineStr"/>
+      <c r="R72" s="5" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/urbanizo</t>
         </is>
       </c>
-      <c r="S72" t="inlineStr">
+      <c r="U72" t="inlineStr">
         <is>
           <t>urbanizo.png</t>
         </is>
       </c>
-      <c r="T72" t="inlineStr"/>
-      <c r="U72" t="inlineStr"/>
       <c r="V72" t="inlineStr"/>
       <c r="W72" t="inlineStr"/>
       <c r="X72" t="inlineStr"/>
       <c r="Y72" t="inlineStr"/>
       <c r="Z72" t="inlineStr"/>
+      <c r="AA72" t="inlineStr"/>
+      <c r="AB72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
@@ -5964,24 +6223,30 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q73" t="inlineStr"/>
-      <c r="R73" t="inlineStr">
+      <c r="Q73" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R73" s="5" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/pagosonline</t>
         </is>
       </c>
-      <c r="S73" t="inlineStr">
+      <c r="U73" t="inlineStr">
         <is>
           <t>pagosonline.png</t>
         </is>
       </c>
-      <c r="T73" t="inlineStr"/>
-      <c r="U73" t="inlineStr"/>
       <c r="V73" t="inlineStr"/>
       <c r="W73" t="inlineStr"/>
       <c r="X73" t="inlineStr"/>
       <c r="Y73" t="inlineStr"/>
       <c r="Z73" t="inlineStr"/>
+      <c r="AA73" t="inlineStr"/>
+      <c r="AB73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
@@ -6027,24 +6292,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q74" t="inlineStr"/>
-      <c r="R74" t="inlineStr">
+      <c r="Q74" s="5" t="inlineStr"/>
+      <c r="R74" s="5" t="inlineStr"/>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/saveme</t>
         </is>
       </c>
-      <c r="S74" t="inlineStr">
+      <c r="U74" t="inlineStr">
         <is>
           <t>saveme-2026.png</t>
         </is>
       </c>
-      <c r="T74" t="inlineStr"/>
-      <c r="U74" t="inlineStr"/>
       <c r="V74" t="inlineStr"/>
       <c r="W74" t="inlineStr"/>
       <c r="X74" t="inlineStr"/>
       <c r="Y74" t="inlineStr"/>
       <c r="Z74" t="inlineStr"/>
+      <c r="AA74" t="inlineStr"/>
+      <c r="AB74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
@@ -6090,24 +6357,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q75" t="inlineStr"/>
-      <c r="R75" t="inlineStr">
+      <c r="Q75" s="5" t="inlineStr"/>
+      <c r="R75" s="5" t="inlineStr"/>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/ebehavior-b888</t>
         </is>
       </c>
-      <c r="S75" t="inlineStr">
+      <c r="U75" t="inlineStr">
         <is>
           <t>ebehavior.png</t>
         </is>
       </c>
-      <c r="T75" t="inlineStr"/>
-      <c r="U75" t="inlineStr"/>
       <c r="V75" t="inlineStr"/>
       <c r="W75" t="inlineStr"/>
       <c r="X75" t="inlineStr"/>
       <c r="Y75" t="inlineStr"/>
       <c r="Z75" t="inlineStr"/>
+      <c r="AA75" t="inlineStr"/>
+      <c r="AB75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
@@ -6157,24 +6426,30 @@
           <t>Saída · 2024</t>
         </is>
       </c>
-      <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="inlineStr">
+      <c r="Q76" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R76" s="5" t="inlineStr"/>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/lomadee</t>
         </is>
       </c>
-      <c r="S76" t="inlineStr">
+      <c r="U76" t="inlineStr">
         <is>
           <t>lomadee.png</t>
         </is>
       </c>
-      <c r="T76" t="inlineStr"/>
-      <c r="U76" t="inlineStr"/>
       <c r="V76" t="inlineStr"/>
       <c r="W76" t="inlineStr"/>
       <c r="X76" t="inlineStr"/>
       <c r="Y76" t="inlineStr"/>
       <c r="Z76" t="inlineStr"/>
+      <c r="AA76" t="inlineStr"/>
+      <c r="AB76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
@@ -6228,32 +6503,38 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q77" t="inlineStr"/>
-      <c r="R77" t="inlineStr">
+      <c r="Q77" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R77" s="5" t="inlineStr"/>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/pagamento-digital</t>
         </is>
       </c>
-      <c r="S77" t="inlineStr">
+      <c r="U77" t="inlineStr">
         <is>
           <t>pagamento-digital.png</t>
         </is>
       </c>
-      <c r="T77" t="inlineStr"/>
-      <c r="U77" t="inlineStr">
+      <c r="V77" t="inlineStr"/>
+      <c r="W77" t="inlineStr">
         <is>
           <t>Bcash</t>
         </is>
       </c>
-      <c r="V77" t="inlineStr">
+      <c r="X77" t="inlineStr">
         <is>
           <t>Pagamento Digital</t>
         </is>
       </c>
-      <c r="W77" t="inlineStr"/>
-      <c r="X77" t="inlineStr"/>
       <c r="Y77" t="inlineStr"/>
       <c r="Z77" t="inlineStr"/>
+      <c r="AA77" t="inlineStr"/>
+      <c r="AB77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -6303,24 +6584,30 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q78" t="inlineStr"/>
-      <c r="R78" t="inlineStr">
+      <c r="Q78" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R78" s="5" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/f-control</t>
         </is>
       </c>
-      <c r="S78" t="inlineStr">
+      <c r="U78" t="inlineStr">
         <is>
           <t>fcontrol.png</t>
         </is>
       </c>
-      <c r="T78" t="inlineStr"/>
-      <c r="U78" t="inlineStr"/>
       <c r="V78" t="inlineStr"/>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
       <c r="Y78" t="inlineStr"/>
       <c r="Z78" t="inlineStr"/>
+      <c r="AA78" t="inlineStr"/>
+      <c r="AB78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
@@ -6370,24 +6657,30 @@
           <t>Saída · 2024</t>
         </is>
       </c>
-      <c r="Q79" t="inlineStr"/>
-      <c r="R79" t="inlineStr">
+      <c r="Q79" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R79" s="5" t="inlineStr"/>
+      <c r="S79" t="inlineStr"/>
+      <c r="T79" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/e-bit</t>
         </is>
       </c>
-      <c r="S79" t="inlineStr">
+      <c r="U79" t="inlineStr">
         <is>
           <t>e-bit.png</t>
         </is>
       </c>
-      <c r="T79" t="inlineStr"/>
-      <c r="U79" t="inlineStr"/>
       <c r="V79" t="inlineStr"/>
       <c r="W79" t="inlineStr"/>
       <c r="X79" t="inlineStr"/>
       <c r="Y79" t="inlineStr"/>
       <c r="Z79" t="inlineStr"/>
+      <c r="AA79" t="inlineStr"/>
+      <c r="AB79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
@@ -6429,28 +6722,30 @@
         </is>
       </c>
       <c r="P80" t="inlineStr"/>
-      <c r="Q80" t="inlineStr">
+      <c r="Q80" s="5" t="inlineStr"/>
+      <c r="R80" s="5" t="inlineStr"/>
+      <c r="S80" t="inlineStr">
         <is>
           <t>https://www.bondfaro.com.br/</t>
         </is>
       </c>
-      <c r="R80" t="inlineStr">
+      <c r="T80" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/bondfaro</t>
         </is>
       </c>
-      <c r="S80" t="inlineStr">
+      <c r="U80" t="inlineStr">
         <is>
           <t>bondfaro-2026.png</t>
         </is>
       </c>
-      <c r="T80" t="inlineStr"/>
-      <c r="U80" t="inlineStr"/>
       <c r="V80" t="inlineStr"/>
       <c r="W80" t="inlineStr"/>
       <c r="X80" t="inlineStr"/>
       <c r="Y80" t="inlineStr"/>
       <c r="Z80" t="inlineStr"/>
+      <c r="AA80" t="inlineStr"/>
+      <c r="AB80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
@@ -6496,24 +6791,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q81" t="inlineStr"/>
-      <c r="R81" t="inlineStr">
+      <c r="Q81" s="5" t="inlineStr"/>
+      <c r="R81" s="5" t="inlineStr"/>
+      <c r="S81" t="inlineStr"/>
+      <c r="T81" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/cortacontas</t>
         </is>
       </c>
-      <c r="S81" t="inlineStr">
+      <c r="U81" t="inlineStr">
         <is>
           <t>cortacontas.png</t>
         </is>
       </c>
-      <c r="T81" t="inlineStr"/>
-      <c r="U81" t="inlineStr"/>
       <c r="V81" t="inlineStr"/>
       <c r="W81" t="inlineStr"/>
       <c r="X81" t="inlineStr"/>
       <c r="Y81" t="inlineStr"/>
       <c r="Z81" t="inlineStr"/>
+      <c r="AA81" t="inlineStr"/>
+      <c r="AB81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
@@ -6559,28 +6856,30 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q82" t="inlineStr">
+      <c r="Q82" s="5" t="inlineStr"/>
+      <c r="R82" s="5" t="inlineStr"/>
+      <c r="S82" t="inlineStr">
         <is>
           <t>https://www.quebarato.com.br/</t>
         </is>
       </c>
-      <c r="R82" t="inlineStr">
+      <c r="T82" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/quebarato</t>
         </is>
       </c>
-      <c r="S82" t="inlineStr">
+      <c r="U82" t="inlineStr">
         <is>
           <t>quebarato.png</t>
         </is>
       </c>
-      <c r="T82" t="inlineStr"/>
-      <c r="U82" t="inlineStr"/>
       <c r="V82" t="inlineStr"/>
       <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr"/>
       <c r="Y82" t="inlineStr"/>
       <c r="Z82" t="inlineStr"/>
+      <c r="AA82" t="inlineStr"/>
+      <c r="AB82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
@@ -6630,8 +6929,12 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q83" t="inlineStr"/>
-      <c r="R83" t="inlineStr"/>
+      <c r="Q83" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R83" s="5" t="inlineStr"/>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="inlineStr"/>
       <c r="U83" t="inlineStr"/>
@@ -6640,6 +6943,8 @@
       <c r="X83" t="inlineStr"/>
       <c r="Y83" t="inlineStr"/>
       <c r="Z83" t="inlineStr"/>
+      <c r="AA83" t="inlineStr"/>
+      <c r="AB83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -6689,24 +6994,30 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q84" t="inlineStr"/>
-      <c r="R84" t="inlineStr">
+      <c r="Q84" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R84" s="5" t="inlineStr"/>
+      <c r="S84" t="inlineStr"/>
+      <c r="T84" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/mirum-agency; https://www.crunchbase.com/organization/m%C3%ADdia-digital</t>
         </is>
       </c>
-      <c r="S84" t="inlineStr">
+      <c r="U84" t="inlineStr">
         <is>
           <t>mirum.png</t>
         </is>
       </c>
-      <c r="T84" t="inlineStr"/>
-      <c r="U84" t="inlineStr"/>
       <c r="V84" t="inlineStr"/>
       <c r="W84" t="inlineStr"/>
       <c r="X84" t="inlineStr"/>
       <c r="Y84" t="inlineStr"/>
       <c r="Z84" t="inlineStr"/>
+      <c r="AA84" t="inlineStr"/>
+      <c r="AB84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
@@ -6756,8 +7067,8 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q85" t="inlineStr"/>
-      <c r="R85" t="inlineStr"/>
+      <c r="Q85" s="5" t="inlineStr"/>
+      <c r="R85" s="5" t="inlineStr"/>
       <c r="S85" t="inlineStr"/>
       <c r="T85" t="inlineStr"/>
       <c r="U85" t="inlineStr"/>
@@ -6766,6 +7077,8 @@
       <c r="X85" t="inlineStr"/>
       <c r="Y85" t="inlineStr"/>
       <c r="Z85" t="inlineStr"/>
+      <c r="AA85" t="inlineStr"/>
+      <c r="AB85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
@@ -6811,28 +7124,34 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q86" t="inlineStr">
+      <c r="Q86" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R86" s="5" t="inlineStr"/>
+      <c r="S86" t="inlineStr">
         <is>
           <t>https://awl.com/</t>
         </is>
       </c>
-      <c r="R86" t="inlineStr">
+      <c r="T86" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/awl-fee7</t>
         </is>
       </c>
-      <c r="S86" t="inlineStr">
+      <c r="U86" t="inlineStr">
         <is>
           <t>awl-leads.png</t>
         </is>
       </c>
-      <c r="T86" t="inlineStr"/>
-      <c r="U86" t="inlineStr"/>
       <c r="V86" t="inlineStr"/>
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr"/>
       <c r="Y86" t="inlineStr"/>
       <c r="Z86" t="inlineStr"/>
+      <c r="AA86" t="inlineStr"/>
+      <c r="AB86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
@@ -6886,28 +7205,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q87" t="inlineStr">
+      <c r="Q87" s="5" t="inlineStr"/>
+      <c r="R87" s="5" t="inlineStr"/>
+      <c r="S87" t="inlineStr">
         <is>
           <t>https://biosphera.network/en/</t>
         </is>
       </c>
-      <c r="R87" t="inlineStr">
+      <c r="T87" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/b-partners-6cab</t>
         </is>
       </c>
-      <c r="S87" t="inlineStr">
+      <c r="U87" t="inlineStr">
         <is>
           <t>biosphera.png</t>
         </is>
       </c>
-      <c r="T87" t="inlineStr"/>
-      <c r="U87" t="inlineStr"/>
       <c r="V87" t="inlineStr"/>
       <c r="W87" t="inlineStr"/>
       <c r="X87" t="inlineStr"/>
       <c r="Y87" t="inlineStr"/>
-      <c r="Z87" t="inlineStr">
+      <c r="Z87" t="inlineStr"/>
+      <c r="AA87" t="inlineStr"/>
+      <c r="AB87" t="inlineStr">
         <is>
           <t>Anjo. Crunchbase ainda aponta o site antigo (bpartners.com.br).</t>
         </is>
@@ -6953,28 +7274,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q88" t="inlineStr">
+      <c r="Q88" s="5" t="inlineStr"/>
+      <c r="R88" s="5" t="inlineStr"/>
+      <c r="S88" t="inlineStr">
         <is>
           <t>https://bovplatform.com/about</t>
         </is>
       </c>
-      <c r="R88" t="inlineStr">
+      <c r="T88" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/bovcontrol</t>
         </is>
       </c>
-      <c r="S88" t="inlineStr">
+      <c r="U88" t="inlineStr">
         <is>
           <t>bovcontrol.png</t>
         </is>
       </c>
-      <c r="T88" t="inlineStr"/>
-      <c r="U88" t="inlineStr"/>
       <c r="V88" t="inlineStr"/>
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr"/>
       <c r="Y88" t="inlineStr"/>
       <c r="Z88" t="inlineStr"/>
+      <c r="AA88" t="inlineStr"/>
+      <c r="AB88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
@@ -7020,28 +7343,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q89" t="inlineStr">
+      <c r="Q89" s="5" t="inlineStr"/>
+      <c r="R89" s="5" t="inlineStr"/>
+      <c r="S89" t="inlineStr">
         <is>
           <t>https://www.canaldapeca.com.br/</t>
         </is>
       </c>
-      <c r="R89" t="inlineStr">
+      <c r="T89" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/canal-da-pe%C3%A7a</t>
         </is>
       </c>
-      <c r="S89" t="inlineStr">
+      <c r="U89" t="inlineStr">
         <is>
           <t>canal-da-peca.png</t>
         </is>
       </c>
-      <c r="T89" t="inlineStr"/>
-      <c r="U89" t="inlineStr"/>
       <c r="V89" t="inlineStr"/>
       <c r="W89" t="inlineStr"/>
       <c r="X89" t="inlineStr"/>
       <c r="Y89" t="inlineStr"/>
       <c r="Z89" t="inlineStr"/>
+      <c r="AA89" t="inlineStr"/>
+      <c r="AB89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
@@ -7087,28 +7412,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q90" t="inlineStr">
+      <c r="Q90" s="5" t="inlineStr"/>
+      <c r="R90" s="5" t="inlineStr"/>
+      <c r="S90" t="inlineStr">
         <is>
           <t>https://www.clicksign.com</t>
         </is>
       </c>
-      <c r="R90" t="inlineStr">
+      <c r="T90" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/clicksign</t>
         </is>
       </c>
-      <c r="S90" t="inlineStr">
+      <c r="U90" t="inlineStr">
         <is>
           <t>clicksign.png</t>
         </is>
       </c>
-      <c r="T90" t="inlineStr"/>
-      <c r="U90" t="inlineStr"/>
       <c r="V90" t="inlineStr"/>
       <c r="W90" t="inlineStr"/>
       <c r="X90" t="inlineStr"/>
       <c r="Y90" t="inlineStr"/>
       <c r="Z90" t="inlineStr"/>
+      <c r="AA90" t="inlineStr"/>
+      <c r="AB90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
@@ -7150,24 +7477,26 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q91" t="inlineStr"/>
-      <c r="R91" t="inlineStr">
+      <c r="Q91" s="5" t="inlineStr"/>
+      <c r="R91" s="5" t="inlineStr"/>
+      <c r="S91" t="inlineStr"/>
+      <c r="T91" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/hi-platform</t>
         </is>
       </c>
-      <c r="S91" t="inlineStr">
+      <c r="U91" t="inlineStr">
         <is>
           <t>directtalk.png</t>
         </is>
       </c>
-      <c r="T91" t="inlineStr"/>
-      <c r="U91" t="inlineStr"/>
       <c r="V91" t="inlineStr"/>
       <c r="W91" t="inlineStr"/>
       <c r="X91" t="inlineStr"/>
       <c r="Y91" t="inlineStr"/>
       <c r="Z91" t="inlineStr"/>
+      <c r="AA91" t="inlineStr"/>
+      <c r="AB91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
@@ -7209,28 +7538,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q92" t="inlineStr">
+      <c r="Q92" s="5" t="inlineStr"/>
+      <c r="R92" s="5" t="inlineStr"/>
+      <c r="S92" t="inlineStr">
         <is>
           <t>https://www.galena.com</t>
         </is>
       </c>
-      <c r="R92" t="inlineStr">
+      <c r="T92" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/galena-c08c</t>
         </is>
       </c>
-      <c r="S92" t="inlineStr">
+      <c r="U92" t="inlineStr">
         <is>
           <t>galena.png</t>
         </is>
       </c>
-      <c r="T92" t="inlineStr"/>
-      <c r="U92" t="inlineStr"/>
       <c r="V92" t="inlineStr"/>
       <c r="W92" t="inlineStr"/>
       <c r="X92" t="inlineStr"/>
       <c r="Y92" t="inlineStr"/>
       <c r="Z92" t="inlineStr"/>
+      <c r="AA92" t="inlineStr"/>
+      <c r="AB92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
@@ -7272,24 +7603,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q93" t="inlineStr"/>
-      <c r="R93" t="inlineStr">
+      <c r="Q93" s="5" t="inlineStr"/>
+      <c r="R93" s="5" t="inlineStr"/>
+      <c r="S93" t="inlineStr"/>
+      <c r="T93" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/grubster</t>
         </is>
       </c>
-      <c r="S93" t="inlineStr">
+      <c r="U93" t="inlineStr">
         <is>
           <t>chefsclub-grubster.png</t>
         </is>
       </c>
-      <c r="T93" t="inlineStr"/>
-      <c r="U93" t="inlineStr"/>
       <c r="V93" t="inlineStr"/>
       <c r="W93" t="inlineStr"/>
       <c r="X93" t="inlineStr"/>
       <c r="Y93" t="inlineStr"/>
       <c r="Z93" t="inlineStr"/>
+      <c r="AA93" t="inlineStr"/>
+      <c r="AB93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
@@ -7331,20 +7664,22 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q94" t="inlineStr"/>
-      <c r="R94" t="inlineStr"/>
-      <c r="S94" t="inlineStr">
+      <c r="Q94" s="5" t="inlineStr"/>
+      <c r="R94" s="5" t="inlineStr"/>
+      <c r="S94" t="inlineStr"/>
+      <c r="T94" t="inlineStr"/>
+      <c r="U94" t="inlineStr">
         <is>
           <t>humortadela.png</t>
         </is>
       </c>
-      <c r="T94" t="inlineStr"/>
-      <c r="U94" t="inlineStr"/>
       <c r="V94" t="inlineStr"/>
       <c r="W94" t="inlineStr"/>
       <c r="X94" t="inlineStr"/>
       <c r="Y94" t="inlineStr"/>
       <c r="Z94" t="inlineStr"/>
+      <c r="AA94" t="inlineStr"/>
+      <c r="AB94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
@@ -7386,28 +7721,34 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q95" t="inlineStr">
+      <c r="Q95" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R95" s="5" t="inlineStr"/>
+      <c r="S95" t="inlineStr">
         <is>
           <t>https://ingresse.com/</t>
         </is>
       </c>
-      <c r="R95" t="inlineStr">
+      <c r="T95" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/ingresse</t>
         </is>
       </c>
-      <c r="S95" t="inlineStr">
+      <c r="U95" t="inlineStr">
         <is>
           <t>ingresse.png</t>
         </is>
       </c>
-      <c r="T95" t="inlineStr"/>
-      <c r="U95" t="inlineStr"/>
       <c r="V95" t="inlineStr"/>
       <c r="W95" t="inlineStr"/>
       <c r="X95" t="inlineStr"/>
       <c r="Y95" t="inlineStr"/>
       <c r="Z95" t="inlineStr"/>
+      <c r="AA95" t="inlineStr"/>
+      <c r="AB95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
@@ -7453,24 +7794,30 @@
           <t>Adquirida</t>
         </is>
       </c>
-      <c r="Q96" t="inlineStr"/>
-      <c r="R96" t="inlineStr">
+      <c r="Q96" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R96" s="5" t="inlineStr"/>
+      <c r="S96" t="inlineStr"/>
+      <c r="T96" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/lema21</t>
         </is>
       </c>
-      <c r="S96" t="inlineStr">
+      <c r="U96" t="inlineStr">
         <is>
           <t>lema21.png</t>
         </is>
       </c>
-      <c r="T96" t="inlineStr"/>
-      <c r="U96" t="inlineStr"/>
       <c r="V96" t="inlineStr"/>
       <c r="W96" t="inlineStr"/>
       <c r="X96" t="inlineStr"/>
       <c r="Y96" t="inlineStr"/>
       <c r="Z96" t="inlineStr"/>
+      <c r="AA96" t="inlineStr"/>
+      <c r="AB96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
@@ -7512,28 +7859,30 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q97" t="inlineStr">
+      <c r="Q97" s="5" t="inlineStr"/>
+      <c r="R97" s="5" t="inlineStr"/>
+      <c r="S97" t="inlineStr">
         <is>
           <t>https://www.prontmed.com</t>
         </is>
       </c>
-      <c r="R97" t="inlineStr">
+      <c r="T97" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/prontmed</t>
         </is>
       </c>
-      <c r="S97" t="inlineStr">
+      <c r="U97" t="inlineStr">
         <is>
           <t>prontmed.png</t>
         </is>
       </c>
-      <c r="T97" t="inlineStr"/>
-      <c r="U97" t="inlineStr"/>
       <c r="V97" t="inlineStr"/>
       <c r="W97" t="inlineStr"/>
       <c r="X97" t="inlineStr"/>
       <c r="Y97" t="inlineStr"/>
       <c r="Z97" t="inlineStr"/>
+      <c r="AA97" t="inlineStr"/>
+      <c r="AB97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
@@ -7575,28 +7924,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q98" t="inlineStr">
+      <c r="Q98" s="5" t="inlineStr"/>
+      <c r="R98" s="5" t="inlineStr"/>
+      <c r="S98" t="inlineStr">
         <is>
           <t>https://qipu.com.br/</t>
         </is>
       </c>
-      <c r="R98" t="inlineStr">
+      <c r="T98" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/qipu</t>
         </is>
       </c>
-      <c r="S98" t="inlineStr">
+      <c r="U98" t="inlineStr">
         <is>
           <t>qipu-mei-gratis.png</t>
         </is>
       </c>
-      <c r="T98" t="inlineStr"/>
-      <c r="U98" t="inlineStr"/>
       <c r="V98" t="inlineStr"/>
       <c r="W98" t="inlineStr"/>
       <c r="X98" t="inlineStr"/>
       <c r="Y98" t="inlineStr"/>
       <c r="Z98" t="inlineStr"/>
+      <c r="AA98" t="inlineStr"/>
+      <c r="AB98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
@@ -7638,24 +7989,26 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q99" t="inlineStr"/>
-      <c r="R99" t="inlineStr">
+      <c r="Q99" s="5" t="inlineStr"/>
+      <c r="R99" s="5" t="inlineStr"/>
+      <c r="S99" t="inlineStr"/>
+      <c r="T99" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/quero-education</t>
         </is>
       </c>
-      <c r="S99" t="inlineStr">
+      <c r="U99" t="inlineStr">
         <is>
           <t>quero-educacao.png</t>
         </is>
       </c>
-      <c r="T99" t="inlineStr"/>
-      <c r="U99" t="inlineStr"/>
       <c r="V99" t="inlineStr"/>
       <c r="W99" t="inlineStr"/>
       <c r="X99" t="inlineStr"/>
       <c r="Y99" t="inlineStr"/>
       <c r="Z99" t="inlineStr"/>
+      <c r="AA99" t="inlineStr"/>
+      <c r="AB99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
@@ -7701,28 +8054,34 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q100" t="inlineStr">
+      <c r="Q100" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R100" s="5" t="inlineStr"/>
+      <c r="S100" t="inlineStr">
         <is>
           <t>https://spventures.com.br/</t>
         </is>
       </c>
-      <c r="R100" t="inlineStr">
+      <c r="T100" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/sp-ventures</t>
         </is>
       </c>
-      <c r="S100" t="inlineStr">
+      <c r="U100" t="inlineStr">
         <is>
           <t>sp-ventures-2026.png</t>
         </is>
       </c>
-      <c r="T100" t="inlineStr"/>
-      <c r="U100" t="inlineStr"/>
       <c r="V100" t="inlineStr"/>
       <c r="W100" t="inlineStr"/>
       <c r="X100" t="inlineStr"/>
       <c r="Y100" t="inlineStr"/>
       <c r="Z100" t="inlineStr"/>
+      <c r="AA100" t="inlineStr"/>
+      <c r="AB100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
@@ -7764,28 +8123,30 @@
           <t>Ativa</t>
         </is>
       </c>
-      <c r="Q101" t="inlineStr">
+      <c r="Q101" s="5" t="inlineStr"/>
+      <c r="R101" s="5" t="inlineStr"/>
+      <c r="S101" t="inlineStr">
         <is>
           <t>https://setyou.com.br/</t>
         </is>
       </c>
-      <c r="R101" t="inlineStr">
+      <c r="T101" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/set-you</t>
         </is>
       </c>
-      <c r="S101" t="inlineStr">
+      <c r="U101" t="inlineStr">
         <is>
           <t>setyou.png</t>
         </is>
       </c>
-      <c r="T101" t="inlineStr"/>
-      <c r="U101" t="inlineStr"/>
       <c r="V101" t="inlineStr"/>
       <c r="W101" t="inlineStr"/>
       <c r="X101" t="inlineStr"/>
       <c r="Y101" t="inlineStr"/>
       <c r="Z101" t="inlineStr"/>
+      <c r="AA101" t="inlineStr"/>
+      <c r="AB101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
@@ -7831,24 +8192,30 @@
           <t>Saída</t>
         </is>
       </c>
-      <c r="Q102" t="inlineStr"/>
-      <c r="R102" t="inlineStr">
+      <c r="Q102" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R102" s="5" t="inlineStr"/>
+      <c r="S102" t="inlineStr"/>
+      <c r="T102" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/viajanet</t>
         </is>
       </c>
-      <c r="S102" t="inlineStr">
+      <c r="U102" t="inlineStr">
         <is>
           <t>viajanet.png</t>
         </is>
       </c>
-      <c r="T102" t="inlineStr"/>
-      <c r="U102" t="inlineStr"/>
       <c r="V102" t="inlineStr"/>
       <c r="W102" t="inlineStr"/>
       <c r="X102" t="inlineStr"/>
       <c r="Y102" t="inlineStr"/>
       <c r="Z102" t="inlineStr"/>
+      <c r="AA102" t="inlineStr"/>
+      <c r="AB102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
@@ -7890,28 +8257,30 @@
         </is>
       </c>
       <c r="P103" t="inlineStr"/>
-      <c r="Q103" t="inlineStr">
+      <c r="Q103" s="5" t="inlineStr"/>
+      <c r="R103" s="5" t="inlineStr"/>
+      <c r="S103" t="inlineStr">
         <is>
           <t>https://www.ceneo.pl/</t>
         </is>
       </c>
-      <c r="R103" t="inlineStr">
+      <c r="T103" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/ceneo</t>
         </is>
       </c>
-      <c r="S103" t="inlineStr">
+      <c r="U103" t="inlineStr">
         <is>
           <t>ceneo.png</t>
         </is>
       </c>
-      <c r="T103" t="inlineStr"/>
-      <c r="U103" t="inlineStr"/>
       <c r="V103" t="inlineStr"/>
       <c r="W103" t="inlineStr"/>
       <c r="X103" t="inlineStr"/>
       <c r="Y103" t="inlineStr"/>
       <c r="Z103" t="inlineStr"/>
+      <c r="AA103" t="inlineStr"/>
+      <c r="AB103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
@@ -7953,20 +8322,22 @@
         </is>
       </c>
       <c r="P104" t="inlineStr"/>
-      <c r="Q104" t="inlineStr"/>
-      <c r="R104" t="inlineStr"/>
-      <c r="S104" t="inlineStr">
+      <c r="Q104" s="5" t="inlineStr"/>
+      <c r="R104" s="5" t="inlineStr"/>
+      <c r="S104" t="inlineStr"/>
+      <c r="T104" t="inlineStr"/>
+      <c r="U104" t="inlineStr">
         <is>
           <t>compari.png</t>
         </is>
       </c>
-      <c r="T104" t="inlineStr"/>
-      <c r="U104" t="inlineStr"/>
       <c r="V104" t="inlineStr"/>
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr"/>
       <c r="Y104" t="inlineStr"/>
       <c r="Z104" t="inlineStr"/>
+      <c r="AA104" t="inlineStr"/>
+      <c r="AB104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
@@ -8008,20 +8379,22 @@
         </is>
       </c>
       <c r="P105" t="inlineStr"/>
-      <c r="Q105" t="inlineStr"/>
-      <c r="R105" t="inlineStr">
+      <c r="Q105" s="5" t="inlineStr"/>
+      <c r="R105" s="5" t="inlineStr"/>
+      <c r="S105" t="inlineStr"/>
+      <c r="T105" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/drezzy</t>
         </is>
       </c>
-      <c r="S105" t="inlineStr"/>
-      <c r="T105" t="inlineStr"/>
       <c r="U105" t="inlineStr"/>
       <c r="V105" t="inlineStr"/>
       <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr"/>
       <c r="Y105" t="inlineStr"/>
       <c r="Z105" t="inlineStr"/>
+      <c r="AA105" t="inlineStr"/>
+      <c r="AB105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
@@ -8063,24 +8436,26 @@
         </is>
       </c>
       <c r="P106" t="inlineStr"/>
-      <c r="Q106" t="inlineStr"/>
-      <c r="R106" t="inlineStr">
+      <c r="Q106" s="5" t="inlineStr"/>
+      <c r="R106" s="5" t="inlineStr"/>
+      <c r="S106" t="inlineStr"/>
+      <c r="T106" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/heureka-group</t>
         </is>
       </c>
-      <c r="S106" t="inlineStr">
+      <c r="U106" t="inlineStr">
         <is>
           <t>heureka.png</t>
         </is>
       </c>
-      <c r="T106" t="inlineStr"/>
-      <c r="U106" t="inlineStr"/>
       <c r="V106" t="inlineStr"/>
       <c r="W106" t="inlineStr"/>
       <c r="X106" t="inlineStr"/>
       <c r="Y106" t="inlineStr"/>
       <c r="Z106" t="inlineStr"/>
+      <c r="AA106" t="inlineStr"/>
+      <c r="AB106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
@@ -8122,24 +8497,26 @@
         </is>
       </c>
       <c r="P107" t="inlineStr"/>
-      <c r="Q107" t="inlineStr">
+      <c r="Q107" s="5" t="inlineStr"/>
+      <c r="R107" s="5" t="inlineStr"/>
+      <c r="S107" t="inlineStr">
         <is>
           <t>https://www.misshobby.com/it</t>
         </is>
       </c>
-      <c r="R107" t="inlineStr"/>
-      <c r="S107" t="inlineStr">
+      <c r="T107" t="inlineStr"/>
+      <c r="U107" t="inlineStr">
         <is>
           <t>misshobby.png</t>
         </is>
       </c>
-      <c r="T107" t="inlineStr"/>
-      <c r="U107" t="inlineStr"/>
       <c r="V107" t="inlineStr"/>
       <c r="W107" t="inlineStr"/>
       <c r="X107" t="inlineStr"/>
       <c r="Y107" t="inlineStr"/>
       <c r="Z107" t="inlineStr"/>
+      <c r="AA107" t="inlineStr"/>
+      <c r="AB107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
@@ -8181,20 +8558,22 @@
         </is>
       </c>
       <c r="P108" t="inlineStr"/>
-      <c r="Q108" t="inlineStr"/>
-      <c r="R108" t="inlineStr"/>
-      <c r="S108" t="inlineStr">
+      <c r="Q108" s="5" t="inlineStr"/>
+      <c r="R108" s="5" t="inlineStr"/>
+      <c r="S108" t="inlineStr"/>
+      <c r="T108" t="inlineStr"/>
+      <c r="U108" t="inlineStr">
         <is>
           <t>pazaruvaj.png</t>
         </is>
       </c>
-      <c r="T108" t="inlineStr"/>
-      <c r="U108" t="inlineStr"/>
       <c r="V108" t="inlineStr"/>
       <c r="W108" t="inlineStr"/>
       <c r="X108" t="inlineStr"/>
       <c r="Y108" t="inlineStr"/>
       <c r="Z108" t="inlineStr"/>
+      <c r="AA108" t="inlineStr"/>
+      <c r="AB108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
@@ -8236,24 +8615,26 @@
         </is>
       </c>
       <c r="P109" t="inlineStr"/>
-      <c r="Q109" t="inlineStr"/>
-      <c r="R109" t="inlineStr">
+      <c r="Q109" s="5" t="inlineStr"/>
+      <c r="R109" s="5" t="inlineStr"/>
+      <c r="S109" t="inlineStr"/>
+      <c r="T109" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/pricecheck</t>
         </is>
       </c>
-      <c r="S109" t="inlineStr">
+      <c r="U109" t="inlineStr">
         <is>
           <t>pricecheck.png</t>
         </is>
       </c>
-      <c r="T109" t="inlineStr"/>
-      <c r="U109" t="inlineStr"/>
       <c r="V109" t="inlineStr"/>
       <c r="W109" t="inlineStr"/>
       <c r="X109" t="inlineStr"/>
       <c r="Y109" t="inlineStr"/>
       <c r="Z109" t="inlineStr"/>
+      <c r="AA109" t="inlineStr"/>
+      <c r="AB109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
@@ -8295,28 +8676,30 @@
         </is>
       </c>
       <c r="P110" t="inlineStr"/>
-      <c r="Q110" t="inlineStr">
+      <c r="Q110" s="5" t="inlineStr"/>
+      <c r="R110" s="5" t="inlineStr"/>
+      <c r="S110" t="inlineStr">
         <is>
           <t>https://www.shoppydoo.it/</t>
         </is>
       </c>
-      <c r="R110" t="inlineStr">
+      <c r="T110" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/shoppydoo</t>
         </is>
       </c>
-      <c r="S110" t="inlineStr">
+      <c r="U110" t="inlineStr">
         <is>
           <t>shoppydoo.png</t>
         </is>
       </c>
-      <c r="T110" t="inlineStr"/>
-      <c r="U110" t="inlineStr"/>
       <c r="V110" t="inlineStr"/>
       <c r="W110" t="inlineStr"/>
       <c r="X110" t="inlineStr"/>
       <c r="Y110" t="inlineStr"/>
       <c r="Z110" t="inlineStr"/>
+      <c r="AA110" t="inlineStr"/>
+      <c r="AB110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
@@ -8358,24 +8741,26 @@
         </is>
       </c>
       <c r="P111" t="inlineStr"/>
-      <c r="Q111" t="inlineStr"/>
-      <c r="R111" t="inlineStr">
+      <c r="Q111" s="5" t="inlineStr"/>
+      <c r="R111" s="5" t="inlineStr"/>
+      <c r="S111" t="inlineStr"/>
+      <c r="T111" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/trovaprezzi-it-d087</t>
         </is>
       </c>
-      <c r="S111" t="inlineStr">
+      <c r="U111" t="inlineStr">
         <is>
           <t>trovaprezzi.png</t>
         </is>
       </c>
-      <c r="T111" t="inlineStr"/>
-      <c r="U111" t="inlineStr"/>
       <c r="V111" t="inlineStr"/>
       <c r="W111" t="inlineStr"/>
       <c r="X111" t="inlineStr"/>
       <c r="Y111" t="inlineStr"/>
       <c r="Z111" t="inlineStr"/>
+      <c r="AA111" t="inlineStr"/>
+      <c r="AB111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
@@ -8417,8 +8802,8 @@
         </is>
       </c>
       <c r="P112" t="inlineStr"/>
-      <c r="Q112" t="inlineStr"/>
-      <c r="R112" t="inlineStr"/>
+      <c r="Q112" s="5" t="inlineStr"/>
+      <c r="R112" s="5" t="inlineStr"/>
       <c r="S112" t="inlineStr"/>
       <c r="T112" t="inlineStr"/>
       <c r="U112" t="inlineStr"/>
@@ -8427,6 +8812,8 @@
       <c r="X112" t="inlineStr"/>
       <c r="Y112" t="inlineStr"/>
       <c r="Z112" t="inlineStr"/>
+      <c r="AA112" t="inlineStr"/>
+      <c r="AB112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
@@ -8468,20 +8855,22 @@
         </is>
       </c>
       <c r="P113" t="inlineStr"/>
-      <c r="Q113" t="inlineStr"/>
-      <c r="R113" t="inlineStr">
+      <c r="Q113" s="5" t="inlineStr"/>
+      <c r="R113" s="5" t="inlineStr"/>
+      <c r="S113" t="inlineStr"/>
+      <c r="T113" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/vcene</t>
         </is>
       </c>
-      <c r="S113" t="inlineStr"/>
-      <c r="T113" t="inlineStr"/>
       <c r="U113" t="inlineStr"/>
       <c r="V113" t="inlineStr"/>
       <c r="W113" t="inlineStr"/>
       <c r="X113" t="inlineStr"/>
       <c r="Y113" t="inlineStr"/>
       <c r="Z113" t="inlineStr"/>
+      <c r="AA113" t="inlineStr"/>
+      <c r="AB113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
@@ -8523,24 +8912,26 @@
         </is>
       </c>
       <c r="P114" t="inlineStr"/>
-      <c r="Q114" t="inlineStr"/>
-      <c r="R114" t="inlineStr">
+      <c r="Q114" s="5" t="inlineStr"/>
+      <c r="R114" s="5" t="inlineStr"/>
+      <c r="S114" t="inlineStr"/>
+      <c r="T114" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/%C3%A1rukeres%C5%91</t>
         </is>
       </c>
-      <c r="S114" t="inlineStr">
+      <c r="U114" t="inlineStr">
         <is>
           <t>arukereso.png</t>
         </is>
       </c>
-      <c r="T114" t="inlineStr"/>
-      <c r="U114" t="inlineStr"/>
       <c r="V114" t="inlineStr"/>
       <c r="W114" t="inlineStr"/>
       <c r="X114" t="inlineStr"/>
       <c r="Y114" t="inlineStr"/>
       <c r="Z114" t="inlineStr"/>
+      <c r="AA114" t="inlineStr"/>
+      <c r="AB114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
@@ -8582,8 +8973,8 @@
         </is>
       </c>
       <c r="P115" t="inlineStr"/>
-      <c r="Q115" t="inlineStr"/>
-      <c r="R115" t="inlineStr"/>
+      <c r="Q115" s="5" t="inlineStr"/>
+      <c r="R115" s="5" t="inlineStr"/>
       <c r="S115" t="inlineStr"/>
       <c r="T115" t="inlineStr"/>
       <c r="U115" t="inlineStr"/>
@@ -8592,6 +8983,8 @@
       <c r="X115" t="inlineStr"/>
       <c r="Y115" t="inlineStr"/>
       <c r="Z115" t="inlineStr"/>
+      <c r="AA115" t="inlineStr"/>
+      <c r="AB115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
@@ -8637,24 +9030,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q116" t="inlineStr"/>
-      <c r="R116" t="inlineStr">
+      <c r="Q116" s="5" t="inlineStr"/>
+      <c r="R116" s="5" t="inlineStr"/>
+      <c r="S116" t="inlineStr"/>
+      <c r="T116" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/curupira</t>
         </is>
       </c>
-      <c r="S116" t="inlineStr">
+      <c r="U116" t="inlineStr">
         <is>
           <t>curupira.png</t>
         </is>
       </c>
-      <c r="T116" t="inlineStr"/>
-      <c r="U116" t="inlineStr"/>
       <c r="V116" t="inlineStr"/>
       <c r="W116" t="inlineStr"/>
       <c r="X116" t="inlineStr"/>
       <c r="Y116" t="inlineStr"/>
       <c r="Z116" t="inlineStr"/>
+      <c r="AA116" t="inlineStr"/>
+      <c r="AB116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
@@ -8700,20 +9095,22 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q117" t="inlineStr"/>
-      <c r="R117" t="inlineStr"/>
-      <c r="S117" t="inlineStr">
+      <c r="Q117" s="5" t="inlineStr"/>
+      <c r="R117" s="5" t="inlineStr"/>
+      <c r="S117" t="inlineStr"/>
+      <c r="T117" t="inlineStr"/>
+      <c r="U117" t="inlineStr">
         <is>
           <t>cybercook.png</t>
         </is>
       </c>
-      <c r="T117" t="inlineStr"/>
-      <c r="U117" t="inlineStr"/>
       <c r="V117" t="inlineStr"/>
       <c r="W117" t="inlineStr"/>
       <c r="X117" t="inlineStr"/>
       <c r="Y117" t="inlineStr"/>
       <c r="Z117" t="inlineStr"/>
+      <c r="AA117" t="inlineStr"/>
+      <c r="AB117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
@@ -8759,20 +9156,22 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q118" t="inlineStr"/>
-      <c r="R118" t="inlineStr"/>
-      <c r="S118" t="inlineStr">
+      <c r="Q118" s="5" t="inlineStr"/>
+      <c r="R118" s="5" t="inlineStr"/>
+      <c r="S118" t="inlineStr"/>
+      <c r="T118" t="inlineStr"/>
+      <c r="U118" t="inlineStr">
         <is>
           <t>loteria-brasil.png</t>
         </is>
       </c>
-      <c r="T118" t="inlineStr"/>
-      <c r="U118" t="inlineStr"/>
       <c r="V118" t="inlineStr"/>
       <c r="W118" t="inlineStr"/>
       <c r="X118" t="inlineStr"/>
       <c r="Y118" t="inlineStr"/>
       <c r="Z118" t="inlineStr"/>
+      <c r="AA118" t="inlineStr"/>
+      <c r="AB118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
@@ -8818,20 +9217,22 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q119" t="inlineStr"/>
-      <c r="R119" t="inlineStr">
+      <c r="Q119" s="5" t="inlineStr"/>
+      <c r="R119" s="5" t="inlineStr"/>
+      <c r="S119" t="inlineStr"/>
+      <c r="T119" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/ehub</t>
         </is>
       </c>
-      <c r="S119" t="inlineStr"/>
-      <c r="T119" t="inlineStr"/>
       <c r="U119" t="inlineStr"/>
       <c r="V119" t="inlineStr"/>
       <c r="W119" t="inlineStr"/>
       <c r="X119" t="inlineStr"/>
       <c r="Y119" t="inlineStr"/>
       <c r="Z119" t="inlineStr"/>
+      <c r="AA119" t="inlineStr"/>
+      <c r="AB119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
@@ -8873,20 +9274,22 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q120" t="inlineStr"/>
-      <c r="R120" t="inlineStr">
+      <c r="Q120" s="5" t="inlineStr"/>
+      <c r="R120" s="5" t="inlineStr"/>
+      <c r="S120" t="inlineStr"/>
+      <c r="T120" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/contapaga</t>
         </is>
       </c>
-      <c r="S120" t="inlineStr"/>
-      <c r="T120" t="inlineStr"/>
       <c r="U120" t="inlineStr"/>
       <c r="V120" t="inlineStr"/>
       <c r="W120" t="inlineStr"/>
       <c r="X120" t="inlineStr"/>
       <c r="Y120" t="inlineStr"/>
       <c r="Z120" t="inlineStr"/>
+      <c r="AA120" t="inlineStr"/>
+      <c r="AB120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
@@ -8928,8 +9331,8 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q121" t="inlineStr"/>
-      <c r="R121" t="inlineStr"/>
+      <c r="Q121" s="5" t="inlineStr"/>
+      <c r="R121" s="5" t="inlineStr"/>
       <c r="S121" t="inlineStr"/>
       <c r="T121" t="inlineStr"/>
       <c r="U121" t="inlineStr"/>
@@ -8938,6 +9341,8 @@
       <c r="X121" t="inlineStr"/>
       <c r="Y121" t="inlineStr"/>
       <c r="Z121" t="inlineStr"/>
+      <c r="AA121" t="inlineStr"/>
+      <c r="AB121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
@@ -8979,24 +9384,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q122" t="inlineStr">
+      <c r="Q122" s="5" t="inlineStr"/>
+      <c r="R122" s="5" t="inlineStr"/>
+      <c r="S122" t="inlineStr">
         <is>
           <t>https://jet8.io/</t>
         </is>
       </c>
-      <c r="R122" t="inlineStr"/>
-      <c r="S122" t="inlineStr">
+      <c r="T122" t="inlineStr"/>
+      <c r="U122" t="inlineStr">
         <is>
           <t>jet8-2026.png</t>
         </is>
       </c>
-      <c r="T122" t="inlineStr"/>
-      <c r="U122" t="inlineStr"/>
       <c r="V122" t="inlineStr"/>
       <c r="W122" t="inlineStr"/>
       <c r="X122" t="inlineStr"/>
       <c r="Y122" t="inlineStr"/>
       <c r="Z122" t="inlineStr"/>
+      <c r="AA122" t="inlineStr"/>
+      <c r="AB122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
@@ -9038,24 +9445,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q123" t="inlineStr">
+      <c r="Q123" s="5" t="inlineStr"/>
+      <c r="R123" s="5" t="inlineStr"/>
+      <c r="S123" t="inlineStr">
         <is>
           <t>https://roomorama.com/</t>
         </is>
       </c>
-      <c r="R123" t="inlineStr">
+      <c r="T123" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/roomorama; https://www.crunchbase.com/organization/lofty-ai</t>
         </is>
       </c>
-      <c r="S123" t="inlineStr"/>
-      <c r="T123" t="inlineStr"/>
       <c r="U123" t="inlineStr"/>
       <c r="V123" t="inlineStr"/>
       <c r="W123" t="inlineStr"/>
       <c r="X123" t="inlineStr"/>
       <c r="Y123" t="inlineStr"/>
       <c r="Z123" t="inlineStr"/>
+      <c r="AA123" t="inlineStr"/>
+      <c r="AB123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
@@ -9097,24 +9506,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q124" t="inlineStr"/>
-      <c r="R124" t="inlineStr">
+      <c r="Q124" s="5" t="inlineStr"/>
+      <c r="R124" s="5" t="inlineStr"/>
+      <c r="S124" t="inlineStr"/>
+      <c r="T124" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/lulu-2</t>
         </is>
       </c>
-      <c r="S124" t="inlineStr">
+      <c r="U124" t="inlineStr">
         <is>
           <t>lulu-app.png</t>
         </is>
       </c>
-      <c r="T124" t="inlineStr"/>
-      <c r="U124" t="inlineStr"/>
       <c r="V124" t="inlineStr"/>
       <c r="W124" t="inlineStr"/>
       <c r="X124" t="inlineStr"/>
       <c r="Y124" t="inlineStr"/>
       <c r="Z124" t="inlineStr"/>
+      <c r="AA124" t="inlineStr"/>
+      <c r="AB124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
@@ -9156,24 +9567,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q125" t="inlineStr"/>
-      <c r="R125" t="inlineStr">
+      <c r="Q125" s="5" t="inlineStr"/>
+      <c r="R125" s="5" t="inlineStr"/>
+      <c r="S125" t="inlineStr"/>
+      <c r="T125" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/contapaga</t>
         </is>
       </c>
-      <c r="S125" t="inlineStr">
+      <c r="U125" t="inlineStr">
         <is>
           <t>moneto.png</t>
         </is>
       </c>
-      <c r="T125" t="inlineStr"/>
-      <c r="U125" t="inlineStr"/>
       <c r="V125" t="inlineStr"/>
       <c r="W125" t="inlineStr"/>
       <c r="X125" t="inlineStr"/>
       <c r="Y125" t="inlineStr"/>
       <c r="Z125" t="inlineStr"/>
+      <c r="AA125" t="inlineStr"/>
+      <c r="AB125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
@@ -9215,24 +9628,26 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q126" t="inlineStr"/>
-      <c r="R126" t="inlineStr">
+      <c r="Q126" s="5" t="inlineStr"/>
+      <c r="R126" s="5" t="inlineStr"/>
+      <c r="S126" t="inlineStr"/>
+      <c r="T126" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/orderin</t>
         </is>
       </c>
-      <c r="S126" t="inlineStr">
+      <c r="U126" t="inlineStr">
         <is>
           <t>orderin-2026.png</t>
         </is>
       </c>
-      <c r="T126" t="inlineStr"/>
-      <c r="U126" t="inlineStr"/>
       <c r="V126" t="inlineStr"/>
       <c r="W126" t="inlineStr"/>
       <c r="X126" t="inlineStr"/>
       <c r="Y126" t="inlineStr"/>
       <c r="Z126" t="inlineStr"/>
+      <c r="AA126" t="inlineStr"/>
+      <c r="AB126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
@@ -9278,24 +9693,30 @@
           <t>Saída · 2015</t>
         </is>
       </c>
-      <c r="Q127" t="inlineStr"/>
-      <c r="R127" t="inlineStr">
+      <c r="Q127" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="R127" s="5" t="inlineStr"/>
+      <c r="S127" t="inlineStr"/>
+      <c r="T127" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/scup</t>
         </is>
       </c>
-      <c r="S127" t="inlineStr">
+      <c r="U127" t="inlineStr">
         <is>
           <t>scup-2026.png</t>
         </is>
       </c>
-      <c r="T127" t="inlineStr"/>
-      <c r="U127" t="inlineStr"/>
       <c r="V127" t="inlineStr"/>
       <c r="W127" t="inlineStr"/>
       <c r="X127" t="inlineStr"/>
       <c r="Y127" t="inlineStr"/>
       <c r="Z127" t="inlineStr"/>
+      <c r="AA127" t="inlineStr"/>
+      <c r="AB127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
@@ -9337,28 +9758,30 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q128" t="inlineStr">
+      <c r="Q128" s="5" t="inlineStr"/>
+      <c r="R128" s="5" t="inlineStr"/>
+      <c r="S128" t="inlineStr">
         <is>
           <t>https://shoes4you.com.br/</t>
         </is>
       </c>
-      <c r="R128" t="inlineStr">
+      <c r="T128" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/shoes4you</t>
         </is>
       </c>
-      <c r="S128" t="inlineStr">
+      <c r="U128" t="inlineStr">
         <is>
           <t>shoes4you.png</t>
         </is>
       </c>
-      <c r="T128" t="inlineStr"/>
-      <c r="U128" t="inlineStr"/>
       <c r="V128" t="inlineStr"/>
       <c r="W128" t="inlineStr"/>
       <c r="X128" t="inlineStr"/>
       <c r="Y128" t="inlineStr"/>
       <c r="Z128" t="inlineStr"/>
+      <c r="AA128" t="inlineStr"/>
+      <c r="AB128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
@@ -9400,20 +9823,22 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q129" t="inlineStr"/>
-      <c r="R129" t="inlineStr">
+      <c r="Q129" s="5" t="inlineStr"/>
+      <c r="R129" s="5" t="inlineStr"/>
+      <c r="S129" t="inlineStr"/>
+      <c r="T129" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/sigaseutime</t>
         </is>
       </c>
-      <c r="S129" t="inlineStr"/>
-      <c r="T129" t="inlineStr"/>
       <c r="U129" t="inlineStr"/>
       <c r="V129" t="inlineStr"/>
       <c r="W129" t="inlineStr"/>
       <c r="X129" t="inlineStr"/>
       <c r="Y129" t="inlineStr"/>
       <c r="Z129" t="inlineStr"/>
+      <c r="AA129" t="inlineStr"/>
+      <c r="AB129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
@@ -9455,29 +9880,31 @@
           <t>Encerrada</t>
         </is>
       </c>
-      <c r="Q130" t="inlineStr"/>
-      <c r="R130" t="inlineStr">
+      <c r="Q130" s="5" t="inlineStr"/>
+      <c r="R130" s="5" t="inlineStr"/>
+      <c r="S130" t="inlineStr"/>
+      <c r="T130" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/youhotel</t>
         </is>
       </c>
-      <c r="S130" t="inlineStr">
+      <c r="U130" t="inlineStr">
         <is>
           <t>youhotel.png</t>
         </is>
       </c>
-      <c r="T130" t="inlineStr"/>
-      <c r="U130" t="inlineStr"/>
       <c r="V130" t="inlineStr"/>
       <c r="W130" t="inlineStr"/>
       <c r="X130" t="inlineStr"/>
       <c r="Y130" t="inlineStr"/>
       <c r="Z130" t="inlineStr"/>
+      <c r="AA130" t="inlineStr"/>
+      <c r="AB130" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z130"/>
+  <autoFilter ref="A1:AB130"/>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B2000 F2:F2000 G2:G2000 H2:H2000 I2:I2000 J2:J2000 K2:K2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use x para marcar ou deixe vazio." type="list">
+    <dataValidation sqref="B2:B2000 F2:F2000 G2:G2000 H2:H2000 I2:I2000 J2:J2000 K2:K2000 Q2:Q2000 R2:R2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use x para marcar ou deixe vazio." type="list">
       <formula1>"x"</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
feat(portfolio): matérias de 14 investidas da Headline
Datamint, Vixtra, Fin-X, Fiibo, Horuss, Trinus, Upik (Arquiteto de Bolso),
PipeImob, Neurogram, Vaas, Avenia, Alia.do, Blips e Hero Seguros. Links do
Romero; título como o veículo publicou e fonte · data conferidos em cada
página (a empresa de quatro peças sem nome no link identificada pelo texto).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -2708,9 +2708,21 @@
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>https://braziljournal.com/headline-avalia-a-blips-em-r-500-milhoes/</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>Headline avalia a Blips em R$ 500 milhões</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Brazil Journal · mai 2025</t>
+        </is>
+      </c>
       <c r="AB22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -2777,9 +2789,21 @@
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>https://braziljournal.com/swift-killer-a-rodada-da-avenia-a-emissora-da-maior-stablecoin-em-real/</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>‘SWIFT killer’. A rodada da Avenia, a emissora da maior stablecoin em real</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>Brazil Journal · fev 2026</t>
+        </is>
+      </c>
       <c r="AB23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -2846,9 +2870,21 @@
       <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>https://braziljournal.com/sujeira-no-painel-mato-ao-redor-a-datamint-tem-uma-ai-que-apita/</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>Sujeira no painel? Mato ao redor? A DataMint tem uma AI que apita</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>Brazil Journal · jun 2026</t>
+        </is>
+      </c>
       <c r="AB24" t="inlineStr">
         <is>
           <t>Headline: Series A de jun 2026 (Crunchbase).</t>
@@ -2919,9 +2955,21 @@
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>https://pipelinevalor.globo.com/negocios/noticia/vixtra-capta-r-45-milhoes-para-ampliar-trade-finance.ghtml</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>Vixtra capta R$ 45 milhões para ampliar trade finance</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Pipeline Valor · jun 2026</t>
+        </is>
+      </c>
       <c r="AB25" t="inlineStr">
         <is>
           <t>Headline: Series A de jun 2026 (Crunchbase). Logo original é branco; convertido para escuro.</t>
@@ -3061,9 +3109,21 @@
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>https://braziljournal.com/a-rodada-da-hero-que-quer-transformar-o-seguro-viagem/</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>A rodada da Hero, que quer transformar o seguro viagem</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Brazil Journal · mar 2026</t>
+        </is>
+      </c>
       <c r="AB27" t="inlineStr"/>
     </row>
     <row r="28">
@@ -3199,9 +3259,21 @@
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="inlineStr"/>
-      <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>https://forbes.com.br/escolhas-do-editor/2025/08/aos-21-anos-ela-criou-uma-startup-que-ja-captou-r-23-milhoes/</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>Aos 21 Anos, Ela Criou uma Startup Que Já Captou R$ 23 Milhões</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Forbes Brasil · ago 2025</t>
+        </is>
+      </c>
       <c r="AB29" t="inlineStr"/>
     </row>
     <row r="30">
@@ -3337,9 +3409,21 @@
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
-      <c r="Z31" t="inlineStr"/>
-      <c r="AA31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>https://neofeed.com.br/startups/esse-trio-vendeu-sua-primeira-startup-por-us-100-milhoes-agora-quer-prevenir-fraudes/</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>Esse trio vendeu sua primeira startup por US$ 100 milhões. Agora, quer prevenir fraudes</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>NeoFeed · ago 2025</t>
+        </is>
+      </c>
       <c r="AB31" t="inlineStr"/>
     </row>
     <row r="32">
@@ -3747,9 +3831,21 @@
       <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr"/>
       <c r="X37" t="inlineStr"/>
-      <c r="Y37" t="inlineStr"/>
-      <c r="Z37" t="inlineStr"/>
-      <c r="AA37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>https://exame.com/negocios/startup-de-ia-que-ouve-vendedores-em-lojas-fisicas-levanta-r-13-milhoes/</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>Startup de IA que ‘ouve’ vendedores em lojas físicas levanta R$ 13 milhões</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>Exame · jan 2026</t>
+        </is>
+      </c>
       <c r="AB37" t="inlineStr"/>
     </row>
     <row r="38">
@@ -4019,9 +4115,21 @@
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr"/>
       <c r="X41" t="inlineStr"/>
-      <c r="Y41" t="inlineStr"/>
-      <c r="Z41" t="inlineStr"/>
-      <c r="AA41" t="inlineStr"/>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>https://neofeed.com.br/startups/ele-vendeu-o-zap-a-suahouse-e-a-kzas-e-agora-atraiu-um-cheque-da-headline-para-sua-nova-startup/</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Ele vendeu o ZAP, a SuaHouse e a Kzas. E, agora, atraiu um cheque da Headline para sua nova startup</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>NeoFeed · ago 2025</t>
+        </is>
+      </c>
       <c r="AB41" t="inlineStr"/>
     </row>
     <row r="42">
@@ -4088,9 +4196,21 @@
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="inlineStr"/>
       <c r="X42" t="inlineStr"/>
-      <c r="Y42" t="inlineStr"/>
-      <c r="Z42" t="inlineStr"/>
-      <c r="AA42" t="inlineStr"/>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>https://braziljournal.com/a-horuss-ai-quer-levar-eficiencia-aos-planos-de-saude-com-dados-e-machine-learning/</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>A Horuss AI quer levar eficiência aos planos de saúde (com dados e machine learning)</t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>Brazil Journal · set 2024</t>
+        </is>
+      </c>
       <c r="AB42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -4291,9 +4411,21 @@
       <c r="V45" t="inlineStr"/>
       <c r="W45" t="inlineStr"/>
       <c r="X45" t="inlineStr"/>
-      <c r="Y45" t="inlineStr"/>
-      <c r="Z45" t="inlineStr"/>
-      <c r="AA45" t="inlineStr"/>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>https://pipelinevalor.globo.com/startups/noticia/marketplace-de-saude-fiibo-atrai-headline-brasil-e-fundo-do-einstein.ghtml</t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>Marketplace de saúde, Fiibo atrai Headline Brasil e fundo do Einstein</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>Pipeline Valor · ago 2023</t>
+        </is>
+      </c>
       <c r="AB45" t="inlineStr"/>
     </row>
     <row r="46">
@@ -4356,9 +4488,21 @@
       <c r="V46" t="inlineStr"/>
       <c r="W46" t="inlineStr"/>
       <c r="X46" t="inlineStr"/>
-      <c r="Y46" t="inlineStr"/>
-      <c r="Z46" t="inlineStr"/>
-      <c r="AA46" t="inlineStr"/>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>https://www.infomoney.com.br/negocios/fundo-headline-xp-mira-na-saude-e-investe-r-78-mi-na-healtech-fin-x/</t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>Fundo Headline XP mira na saúde e investe R$ 7,8 mi na healtech Fin-X</t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>InfoMoney · mar 2023</t>
+        </is>
+      </c>
       <c r="AB46" t="inlineStr"/>
     </row>
     <row r="47">
@@ -4563,9 +4707,21 @@
       <c r="V49" t="inlineStr"/>
       <c r="W49" t="inlineStr"/>
       <c r="X49" t="inlineStr"/>
-      <c r="Y49" t="inlineStr"/>
-      <c r="Z49" t="inlineStr"/>
-      <c r="AA49" t="inlineStr"/>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>https://valor.globo.com/financas/noticia/2023/12/15/headline-lidera-rodada-na-trinus-de-ate-r-70-milhoes.ghtml</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>Headline, de Romero Rodrigues, lidera rodada na Trinus de até R$ 70 milhões</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>Valor · dez 2023</t>
+        </is>
+      </c>
       <c r="AB49" t="inlineStr"/>
     </row>
     <row r="50">
@@ -4628,9 +4784,21 @@
       <c r="V50" t="inlineStr"/>
       <c r="W50" t="inlineStr"/>
       <c r="X50" t="inlineStr"/>
-      <c r="Y50" t="inlineStr"/>
-      <c r="Z50" t="inlineStr"/>
-      <c r="AA50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>https://imoveis.estadao.com.br/noticias/startup-arquiteto-de-bolso-recebe-aporte-de-r-15-milhoes-para-desenvolver-novos-produtos/</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>Startup Arquiteto de Bolso recebe aporte de R$ 15 milhões para desenvolver novos produtos</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>Estadão · mar 2024</t>
+        </is>
+      </c>
       <c r="AB50" t="inlineStr"/>
     </row>
     <row r="51">

</xml_diff>

<commit_message>
feat(portfolio): matérias de Mercado de Recebíveis, Turn2C, Revert, Celero, Doc9 e Mission Brasil
Links do Romero; título como o veículo publicou e data conferidos em cada
página. Duas peças sem a empresa no link identificadas pelo texto
(Mercado de Recebíveis e Doc9).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -3190,9 +3190,21 @@
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>https://neofeed.com.br/startups/a-fintech-multiplicou-seu-valor-por-quatro-em-menos-de-dois-anos-e-ja-vale-r-300-milhoes/</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>A fintech que multiplicou seu valor por quatro em menos de dois anos. E já vale R$ 300 milhões</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>NeoFeed · ago 2025</t>
+        </is>
+      </c>
       <c r="AB28" t="inlineStr"/>
     </row>
     <row r="29">
@@ -3762,9 +3774,21 @@
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="inlineStr"/>
       <c r="X36" t="inlineStr"/>
-      <c r="Y36" t="inlineStr"/>
-      <c r="Z36" t="inlineStr"/>
-      <c r="AA36" t="inlineStr"/>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>https://exame.com/insight/com-r-5-bilhoes-processados-revert-atrai-valor-capital-e-ja-mira-nova-rodada/p</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>Com R$ 5 bilhões processados, Revert atrai Valor Capital e já mira nova rodada</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>Exame · ago 2026</t>
+        </is>
+      </c>
       <c r="AB36" t="inlineStr"/>
     </row>
     <row r="37">
@@ -3912,9 +3936,21 @@
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr"/>
       <c r="X38" t="inlineStr"/>
-      <c r="Y38" t="inlineStr"/>
-      <c r="Z38" t="inlineStr"/>
-      <c r="AA38" t="inlineStr"/>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>https://neofeed.com.br/startups/o-que-visa-e-headline-viram-na-celero/</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>O que Visa e Headline viram na Celero</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>NeoFeed · mar 2026</t>
+        </is>
+      </c>
       <c r="AB38" t="inlineStr"/>
     </row>
     <row r="39">
@@ -3981,9 +4017,21 @@
       <c r="V39" t="inlineStr"/>
       <c r="W39" t="inlineStr"/>
       <c r="X39" t="inlineStr"/>
-      <c r="Y39" t="inlineStr"/>
-      <c r="Z39" t="inlineStr"/>
-      <c r="AA39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>https://neofeed.com.br/startups/headline-da-o-veredito-para-seu-13o-investimento/</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>Headline dá o "veredito" para seu 13º investimento</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>NeoFeed · abr 2025</t>
+        </is>
+      </c>
       <c r="AB39" t="inlineStr"/>
     </row>
     <row r="40">
@@ -4277,9 +4325,21 @@
       <c r="V43" t="inlineStr"/>
       <c r="W43" t="inlineStr"/>
       <c r="X43" t="inlineStr"/>
-      <c r="Y43" t="inlineStr"/>
-      <c r="Z43" t="inlineStr"/>
-      <c r="AA43" t="inlineStr"/>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>https://neofeed.com.br/startups/em-seu-setimo-cheque-headline-investe-em-fintech-de-consorcio-turn2c/</t>
+        </is>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>Em seu sétimo cheque, Headline investe em fintech de consórcio Turn2C</t>
+        </is>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>NeoFeed · mar 2024</t>
+        </is>
+      </c>
       <c r="AB43" t="inlineStr"/>
     </row>
     <row r="44">
@@ -4638,9 +4698,21 @@
       <c r="V48" t="inlineStr"/>
       <c r="W48" t="inlineStr"/>
       <c r="X48" t="inlineStr"/>
-      <c r="Y48" t="inlineStr"/>
-      <c r="Z48" t="inlineStr"/>
-      <c r="AA48" t="inlineStr"/>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>https://pipelinevalor.globo.com/startups/noticia/headline-e-domo-aumentam-aposta-na-gig-economy-com-mission-brasil.ghtml</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>Headline e Domo aumentam aposta na gig economy com Mission Brasil</t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>Pipeline Valor · dez 2025</t>
+        </is>
+      </c>
       <c r="AB48" t="inlineStr"/>
     </row>
     <row r="49">

</xml_diff>

<commit_message>
fix(seo): revisão final — sem XP na home em inglês, faixa de idioma sem deslocar a página, links mortos
- /en: o carrossel (desde a nova ordem da home) e o destaque de mídia (desde
  a seção Na mídia) mostravam a XP; saem por regras de remover no en.json.
- Faixa "This site is also available in English" fixa no rodapé da tela:
  inserida depois do carregamento, empurrava o conteúdo (CLS).
- GigU: site.stopclub.com.br com certificado quebrado; troca por gigu.co/br.
  Roomorama: site fora do ar (empresa encerrada); card fica sem link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -5290,7 +5290,7 @@
       <c r="R56" s="5" t="inlineStr"/>
       <c r="S56" t="inlineStr">
         <is>
-          <t>https://site.stopclub.com.br/</t>
+          <t>https://gigu.co/br</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -9833,11 +9833,7 @@
       </c>
       <c r="Q125" s="5" t="inlineStr"/>
       <c r="R125" s="5" t="inlineStr"/>
-      <c r="S125" t="inlineStr">
-        <is>
-          <t>https://roomorama.com/</t>
-        </is>
-      </c>
+      <c r="S125" t="inlineStr"/>
       <c r="T125" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/organization/roomorama; https://www.crunchbase.com/organization/lofty-ai</t>
@@ -9850,7 +9846,11 @@
       <c r="Y125" t="inlineStr"/>
       <c r="Z125" t="inlineStr"/>
       <c r="AA125" t="inlineStr"/>
-      <c r="AB125" t="inlineStr"/>
+      <c r="AB125" t="inlineStr">
+        <is>
+          <t>Site roomorama.com fora do ar (certificado inválido) em 28/09/2026; link tirado do card.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat(portfolio): Moneto e ContaPaga num card só; contagens dos filtros em inglês
- ContaPaga mudou de nome para Moneto: um card, "Moneto / ContaPaga", com o
  logo da Moneto e as relações dos dois. Portfólio passa a 128 empresas
  (127 em inglês); totais, descriptions, filtros e ItemList recalculados.
- Bug antigo: todos os filtros de /en/portfolio mostravam 0. A recontagem
  procurava <li data-cats=…>, mas desde 24/09 o card começa com id=…

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Empresas'!$A$1:$AB$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Empresas'!$A$1:$AB$131</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -753,7 +753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB132"/>
+  <dimension ref="A1:AB131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9623,7 +9623,7 @@
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>2060</t>
         </is>
       </c>
       <c r="B122" s="5" t="inlineStr">
@@ -9634,7 +9634,7 @@
       <c r="C122" s="5" t="inlineStr"/>
       <c r="D122" t="inlineStr">
         <is>
-          <t>ContaPaga</t>
+          <t>HospedeVIP</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -9663,11 +9663,7 @@
       <c r="Q122" s="5" t="inlineStr"/>
       <c r="R122" s="5" t="inlineStr"/>
       <c r="S122" t="inlineStr"/>
-      <c r="T122" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/contapaga</t>
-        </is>
-      </c>
+      <c r="T122" t="inlineStr"/>
       <c r="U122" t="inlineStr"/>
       <c r="V122" t="inlineStr"/>
       <c r="W122" t="inlineStr"/>
@@ -9680,7 +9676,7 @@
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>2060</t>
+          <t>2070</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
@@ -9691,7 +9687,7 @@
       <c r="C123" s="5" t="inlineStr"/>
       <c r="D123" t="inlineStr">
         <is>
-          <t>HospedeVIP</t>
+          <t>Jet8</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
@@ -9719,9 +9715,17 @@
       </c>
       <c r="Q123" s="5" t="inlineStr"/>
       <c r="R123" s="5" t="inlineStr"/>
-      <c r="S123" t="inlineStr"/>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>https://jet8.io/</t>
+        </is>
+      </c>
       <c r="T123" t="inlineStr"/>
-      <c r="U123" t="inlineStr"/>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>jet8-2026.png</t>
+        </is>
+      </c>
       <c r="V123" t="inlineStr"/>
       <c r="W123" t="inlineStr"/>
       <c r="X123" t="inlineStr"/>
@@ -9733,7 +9737,7 @@
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>2070</t>
+          <t>2080</t>
         </is>
       </c>
       <c r="B124" s="5" t="inlineStr">
@@ -9744,7 +9748,7 @@
       <c r="C124" s="5" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Jet8</t>
+          <t>LOFTY / ROOMORAMA</t>
         </is>
       </c>
       <c r="E124" t="inlineStr"/>
@@ -9772,29 +9776,29 @@
       </c>
       <c r="Q124" s="5" t="inlineStr"/>
       <c r="R124" s="5" t="inlineStr"/>
-      <c r="S124" t="inlineStr">
-        <is>
-          <t>https://jet8.io/</t>
-        </is>
-      </c>
-      <c r="T124" t="inlineStr"/>
-      <c r="U124" t="inlineStr">
-        <is>
-          <t>jet8-2026.png</t>
-        </is>
-      </c>
+      <c r="S124" t="inlineStr"/>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>https://www.crunchbase.com/organization/roomorama; https://www.crunchbase.com/organization/lofty-ai</t>
+        </is>
+      </c>
+      <c r="U124" t="inlineStr"/>
       <c r="V124" t="inlineStr"/>
       <c r="W124" t="inlineStr"/>
       <c r="X124" t="inlineStr"/>
       <c r="Y124" t="inlineStr"/>
       <c r="Z124" t="inlineStr"/>
       <c r="AA124" t="inlineStr"/>
-      <c r="AB124" t="inlineStr"/>
+      <c r="AB124" t="inlineStr">
+        <is>
+          <t>Site roomorama.com fora do ar (certificado inválido) em 28/09/2026; link tirado do card.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>2080</t>
+          <t>2090</t>
         </is>
       </c>
       <c r="B125" s="5" t="inlineStr">
@@ -9805,7 +9809,7 @@
       <c r="C125" s="5" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
-          <t>LOFTY / ROOMORAMA</t>
+          <t>Lulu App</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -9836,26 +9840,26 @@
       <c r="S125" t="inlineStr"/>
       <c r="T125" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/roomorama; https://www.crunchbase.com/organization/lofty-ai</t>
-        </is>
-      </c>
-      <c r="U125" t="inlineStr"/>
+          <t>https://www.crunchbase.com/organization/lulu-2</t>
+        </is>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>lulu-app.png</t>
+        </is>
+      </c>
       <c r="V125" t="inlineStr"/>
       <c r="W125" t="inlineStr"/>
       <c r="X125" t="inlineStr"/>
       <c r="Y125" t="inlineStr"/>
       <c r="Z125" t="inlineStr"/>
       <c r="AA125" t="inlineStr"/>
-      <c r="AB125" t="inlineStr">
-        <is>
-          <t>Site roomorama.com fora do ar (certificado inválido) em 28/09/2026; link tirado do card.</t>
-        </is>
-      </c>
+      <c r="AB125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>2090</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="B126" s="5" t="inlineStr">
@@ -9866,7 +9870,7 @@
       <c r="C126" s="5" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Lulu App</t>
+          <t>Moneto / ContaPaga</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -9897,12 +9901,12 @@
       <c r="S126" t="inlineStr"/>
       <c r="T126" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/lulu-2</t>
+          <t>https://www.crunchbase.com/organization/contapaga</t>
         </is>
       </c>
       <c r="U126" t="inlineStr">
         <is>
-          <t>lulu-app.png</t>
+          <t>moneto.png</t>
         </is>
       </c>
       <c r="V126" t="inlineStr"/>
@@ -9911,12 +9915,16 @@
       <c r="Y126" t="inlineStr"/>
       <c r="Z126" t="inlineStr"/>
       <c r="AA126" t="inlineStr"/>
-      <c r="AB126" t="inlineStr"/>
+      <c r="AB126" t="inlineStr">
+        <is>
+          <t>ContaPaga mudou de nome para Moneto; cards unificados em 29/09/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
@@ -9927,7 +9935,7 @@
       <c r="C127" s="5" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Moneto</t>
+          <t>OrderIn</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -9958,12 +9966,12 @@
       <c r="S127" t="inlineStr"/>
       <c r="T127" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/contapaga</t>
+          <t>https://www.crunchbase.com/organization/orderin</t>
         </is>
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>moneto.png</t>
+          <t>orderin-2026.png</t>
         </is>
       </c>
       <c r="V127" t="inlineStr"/>
@@ -9977,7 +9985,7 @@
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>2120</t>
         </is>
       </c>
       <c r="B128" s="5" t="inlineStr">
@@ -9988,7 +9996,7 @@
       <c r="C128" s="5" t="inlineStr"/>
       <c r="D128" t="inlineStr">
         <is>
-          <t>OrderIn</t>
+          <t>Scup</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -10007,24 +10015,32 @@
         <f>IF(L128&lt;&gt;"",L128,_xlfn.TEXTJOIN(" · ",TRUE,IF(F128&lt;&gt;"","Fundador",""),IF(G128&lt;&gt;"","Anjo",""),IF(H128&lt;&gt;"","VC",""),IF(I128&lt;&gt;"","Gestão",""),IF(J128&lt;&gt;"","Conselho",""),IF(K128&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N128" t="inlineStr"/>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>Vendida à Sprinkr</t>
+        </is>
+      </c>
       <c r="O128" s="5" t="inlineStr"/>
       <c r="P128" t="inlineStr">
         <is>
-          <t>Encerrada</t>
-        </is>
-      </c>
-      <c r="Q128" s="5" t="inlineStr"/>
+          <t>Saída · 2015</t>
+        </is>
+      </c>
+      <c r="Q128" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="R128" s="5" t="inlineStr"/>
       <c r="S128" t="inlineStr"/>
       <c r="T128" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/orderin</t>
+          <t>https://www.crunchbase.com/organization/scup</t>
         </is>
       </c>
       <c r="U128" t="inlineStr">
         <is>
-          <t>orderin-2026.png</t>
+          <t>scup-2026.png</t>
         </is>
       </c>
       <c r="V128" t="inlineStr"/>
@@ -10038,7 +10054,7 @@
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>2120</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="B129" s="5" t="inlineStr">
@@ -10049,7 +10065,7 @@
       <c r="C129" s="5" t="inlineStr"/>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Scup</t>
+          <t>Shoes4you</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -10068,32 +10084,28 @@
         <f>IF(L129&lt;&gt;"",L129,_xlfn.TEXTJOIN(" · ",TRUE,IF(F129&lt;&gt;"","Fundador",""),IF(G129&lt;&gt;"","Anjo",""),IF(H129&lt;&gt;"","VC",""),IF(I129&lt;&gt;"","Gestão",""),IF(J129&lt;&gt;"","Conselho",""),IF(K129&lt;&gt;"","Buscapé","")))</f>
         <v/>
       </c>
-      <c r="N129" t="inlineStr">
-        <is>
-          <t>Vendida à Sprinkr</t>
-        </is>
-      </c>
+      <c r="N129" t="inlineStr"/>
       <c r="O129" s="5" t="inlineStr"/>
       <c r="P129" t="inlineStr">
         <is>
-          <t>Saída · 2015</t>
-        </is>
-      </c>
-      <c r="Q129" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Encerrada</t>
+        </is>
+      </c>
+      <c r="Q129" s="5" t="inlineStr"/>
       <c r="R129" s="5" t="inlineStr"/>
-      <c r="S129" t="inlineStr"/>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>https://shoes4you.com.br/</t>
+        </is>
+      </c>
       <c r="T129" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/scup</t>
+          <t>https://www.crunchbase.com/organization/shoes4you</t>
         </is>
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>scup-2026.png</t>
+          <t>shoes4you.png</t>
         </is>
       </c>
       <c r="V129" t="inlineStr"/>
@@ -10107,7 +10119,7 @@
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>2140</t>
         </is>
       </c>
       <c r="B130" s="5" t="inlineStr">
@@ -10118,7 +10130,7 @@
       <c r="C130" s="5" t="inlineStr"/>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Shoes4you</t>
+          <t>Siga Seu Time</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -10146,21 +10158,13 @@
       </c>
       <c r="Q130" s="5" t="inlineStr"/>
       <c r="R130" s="5" t="inlineStr"/>
-      <c r="S130" t="inlineStr">
-        <is>
-          <t>https://shoes4you.com.br/</t>
-        </is>
-      </c>
+      <c r="S130" t="inlineStr"/>
       <c r="T130" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/shoes4you</t>
-        </is>
-      </c>
-      <c r="U130" t="inlineStr">
-        <is>
-          <t>shoes4you.png</t>
-        </is>
-      </c>
+          <t>https://www.crunchbase.com/organization/sigaseutime</t>
+        </is>
+      </c>
+      <c r="U130" t="inlineStr"/>
       <c r="V130" t="inlineStr"/>
       <c r="W130" t="inlineStr"/>
       <c r="X130" t="inlineStr"/>
@@ -10172,7 +10176,7 @@
     <row r="131">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>2140</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="B131" s="5" t="inlineStr">
@@ -10183,7 +10187,7 @@
       <c r="C131" s="5" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Siga Seu Time</t>
+          <t>youHotel</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -10214,10 +10218,14 @@
       <c r="S131" t="inlineStr"/>
       <c r="T131" t="inlineStr">
         <is>
-          <t>https://www.crunchbase.com/organization/sigaseutime</t>
-        </is>
-      </c>
-      <c r="U131" t="inlineStr"/>
+          <t>https://www.crunchbase.com/organization/youhotel</t>
+        </is>
+      </c>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>youhotel.png</t>
+        </is>
+      </c>
       <c r="V131" t="inlineStr"/>
       <c r="W131" t="inlineStr"/>
       <c r="X131" t="inlineStr"/>
@@ -10226,69 +10234,8 @@
       <c r="AA131" t="inlineStr"/>
       <c r="AB131" t="inlineStr"/>
     </row>
-    <row r="132">
-      <c r="A132" s="5" t="inlineStr">
-        <is>
-          <t>2150</t>
-        </is>
-      </c>
-      <c r="B132" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="C132" s="5" t="inlineStr"/>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>youHotel</t>
-        </is>
-      </c>
-      <c r="E132" t="inlineStr"/>
-      <c r="F132" s="5" t="inlineStr"/>
-      <c r="G132" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H132" s="5" t="inlineStr"/>
-      <c r="I132" s="5" t="inlineStr"/>
-      <c r="J132" s="5" t="inlineStr"/>
-      <c r="K132" s="5" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
-      <c r="M132" s="6">
-        <f>IF(L132&lt;&gt;"",L132,_xlfn.TEXTJOIN(" · ",TRUE,IF(F132&lt;&gt;"","Fundador",""),IF(G132&lt;&gt;"","Anjo",""),IF(H132&lt;&gt;"","VC",""),IF(I132&lt;&gt;"","Gestão",""),IF(J132&lt;&gt;"","Conselho",""),IF(K132&lt;&gt;"","Buscapé","")))</f>
-        <v/>
-      </c>
-      <c r="N132" t="inlineStr"/>
-      <c r="O132" s="5" t="inlineStr"/>
-      <c r="P132" t="inlineStr">
-        <is>
-          <t>Encerrada</t>
-        </is>
-      </c>
-      <c r="Q132" s="5" t="inlineStr"/>
-      <c r="R132" s="5" t="inlineStr"/>
-      <c r="S132" t="inlineStr"/>
-      <c r="T132" t="inlineStr">
-        <is>
-          <t>https://www.crunchbase.com/organization/youhotel</t>
-        </is>
-      </c>
-      <c r="U132" t="inlineStr">
-        <is>
-          <t>youhotel.png</t>
-        </is>
-      </c>
-      <c r="V132" t="inlineStr"/>
-      <c r="W132" t="inlineStr"/>
-      <c r="X132" t="inlineStr"/>
-      <c r="Y132" t="inlineStr"/>
-      <c r="Z132" t="inlineStr"/>
-      <c r="AA132" t="inlineStr"/>
-      <c r="AB132" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AB132"/>
+  <autoFilter ref="A1:AB131"/>
   <dataValidations count="2">
     <dataValidation sqref="B2:B2000 F2:F2000 G2:G2000 H2:H2000 I2:I2000 J2:J2000 K2:K2000 Q2:Q2000 R2:R2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Use x para marcar ou deixe vazio." type="list">
       <formula1>"x"</formula1>

</xml_diff>